<commit_message>
C1 suburb source runs and C2 ABS demography columns
- SuburbScorecard col Z: CHECKED source notes for the remaining 45
  passing rows (Wikipedia, Victorian Places, ABS 2021 GCP). Scores
  unchanged; flags for C3 recorded in the pointer.
- SuburbScorecard cols AK-AW: ABS 2021 demography for all 63 suburbs
  (median age, % 65+, % born overseas, % not stated, India-born,
  Indian ancestry, Hinduism, Sikhism, languages).
- Previous workbook archived; pointer and open-work list updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013uWqdtxBL1QFjMDN6afhAy
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -27,10 +27,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="hh:mm"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -156,7 +157,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -247,6 +248,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -427,11 +434,32 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Unknown Author</author>
+    <author>Claude</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <t>27 Oct 2026: columns A–H and Z were Google-only formulas splitting column AA. Converted to plain values so they can be edited in Excel. Blank price (G) = not yet researched (was shown as 0).</t>
+      </text>
+    </comment>
+    <comment ref="AP1" authorId="1" shapeId="0">
+      <text>
+        <t>Born overseas / all people (ABS G01 Birthplace_Elsewhere_P / Tot_P). Not the same as 100 minus Australia-born: that also counts people who did not state a birthplace (see next column). This fixes foundation-report item 11.</t>
+      </text>
+    </comment>
+    <comment ref="AQ1" authorId="1" shapeId="0">
+      <text>
+        <t>All people minus Australia-born minus overseas-born, as a share of all people.</t>
+      </text>
+    </comment>
+    <comment ref="AS1" authorId="1" shapeId="0">
+      <text>
+        <t>Indian ancestry responses / all people (ABS G08). People can give two ancestries.</t>
+      </text>
+    </comment>
+    <comment ref="AW1" authorId="1" shapeId="0">
+      <text>
+        <t>From ABS GCP table G13 (about 45 named languages). Languages ABS groups as "other" there (e.g. Telugu, Burmese, Zomi) cannot appear; QuickStats top-responses may differ.</t>
       </text>
     </comment>
   </commentList>
@@ -6107,8 +6135,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AJ90"/>
+  <dimension ref="A1:AW90"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13" customWidth="1" style="15" min="37" max="37"/>
+    <col width="13" customWidth="1" style="15" min="38" max="38"/>
+    <col width="13" customWidth="1" style="15" min="39" max="39"/>
+    <col width="13" customWidth="1" style="15" min="40" max="40"/>
+    <col width="13" customWidth="1" style="15" min="41" max="41"/>
+    <col width="13" customWidth="1" style="15" min="42" max="42"/>
+    <col width="13" customWidth="1" style="15" min="43" max="43"/>
+    <col width="13" customWidth="1" style="15" min="44" max="44"/>
+    <col width="13" customWidth="1" style="15" min="45" max="45"/>
+    <col width="13" customWidth="1" style="15" min="46" max="46"/>
+    <col width="13" customWidth="1" style="15" min="47" max="47"/>
+    <col width="30" customWidth="1" style="15" min="48" max="48"/>
+    <col width="30" customWidth="1" style="15" min="49" max="49"/>
+  </cols>
   <sheetData>
     <row r="1" ht="41.75" customHeight="1" s="15">
       <c r="A1" s="17" t="inlineStr">
@@ -6289,6 +6332,71 @@
       <c r="AJ1" s="23" t="inlineStr">
         <is>
           <t>Budget note</t>
+        </is>
+      </c>
+      <c r="AK1" s="23" t="inlineStr">
+        <is>
+          <t>ABS SAL code (2021)</t>
+        </is>
+      </c>
+      <c r="AL1" s="23" t="inlineStr">
+        <is>
+          <t>Population (ABS 2021)</t>
+        </is>
+      </c>
+      <c r="AM1" s="23" t="inlineStr">
+        <is>
+          <t>Median age</t>
+        </is>
+      </c>
+      <c r="AN1" s="23" t="inlineStr">
+        <is>
+          <t>% aged 65+</t>
+        </is>
+      </c>
+      <c r="AO1" s="23" t="inlineStr">
+        <is>
+          <t>% born overseas (of all people)</t>
+        </is>
+      </c>
+      <c r="AP1" s="23" t="inlineStr">
+        <is>
+          <t>% birthplace not stated</t>
+        </is>
+      </c>
+      <c r="AQ1" s="23" t="inlineStr">
+        <is>
+          <t>% born in India</t>
+        </is>
+      </c>
+      <c r="AR1" s="23" t="inlineStr">
+        <is>
+          <t>% Indian ancestry</t>
+        </is>
+      </c>
+      <c r="AS1" s="23" t="inlineStr">
+        <is>
+          <t>% Hinduism</t>
+        </is>
+      </c>
+      <c r="AT1" s="23" t="inlineStr">
+        <is>
+          <t>% Sikhism</t>
+        </is>
+      </c>
+      <c r="AU1" s="23" t="inlineStr">
+        <is>
+          <t>% other language at home</t>
+        </is>
+      </c>
+      <c r="AV1" s="23" t="inlineStr">
+        <is>
+          <t>Top 3 languages other than English (% of people)</t>
+        </is>
+      </c>
+      <c r="AW1" s="23" t="inlineStr">
+        <is>
+          <t>Demography source and caveats</t>
         </is>
       </c>
     </row>
@@ -6424,6 +6532,51 @@
           <t>House median $1.60M (OnTheHouse) exceeds $1.5M cap, but unit/villa median is $820k. Awaiting documented search for suitable single-level homes/units under $1.5M.</t>
         </is>
       </c>
+      <c r="AK2" s="22" t="inlineStr">
+        <is>
+          <t>SAL20252</t>
+        </is>
+      </c>
+      <c r="AL2" s="32" t="n">
+        <v>14478</v>
+      </c>
+      <c r="AM2" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN2" s="33" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="AO2" s="33" t="n">
+        <v>0.324</v>
+      </c>
+      <c r="AP2" s="33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AQ2" s="33" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="AR2" s="33" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AS2" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AT2" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AU2" s="33" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="AV2" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 10.4%; Cantonese 3.2%; Hindi 1.3%</t>
+        </is>
+      </c>
+      <c r="AW2" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="15">
       <c r="A3" s="18" t="inlineStr">
@@ -6525,7 +6678,7 @@
       </c>
       <c r="Z3" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 35.7% overseas-born, 33.3% non-Eng HH. Belgrave/Lilydale rail; Maroondah Hospital ED nearby (verify drive). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 35.7% overseas-born, 33.3% non-Eng HH. Belgrave/Lilydale rail; Maroondah Hospital ED nearby (verify drive). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 19,144; 20 km E of CBD [Wikipedia Ringwood] (23 km per Victorian Places). Train: major hub; Ringwood station is the junction of the Lilydale and Belgrave lines; Heatherdale station also in the suburb; many bus routes [Wikipedia]; S 9 consistent. Shops: Eastland Shopping Centre (opened 1967, redeveloped) and Ringwood Town Square [Wikipedia; Victorian Places]; Q 10 consistent. Nature: Ringwood Lake 8.5 ha park with a bushland walking circuit; Jubilee Park [Wikipedia; Victorian Places]; N 4 consistent. Village: commercial centre on a highway with bypass routes [Victorian Places]; R 3 consistent. Indian community: India-born 3.2% (618), Indian ancestry 3.7%, Hinduism 2.7%, Sikhism 0.7% [ABS 2021 GCP SAL22174]; P 6 generous next to Berwick 7 at 6.1% (4-5 arguable). City trip: 20 km by train; journey time not stated; V 7 estimate. NOT checked: GPs, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA3" s="16" t="inlineStr">
@@ -6576,6 +6729,51 @@
           <t>Published house price ($1,045,000) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK3" s="22" t="inlineStr">
+        <is>
+          <t>SAL22174</t>
+        </is>
+      </c>
+      <c r="AL3" s="32" t="n">
+        <v>19144</v>
+      </c>
+      <c r="AM3" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="AN3" s="33" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="AO3" s="33" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="AP3" s="33" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="AQ3" s="33" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AR3" s="33" t="n">
+        <v>0.03700000000000001</v>
+      </c>
+      <c r="AS3" s="33" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AT3" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AU3" s="33" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="AV3" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 9.0%; Cantonese 3.2%; Persian 1.5%</t>
+        </is>
+      </c>
+      <c r="AW3" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1" s="15">
       <c r="A4" s="18" t="inlineStr">
@@ -6677,7 +6875,7 @@
       </c>
       <c r="Z4" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 28.1% overseas-born, 28.4% non-Eng HH. Austin Hospital precinct; verify residential pocket &amp; gradients. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 28.1% overseas-born, 28.4% non-Eng HH. Austin Hospital precinct; verify residential pocket &amp; gradients. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 7,360; 11 km NE of CBD, City of Banyule [Wikipedia Heidelberg]. Hospital: Austin Hospital (with Mercy Hospital for Women) is in the suburb [Wikipedia]. Shops: Heidelberg Central (Burgundy St) 'over 230 retail and professional businesses'; Warringal Shopping Centre [Wikipedia]; Q 8 consistent (9 arguable). Train: station at the west end of Burgundy St [Victorian Places]; Hurstbridge line [AC]; S 8 consistent. Nature: eastern flank is the Yarra Flats and Warringal wetlands [Victorian Places]; N 6 consistent. Village: old Waringal village core (St John's 1849, Old England Hotel 1848) but now 'a mature suburb' dominated by the hospital [Victorian Places]; R 4 consistent. Indian community: India-born 3.0%, Indian ancestry 3.5%, Hinduism 2.9% [ABS 2021 GCP SAL21167]; P 5 consistent. City trip: 11 km by train; V 8 consistent. NOT checked: supermarket name, GPs, journey time. Victorian Places gives '2 km', an error; Wikipedia 11 km used. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA4" s="16" t="inlineStr">
@@ -6728,6 +6926,51 @@
           <t>House median $1.452M (35 sales) is under $1.5M cap. Passes GW drive (25m) and ED drive (4m).</t>
         </is>
       </c>
+      <c r="AK4" s="22" t="inlineStr">
+        <is>
+          <t>SAL21167</t>
+        </is>
+      </c>
+      <c r="AL4" s="32" t="n">
+        <v>7360</v>
+      </c>
+      <c r="AM4" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN4" s="33" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="AO4" s="33" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="AP4" s="33" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AQ4" s="33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AR4" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AS4" s="33" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="AT4" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AU4" s="33" t="n">
+        <v>0.237</v>
+      </c>
+      <c r="AV4" s="22" t="inlineStr">
+        <is>
+          <t>Italian 2.7%; Mandarin 2.7%; Greek 1.8%</t>
+        </is>
+      </c>
+      <c r="AW4" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="15">
       <c r="A5" s="18" t="inlineStr">
@@ -6829,7 +7072,7 @@
       </c>
       <c r="Z5" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 18.5% overseas-born, 14.0% non-Eng HH. Hurstbridge line; verify ED &amp; GW drive times. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 18.5% overseas-born, 14.0% non-Eng HH. Hurstbridge line; verify ED &amp; GW drive times. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 18,847; 20 km NE of CBD, Shire of Nillumbik [Wikipedia Eltham]. Nature: green wedge leaves 'extensive areas undeveloped within and to three sides of the suburb'; Barak Bushlands, Laughing Waters bushland (riparian and open forest), Diamond Creek Trail, Maroondah Aqueduct Trail [Wikipedia]; N 8 consistent. Village: central shopping strip on Main Road, Sunday farmers' market, Montsalvat artists' colony, mud-brick heritage (Alistair Knox) [Wikipedia]; R 7 consistent. Train: Eltham station, Hurstbridge line; major bus interchange (SmartBus 902 etc.) [Wikipedia]; S 8 consistent. Shops: supermarket not named; Q 8 estimate. Indian community: India-born 0.7%, Hinduism 0.6% [ABS 2021 GCP SAL20865]; P 3 generous (2 arguable). City trip: 20 km by train; V 7 estimate. NOT checked: GPs, supermarket, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA5" s="16" t="inlineStr">
@@ -6880,6 +7123,51 @@
           <t>House median $1.273M (195 sales) is under $1.5M cap. Passes GW drive (26m) and ED drive (16m).</t>
         </is>
       </c>
+      <c r="AK5" s="22" t="inlineStr">
+        <is>
+          <t>SAL20865</t>
+        </is>
+      </c>
+      <c r="AL5" s="32" t="n">
+        <v>18847</v>
+      </c>
+      <c r="AM5" s="22" t="n">
+        <v>43</v>
+      </c>
+      <c r="AN5" s="33" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="AO5" s="33" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="AP5" s="33" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AQ5" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AR5" s="33" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AS5" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AT5" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU5" s="33" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="AV5" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 1.6%; Italian 1.0%; Greek 0.9%</t>
+        </is>
+      </c>
+      <c r="AW5" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="15">
       <c r="A6" s="18" t="inlineStr">
@@ -6981,7 +7269,7 @@
       </c>
       <c r="Z6" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 19.2% overseas-born, 12.2% non-Eng HH. Belgrave line; 10-min walk/bus 732 to Angliss Hospital (verify 24-hr ED status &amp; drive). 27 Oct 2026: OnTheHouse gives the same house AVM ($872,133) for Upper Ferntree Gully and Ferntree Gully — likely postcode-level, weak. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price = postcode-level AVM shared with FTG.</t>
+          <t>ABS 2021: 19.2% overseas-born, 12.2% non-Eng HH. Belgrave line; 10-min walk/bus 732 to Angliss Hospital (verify 24-hr ED status &amp; drive). 27 Oct 2026: OnTheHouse gives the same house AVM ($872,133) for Upper Ferntree Gully and Ferntree Gully — likely postcode-level, weak. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price = postcode-level AVM shared with FTG. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 3,417; 32 km E of CBD [Wikipedia Upper Ferntree Gully]. Nature: Ferntree Gully Park (Dandenong Ranges National Park) incl. the '1,000 steps' Kokoda walk; Ferny Creek reserves [Wikipedia]; N 8 consistent. Hospital: Angliss Hospital is in the suburb, with medical consulting rooms nearby [Wikipedia]. Shops: 'limited retail outlets (mainly food, hairdressing, banking, chemist, post office)' along Burwood Hwy; Ferntree Plaza the largest centre [Wikipedia]; Q 6 consistent. Village: highway strip with used-car yards [Wikipedia]; R 5 consistent. Train: station on the Belgrave line [AC]; S 7 not re-checked. Indian community: India-born 1.0%, Hinduism 0.3% [ABS 2021 GCP SAL22614]; P 5 not supported (2 arguable). City trip: 32 km by train; V 6 estimate. NOT checked: GPs by name, supermarket, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA6" s="16" t="inlineStr">
@@ -7030,6 +7318,51 @@
       <c r="AJ6" s="22" t="inlineStr">
         <is>
           <t>Published house price ($872,133) is under $1.5M cap.</t>
+        </is>
+      </c>
+      <c r="AK6" s="22" t="inlineStr">
+        <is>
+          <t>SAL22614</t>
+        </is>
+      </c>
+      <c r="AL6" s="32" t="n">
+        <v>3417</v>
+      </c>
+      <c r="AM6" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN6" s="33" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="AO6" s="33" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="AP6" s="33" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="AQ6" s="33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AR6" s="33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AS6" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" s="33" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="AV6" s="22" t="inlineStr">
+        <is>
+          <t>German 1.2%; Greek 0.8%; Mandarin 0.7%</t>
+        </is>
+      </c>
+      <c r="AW6" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -7164,6 +7497,51 @@
           <t>House median $1.76M (454 sales) exceeds $1.5M cap; unit median $930k. Awaiting documented search for suitable single-level homes/units under $1.5M.</t>
         </is>
       </c>
+      <c r="AK7" s="22" t="inlineStr">
+        <is>
+          <t>SAL21013</t>
+        </is>
+      </c>
+      <c r="AL7" s="32" t="n">
+        <v>42642</v>
+      </c>
+      <c r="AM7" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AN7" s="33" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="AO7" s="33" t="n">
+        <v>0.5870000000000001</v>
+      </c>
+      <c r="AP7" s="33" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AQ7" s="33" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AR7" s="33" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="AS7" s="33" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="AT7" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AU7" s="33" t="n">
+        <v>0.608</v>
+      </c>
+      <c r="AV7" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 23.3%; Cantonese 8.0%; Sinhalese 4.0%</t>
+        </is>
+      </c>
+      <c r="AW7" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="15">
       <c r="A8" s="18" t="inlineStr">
@@ -7266,7 +7644,7 @@
       </c>
       <c r="Z8" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 17.7% aged 65+, 17.0% non-Eng HH. Direct city bus 906; no local rail; check fire overlay &amp; ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 17.7% aged 65+, 17.0% non-Eng HH. Direct city bus 906; no local rail; check fire overlay &amp; ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 5,541; 24 km NE of CBD on the Yarra River; town 'nestled into a gorge on the river' [Wikipedia Warrandyte]. Nature: Warrandyte State Park (Pound Bend, Fourth Hill, Black Flat, Mount Lofty), river swimming, canoeing, bushwalking, many reserves incl. Currawong Bush Park [Wikipedia]; N 9 consistent. Village: surviving colonial-era buildings, shops on Yarra St near the bridge, Mechanics' Institute arts community [Wikipedia]; R 8 consistent. Shops: Goldfields Shopping Centre plus Yarra St shops [Wikipedia]; supermarket not named; Q 6 estimate. Train: no station in either source; S 3 consistent (bus 906 not checked). Two community-run micro-retirement villages [Wikipedia]. Indian community: India-born 0.7%, Hinduism 0.7% [ABS 2021 GCP SAL22702]; P 3 generous (2 arguable). City trip: 24 km but no rail; V 4 estimate. NOT checked: GPs, bus, journey time, bushfire overlay. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA8" s="16" t="inlineStr">
@@ -7317,6 +7695,51 @@
           <t>AVM house value ($1,348,901) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK8" s="22" t="inlineStr">
+        <is>
+          <t>SAL22702</t>
+        </is>
+      </c>
+      <c r="AL8" s="32" t="n">
+        <v>5541</v>
+      </c>
+      <c r="AM8" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AN8" s="33" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="AO8" s="33" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="AP8" s="33" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AQ8" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AR8" s="33" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AS8" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AT8" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AU8" s="33" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AV8" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 2.9%; Greek 1.7%; Italian 1.6%</t>
+        </is>
+      </c>
+      <c r="AW8" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="15">
       <c r="A9" s="18" t="inlineStr">
@@ -7418,7 +7841,7 @@
       </c>
       <c r="Z9" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 13.1% aged 65+, 12.2% non-Eng HH. Hurstbridge line station &amp; trail; verify ED &amp; GW drive. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 13.1% aged 65+, 12.2% non-Eng HH. Hurstbridge line station &amp; trail; verify ED &amp; GW drive. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 12,503; 23 km NE of CBD, Shire of Nillumbik [Wikipedia Diamond Creek]. Train: shopping centre and station sit on the banks of the Diamond Creek; Hurstbridge line [Wikipedia]; S 7 consistent. Shops: a shopping centre near the station and a second centre across the line [Victorian Places]; Q 7 consistent (supermarket not named). Nature: creek corridor and the large Diamond Creek reserve [Victorian Places]; N 7 consistent. Village: 'a pleasant backwater' that grew suburban from the 1970s; heritage St John's (c1867) [Victorian Places; Wikipedia]; R 6 consistent. Community centre was a 2009 bushfire evacuation point [Wikipedia]. Indian community: India-born 0.7%, Hinduism 0.7% [ABS 2021 GCP SAL20752]; P 2 consistent. City trip: 23 km by train; V 6 estimate. NOT checked: GPs, supermarket, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA9" s="16" t="inlineStr">
@@ -7469,6 +7892,51 @@
           <t>Published house price ($885,000) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK9" s="22" t="inlineStr">
+        <is>
+          <t>SAL20752</t>
+        </is>
+      </c>
+      <c r="AL9" s="32" t="n">
+        <v>12503</v>
+      </c>
+      <c r="AM9" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN9" s="33" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="AO9" s="33" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="AP9" s="33" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AQ9" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AR9" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AS9" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AT9" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AU9" s="33" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="AV9" s="22" t="inlineStr">
+        <is>
+          <t>Italian 1.2%; Greek 0.7%; Mandarin 0.7%</t>
+        </is>
+      </c>
+      <c r="AW9" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="15">
       <c r="A10" s="18" t="inlineStr">
@@ -7570,7 +8038,7 @@
       </c>
       <c r="Z10" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 28.8% overseas-born, 22.4% non-Eng HH. Reconcile price sources &amp; verify ED drive. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Mentone Beach + lifesaving club; Woolworths at Thrift Park; Southland next door (Wikipedia Mentone). GPs: Mentone Medical Clinic, St Kerellos Medical Centre (healthdirect). N, P, R, V remain estimates.</t>
+          <t>ABS 2021: 28.8% overseas-born, 22.4% non-Eng HH. Reconcile price sources &amp; verify ED drive. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Mentone Beach + lifesaving club; Woolworths at Thrift Park; Southland next door (Wikipedia Mentone). GPs: Mentone Medical Clinic, St Kerellos Medical Centre (healthdirect). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Mentone Beach along Beaumaris Bay [Wikipedia Mentone]; no bushland or large reserve named; N 4 consistent. Village: 'lively shopping area' on Como Pde West, Balcombe Rd, Mentone Pde with cafés, bakeries, bookshops; Mediterranean-named 1880s township streets [Wikipedia; Victorian Places]; R 6 consistent. Indian community: India-born 1.9%, Indian ancestry 2.5%, Hinduism 1.7% [ABS 2021 GCP SAL21648]; P 5 generous (3 arguable). City trip: 21-22 km SE on the Frankston line [Wikipedia; Victorian Places]; journey time not stated; V 8 plausible. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA10" s="16" t="inlineStr">
@@ -7621,6 +8089,51 @@
           <t>House median $1.497M (CoreLogic) / $1.30M (Woodards) is under $1.5M cap. Passes GW drive (25m) and ED drive (16m).</t>
         </is>
       </c>
+      <c r="AK10" s="22" t="inlineStr">
+        <is>
+          <t>SAL21648</t>
+        </is>
+      </c>
+      <c r="AL10" s="32" t="n">
+        <v>13197</v>
+      </c>
+      <c r="AM10" s="22" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN10" s="33" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="AO10" s="33" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AP10" s="33" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AQ10" s="33" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AR10" s="33" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AS10" s="33" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="AT10" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AU10" s="33" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="AV10" s="22" t="inlineStr">
+        <is>
+          <t>Greek 3.5%; Mandarin 3.0%; Russian 1.5%</t>
+        </is>
+      </c>
+      <c r="AW10" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="15">
       <c r="A11" s="18" t="inlineStr">
@@ -7722,7 +8235,7 @@
       </c>
       <c r="Z11" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 22.5% overseas-born, 15.2% non-Eng HH. Peninsula Univ Hospital ED; ~66m train to CBD. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Rail terminus + bus hub to Mornington, Rosebud etc. (Wikipedia). GP: myhealth Bayside (healthdirect). Beach U and supermarket not individually checked. N, P, R, V remain estimates.</t>
+          <t>ABS 2021: 22.5% overseas-born, 15.2% non-Eng HH. Peninsula Univ Hospital ED; ~66m train to CBD. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Rail terminus + bus hub to Mornington, Rosebud etc. (Wikipedia). GP: myhealth Bayside (healthdirect). Beach U and supermarket not individually checked. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: 'generally a leafy suburb'; natural reserves Bunarong Park, Frankston Foreshore Reserve, Lower Sweetwater Creek Reserve, Paratea Reserve; over 20 indigenous orchid species; McClelland Sculpture Park in 16 ha of park and reserve [Wikipedia Frankston]; N 5 consistent (6 arguable). Village: regional centre with Bayside (250+ stores) and Karingal Hub; several vacant highway buildings noted [Wikipedia; Victorian Places]; R 3 consistent. Health hub: four hospitals in the suburb [Wikipedia]. Indian community: India-born 1.1%, Hinduism 0.8%; Malayalam 0.5% at home [ABS 2021 GCP SAL20947; Wikipedia]; P 4 generous (2 arguable). City trip: 39-40 km SE, line terminus [Wikipedia; Victorian Places]; V 6 plausible. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA11" s="16" t="inlineStr">
@@ -7773,6 +8286,51 @@
           <t>Published house price ($834,296) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK11" s="22" t="inlineStr">
+        <is>
+          <t>SAL20947</t>
+        </is>
+      </c>
+      <c r="AL11" s="32" t="n">
+        <v>37331</v>
+      </c>
+      <c r="AM11" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN11" s="33" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="AO11" s="33" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="AP11" s="33" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="AQ11" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AR11" s="33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AS11" s="33" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AT11" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU11" s="33" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="AV11" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 1.4%; Greek 1.0%; Russian 0.6%</t>
+        </is>
+      </c>
+      <c r="AW11" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="15">
       <c r="A12" s="18" t="inlineStr">
@@ -7874,7 +8432,7 @@
       </c>
       <c r="Z12" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 28.3% overseas-born, 23.8% non-Eng HH. Cross-city drive to Glen Waverley needs testing. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Altona Bay beach, pier, coastal park (Victorian Places). GP: Pier Street Medical Centre (healthdirect). Coles Altona (grocerize). N, P, R, V remain estimates.</t>
+          <t>ABS 2021: 28.3% overseas-born, 23.8% non-Eng HH. Cross-city drive to Glen Waverley needs testing. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Altona Bay beach, pier, coastal park (Victorian Places). GP: Pier Street Medical Centre (healthdirect). Coles Altona (grocerize). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Altona Beach, one of only two swimming beaches in the western suburbs; conservation areas and wetlands along the bay shore; long bayside promenade [Wikipedia Altona]; north-western half is mixed industry [Wikipedia]; N 4 consistent. Village: Pier St and Esplanade precinct; annual beach festival; civic theatre [Wikipedia]; R 6 consistent. Indian community: India-born 1.4%, Indian ancestry 1.9%, Hinduism 1.1% [ABS 2021 GCP SAL20035]; P 6 not supported (3 arguable). City trip: 13 km SW by train (Altona loop) [Wikipedia]; V 8 consistent. Scores unchanged. Victorian Places page not found.</t>
         </is>
       </c>
       <c r="AA12" s="16" t="inlineStr">
@@ -7923,6 +8481,51 @@
       <c r="AJ12" s="22" t="inlineStr">
         <is>
           <t>Published house price ($1,155,073) is under $1.5M cap.</t>
+        </is>
+      </c>
+      <c r="AK12" s="22" t="inlineStr">
+        <is>
+          <t>SAL20035</t>
+        </is>
+      </c>
+      <c r="AL12" s="32" t="n">
+        <v>11490</v>
+      </c>
+      <c r="AM12" s="22" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN12" s="33" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="AO12" s="33" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="AP12" s="33" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="AQ12" s="33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AR12" s="33" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AS12" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AT12" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AU12" s="33" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="AV12" s="22" t="inlineStr">
+        <is>
+          <t>Italian 1.6%; Greek 1.4%; Mandarin 1.4%</t>
+        </is>
+      </c>
+      <c r="AW12" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -8057,6 +8660,51 @@
           <t>Figure is an automated valuation model ($1.64M), not a verified sale median or specific property. Awaiting documented listing search under $1.5M.</t>
         </is>
       </c>
+      <c r="AK13" s="22" t="inlineStr">
+        <is>
+          <t>SAL22792</t>
+        </is>
+      </c>
+      <c r="AL13" s="32" t="n">
+        <v>14407</v>
+      </c>
+      <c r="AM13" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AN13" s="33" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="AO13" s="33" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="AP13" s="33" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AQ13" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AR13" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AS13" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AT13" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU13" s="33" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="AV13" s="22" t="inlineStr">
+        <is>
+          <t>Greek 2.4%; Italian 1.6%; Vietnamese 1.0%</t>
+        </is>
+      </c>
+      <c r="AW13" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="15">
       <c r="A14" s="18" t="inlineStr">
@@ -8159,7 +8807,7 @@
       </c>
       <c r="Z14" s="18" t="inlineStr">
         <is>
-          <t>2021 pop 7,589. CAUTION: Eastern Health directs urgent ED patients to Maroondah Hospital ED (not local). 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>2021 pop 7,589. CAUTION: Eastern Health directs urgent ED patients to Maroondah Hospital ED (not local). 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 7,589; 64 km NE of CBD on the Watts River [Wikipedia Healesville]. Nature: Healesville Sanctuary, Badger Weir picnic area, Maroondah Dam nearby; southern end of the Bicentennial Heritage Trail [Wikipedia]; N 9 consistent. Village: tourist town since the 1880s; Yarra Valley wine and food centre, organic market, cafés, festivals [Wikipedia]; R 8 consistent. Train: only the Yarra Valley tourist railway (Sundays, some holidays) [Wikipedia]; no metro or V/Line station; S 2 consistent. Indian community: India-born 0.2%, Hinduism 0.2% [ABS 2021 GCP SAL21158]; P 1 consistent. Older: median age 46, 23.7% aged 65+ [ABS]. City trip: 64 km, no rail; V 2 consistent. NOT checked: GPs, supermarket, bus. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA14" s="16" t="inlineStr">
@@ -8210,6 +8858,51 @@
           <t>AVM house value ($837,893) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK14" s="22" t="inlineStr">
+        <is>
+          <t>SAL21158</t>
+        </is>
+      </c>
+      <c r="AL14" s="32" t="n">
+        <v>7589</v>
+      </c>
+      <c r="AM14" s="22" t="n">
+        <v>46</v>
+      </c>
+      <c r="AN14" s="33" t="n">
+        <v>0.237</v>
+      </c>
+      <c r="AO14" s="33" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AP14" s="33" t="n">
+        <v>0.05599999999999999</v>
+      </c>
+      <c r="AQ14" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR14" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AS14" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU14" s="33" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="AV14" s="22" t="inlineStr">
+        <is>
+          <t>German 0.7%; Italian 0.6%; Mandarin 0.3%</t>
+        </is>
+      </c>
+      <c r="AW14" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="15">
       <c r="A15" s="18" t="inlineStr">
@@ -8311,7 +9004,7 @@
       </c>
       <c r="Z15" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 25.0% aged 65+, 6.9% non-Eng HH. CAUTION: Local facility is 24-hr Urgent Care Centre, NOT a major public ED. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 25.0% aged 65+, 6.9% non-Eng HH. CAUTION: Local facility is 24-hr Urgent Care Centre, NOT a major public ED. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 7,513; Macedon Ranges, ~75 km NW of Melbourne [Wikipedia Kyneton; Victorian Places]. Train: heritage-listed station south of town, ~86 km from Melbourne on the Bendigo line; 'a terminus for two weekday peak-hour trains' [Wikipedia; Victorian Places]; S 5 consistent (frequency not checked). Village: three main streets; Piper St 'has the oldest streetscape', galleries, bookstores, cafés; historic museum [Wikipedia; Victorian Places]; R 9 consistent. Nature: botanic gardens, Campaspe River walks, Black Hill and Bald Hill reserves nearby [Wikipedia]; N 7 consistent. Indian community: India-born 0.5%, Hinduism 0.3% [ABS 2021 GCP SAL21414]; P 1 consistent. Older: median age 47, 25.0% aged 65+ [ABS]. City trip: 86 km by V/Line; V 5 estimate. NOT checked: GPs, supermarket, train journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA15" s="16" t="inlineStr">
@@ -8362,6 +9055,51 @@
           <t>Published house price ($810,000) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK15" s="22" t="inlineStr">
+        <is>
+          <t>SAL21414</t>
+        </is>
+      </c>
+      <c r="AL15" s="32" t="n">
+        <v>7513</v>
+      </c>
+      <c r="AM15" s="22" t="n">
+        <v>47</v>
+      </c>
+      <c r="AN15" s="33" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AO15" s="33" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="AP15" s="33" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AQ15" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AR15" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AS15" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT15" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU15" s="33" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AV15" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 1.3%; Italian 0.4%; French 0.3%</t>
+        </is>
+      </c>
+      <c r="AW15" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="15">
       <c r="A16" s="18" t="inlineStr">
@@ -8514,6 +9252,51 @@
           <t>Published house price ($890,000) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK16" s="22" t="inlineStr">
+        <is>
+          <t>SAL22833</t>
+        </is>
+      </c>
+      <c r="AL16" s="32" t="n">
+        <v>6732</v>
+      </c>
+      <c r="AM16" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AN16" s="33" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AO16" s="33" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="AP16" s="33" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="AQ16" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR16" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AS16" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AT16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU16" s="33" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AV16" s="22" t="inlineStr">
+        <is>
+          <t>German 0.7%; Italian 0.4%; French 0.3%</t>
+        </is>
+      </c>
+      <c r="AW16" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="15">
       <c r="A17" s="18" t="inlineStr">
@@ -8616,7 +9399,7 @@
       </c>
       <c r="Z17" s="18" t="inlineStr">
         <is>
-          <t>Distinguish Macedon from Mount Macedon; check bushfire overlay, gradients &amp; major ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count.</t>
+          <t>Distinguish Macedon from Mount Macedon; check bushfire overlay, gradients &amp; major ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 2,073; foot of Mount Macedon, 58 km NW of Melbourne, on the Melbourne-Bendigo railway [Wikipedia Macedon; Victorian Places]. Nature: bushland foothills of the Mount Macedon range; vineyards nearby [Wikipedia]; N 10 plausible (9 arguable: town is at the foot, not on the mount). Village: rebuilt shops, churches and hall after the 1983 Ash Wednesday fire (499 houses, 8 lives lost in Macedon and Mount Macedon) [Victorian Places]; cafés and B&amp;Bs, new planning controls 'to protect the character' [Wikipedia]; R 8 consistent. Bushfire risk is real and documented. Shops: small; supermarket not named; Q 3 consistent. Train: station on the Bendigo line [Victorian Places]; S 5 consistent (frequency not checked). Indian community: India-born 0.2%, Hinduism 0.2% [ABS 2021 GCP SAL21562]; P 1 consistent. City trip: 58 km by V/Line; V 5 estimate. NOT checked: GPs, nearest ED, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA17" s="16" t="inlineStr">
@@ -8667,6 +9450,51 @@
           <t>AVM house value ($1,147,643) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK17" s="22" t="inlineStr">
+        <is>
+          <t>SAL21562</t>
+        </is>
+      </c>
+      <c r="AL17" s="32" t="n">
+        <v>2073</v>
+      </c>
+      <c r="AM17" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="AN17" s="33" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="AO17" s="33" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="AP17" s="33" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AQ17" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR17" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AS17" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT17" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU17" s="33" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="AV17" s="22" t="inlineStr">
+        <is>
+          <t>French 0.5%; Polish 0.4%; Italian 0.3%</t>
+        </is>
+      </c>
+      <c r="AW17" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="15">
       <c r="A18" s="18" t="inlineStr">
@@ -8768,7 +9596,7 @@
       </c>
       <c r="Z18" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 16.4% aged 65+, 7.4% non-Eng HH. Bus 54 to Marshall Station; relies on Univ Hospital Geelong for major public ED. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. GW drive 88 min, 2 min under cap. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Buses to Geelong/Marshall: S raised 3-&gt;4 (Bus News). GPs: Surfcoast Medical Centre, Orbit Medical, Banksia (healthdirect). Beach and supermarket not individually checked. N, P, R, V remain estimates.</t>
+          <t>ABS 2021: 16.4% aged 65+, 7.4% non-Eng HH. Bus 54 to Marshall Station; relies on Univ Hospital Geelong for major public ED. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. GW drive 88 min, 2 min under cap. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Buses to Geelong/Marshall: S raised 3-&gt;4 (Bus News). GPs: Surfcoast Medical Centre, Orbit Medical, Banksia (healthdirect). Beach and supermarket not individually checked. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: surf beaches (Jan Juc, Bells Beach on the SW outskirts), Point Danger, Zeally Bay, Spring Creek on the western boundary [Wikipedia Torquay]; N 8 rests on coast, not bush (7 arguable). Village: population doubled 1991-2011 and 'some of its former holiday charm has been lost to redevelopment' [Victorian Places]; population triples in Jan-Feb; Surf Coast Plaza [Wikipedia]; R 6 generous (5 arguable). Indian community: India-born 0.2%, Hinduism 0.1% [ABS 2021 GCP SAL22551]; P 2 generous (1 arguable). City trip: 80 km W of Melbourne, 21 km S of Geelong [Victorian Places], no rail; V 3 plausible; journey time not checked. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA18" s="16" t="inlineStr">
@@ -8817,6 +9645,51 @@
       <c r="AJ18" s="22" t="inlineStr">
         <is>
           <t>House median $1.180M is under $1.5M cap. Passes GW drive (88m &lt;= 90m cap) and ED drive (23m).</t>
+        </is>
+      </c>
+      <c r="AK18" s="22" t="inlineStr">
+        <is>
+          <t>SAL22551</t>
+        </is>
+      </c>
+      <c r="AL18" s="32" t="n">
+        <v>18534</v>
+      </c>
+      <c r="AM18" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN18" s="33" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="AO18" s="33" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="AP18" s="33" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AQ18" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR18" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AS18" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AT18" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU18" s="33" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="AV18" s="22" t="inlineStr">
+        <is>
+          <t>German 0.5%; Italian 0.5%; French 0.4%</t>
+        </is>
+      </c>
+      <c r="AW18" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -8951,6 +9824,51 @@
           <t>Published house price ($980,000) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK19" s="22" t="inlineStr">
+        <is>
+          <t>SAL22005</t>
+        </is>
+      </c>
+      <c r="AL19" s="32" t="n">
+        <v>17714</v>
+      </c>
+      <c r="AM19" s="22" t="n">
+        <v>43</v>
+      </c>
+      <c r="AN19" s="33" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="AO19" s="33" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="AP19" s="33" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="AQ19" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR19" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AS19" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AT19" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU19" s="33" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="AV19" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.4%; German 0.3%; Mandarin 0.3%</t>
+        </is>
+      </c>
+      <c r="AW19" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="15">
       <c r="A20" s="18" t="inlineStr">
@@ -9053,7 +9971,7 @@
       </c>
       <c r="Z20" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 17.6% aged 65+, 10.9% non-Eng HH. Balyang Sanctuary on Barwon River; major public ED at Univ Hospital Geelong. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 17.6% aged 65+, 10.9% non-Eng HH. Balyang Sanctuary on Barwon River; major public ED at Univ Hospital Geelong. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 10,445; inner western Geelong, 'one of the highest points of urban Geelong', many of Geelong's oldest houses [Wikipedia Newtown, Victoria]. Nature: Queens Park beside the Barwon River, Balyang Sanctuary, Chilwell Gardens, Windmill Reserve [Wikipedia]; N 5 consistent. Village: established residential suburb incl. Chilwell; R 6 plausible. Train: no station named in the suburb [Wikipedia]; S 4 consistent. Indian community: India-born 1.3%, Indian ancestry 1.6%, Hinduism 1.1% [ABS 2021 GCP SAL21938]; P 4 generous (3 arguable). NOT checked: shops, GPs, beach distance (U 3), city trip (V 5), Victorian Places page not found. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA20" s="16" t="inlineStr">
@@ -9104,6 +10022,51 @@
           <t>AVM house value ($1,182,945) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK20" s="22" t="inlineStr">
+        <is>
+          <t>SAL21938</t>
+        </is>
+      </c>
+      <c r="AL20" s="32" t="n">
+        <v>10445</v>
+      </c>
+      <c r="AM20" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AN20" s="33" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="AO20" s="33" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="AP20" s="33" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AQ20" s="33" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AR20" s="33" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="AS20" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AT20" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AU20" s="33" t="n">
+        <v>0.08800000000000001</v>
+      </c>
+      <c r="AV20" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 1.3%; Italian 0.6%; Croatian 0.5%</t>
+        </is>
+      </c>
+      <c r="AW20" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Newtown (Greater Geelong), SAL21938.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="15">
       <c r="A21" s="18" t="inlineStr">
@@ -9257,6 +10220,51 @@
           <t>AVM house value ($957,797) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK21" s="22" t="inlineStr">
+        <is>
+          <t>SAL21187</t>
+        </is>
+      </c>
+      <c r="AL21" s="32" t="n">
+        <v>20736</v>
+      </c>
+      <c r="AM21" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN21" s="33" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="AO21" s="33" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="AP21" s="33" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AQ21" s="33" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AR21" s="33" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AS21" s="33" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AT21" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AU21" s="33" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AV21" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 1.9%; Italian 0.8%; Arabic 0.7%</t>
+        </is>
+      </c>
+      <c r="AW21" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="15">
       <c r="A22" s="18" t="inlineStr">
@@ -9359,7 +10367,7 @@
       </c>
       <c r="Z22" s="18" t="inlineStr">
         <is>
-          <t>Belgrave metro rail terminus; check steep gradients, bushfire/storm closures &amp; Angliss/Maroondah ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Terminus (weekend off-peak shuttle) so S 7. Puffing Billy 100 m away. GP: Belgrave Medical Clinic (healthdirect). Supermarket not confirmed; Q partly estimate. N, P, R, V remain estimates.</t>
+          <t>Belgrave metro rail terminus; check steep gradients, bushfire/storm closures &amp; Angliss/Maroondah ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Terminus (weekend off-peak shuttle) so S 7. Puffing Billy 100 m away. GP: Belgrave Medical Clinic (healthdirect). Supermarket not confirmed; Q partly estimate. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Belgrave Lake Park, a biolink between Dandenong Ranges National Park, Birdsland and Lysterfield Lake Park, with platypus in Monbulk Creek and mountain grey gum slopes; Puffing Billy runs through 24 km of cool temperate rainforest and farmland [Wikipedia Belgrave]; N 9 consistent. Village: Main Street commercial district with galleries and bookshops; shops on Bayview Rd [Wikipedia]; R 8 consistent. Indian community: India-born 0.4%, Hinduism 0.2% [ABS 2021 GCP SAL20188]; P 3 generous (1 arguable). City trip: 36 km E, line terminus [Wikipedia]; V 5 estimate. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA22" s="16" t="inlineStr">
@@ -9410,6 +10418,51 @@
           <t>AVM house value ($856,437) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK22" s="22" t="inlineStr">
+        <is>
+          <t>SAL20188</t>
+        </is>
+      </c>
+      <c r="AL22" s="32" t="n">
+        <v>3894</v>
+      </c>
+      <c r="AM22" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="AN22" s="33" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AO22" s="33" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="AP22" s="33" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AQ22" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AR22" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AS22" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU22" s="33" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="AV22" s="22" t="inlineStr">
+        <is>
+          <t>German 0.8%; Mandarin 0.6%; French 0.5%</t>
+        </is>
+      </c>
+      <c r="AW22" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="15">
       <c r="A23" s="18" t="inlineStr">
@@ -9511,7 +10564,7 @@
       </c>
       <c r="Z23" s="18" t="inlineStr">
         <is>
-          <t>Belgrave rail line township; closer to foothills edge than Belgrave. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station beside Main St; medical centre on Main St; no supermarket mentioned: Q lowered 6-&gt;5. Adjoins Dandenong Ranges NP; Ferny, Monbulk creeks (Wikipedia Upwey). N, P, R, V remain estimates.</t>
+          <t>Belgrave rail line township; closer to foothills edge than Belgrave. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station beside Main St; medical centre on Main St; no supermarket mentioned: Q lowered 6-&gt;5. Adjoins Dandenong Ranges NP; Ferny, Monbulk creeks (Wikipedia Upwey). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Glenfern Valley Bushlands, 40 ha of remnant and rehabilitated forest down to Ferny Creek; ridge-top Glenfern Rd with views [Wikipedia Upwey]; N 9 consistent. Village: Main Street 'instilling a traditional community village nature', cafés with kerbside dining, medical and dental centre [Wikipedia]; R 7 consistent (8 arguable); medical centre on Main St supports Q. Indian community: India-born 0.6%, Hinduism 0.3%; 80.7% Australia-born [ABS 2021 GCP SAL22620; Wikipedia]; P 3 generous (1 arguable). City trip: 33 km E on the Belgrave line [Wikipedia]; V 5 estimate. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA23" s="16" t="inlineStr">
@@ -9562,6 +10615,51 @@
           <t>Published house price ($929,500) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK23" s="22" t="inlineStr">
+        <is>
+          <t>SAL22620</t>
+        </is>
+      </c>
+      <c r="AL23" s="32" t="n">
+        <v>6818</v>
+      </c>
+      <c r="AM23" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN23" s="33" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="AO23" s="33" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="AP23" s="33" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AQ23" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AR23" s="33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AS23" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU23" s="33" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="AV23" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 0.5%; Italian 0.4%; Russian 0.4%</t>
+        </is>
+      </c>
+      <c r="AW23" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="15">
       <c r="A24" s="18" t="inlineStr">
@@ -9664,7 +10762,7 @@
       </c>
       <c r="Z24" s="18" t="inlineStr">
         <is>
-          <t>Belgrave rail line; council groups Belgrave-Tecoma-Upwey as established townships. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count.</t>
+          <t>Belgrave rail line; council groups Belgrave-Tecoma-Upwey as established townships. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 2,064; 35 km E of CBD, 1 km W of Belgrave, adjoining Sherbrooke Forest to the north [Wikipedia Tecoma]. Nature: 'residences are built in hilly country, well planted with trees'; bushfire exposure from the National Park to the north [Victorian Places]; N 9 consistent. Village: 'a small strip shopping centre, somewhat held in check by its proximity to Belgrave'; residents campaigned against a fast-food chain as out of character [Victorian Places]; R 6 consistent. Shops: Q 4 consistent (Belgrave next door). Train: Tecoma station on the Belgrave line [Victorian Places]; S 7 consistent. Indian community: India-born 0.3%, Hinduism 0.3%, Sikhism 0.4% [ABS 2021 GCP SAL22476]; P 3 generous (1-2 arguable). City trip: 35 km by train; V 5 estimate. NOT checked: GPs, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA24" s="16" t="inlineStr">
@@ -9715,6 +10813,51 @@
           <t>AVM house value ($894,304) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK24" s="22" t="inlineStr">
+        <is>
+          <t>SAL22476</t>
+        </is>
+      </c>
+      <c r="AL24" s="32" t="n">
+        <v>2064</v>
+      </c>
+      <c r="AM24" s="22" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN24" s="33" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="AO24" s="33" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AP24" s="33" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="AQ24" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AR24" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AS24" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT24" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AU24" s="33" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AV24" s="22" t="inlineStr">
+        <is>
+          <t>German 0.7%; Italian 0.5%; Hindi 0.4%</t>
+        </is>
+      </c>
+      <c r="AW24" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="15">
       <c r="A25" s="18" t="inlineStr">
@@ -9817,7 +10960,7 @@
       </c>
       <c r="Z25" s="18" t="inlineStr">
         <is>
-          <t>Adjoins Dandenong Ranges National Park; verify bus/station link &amp; Angliss Hospital ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Adjoins Dandenong Ranges National Park; verify bus/station link &amp; Angliss Hospital ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 4,497; 31 km E of CBD; part of a Melbourne green wedge, 'nestled into the forest covered foothills of Mount Dandenong' and Dandenong Ranges National Park incl. Doongalla Forest; bushy parks (Wicks Reserve) and farmland [Wikipedia The Basin]. N 8 consistent. Village: shops round 'The Basin Triangle' 'amidst a village atmosphere': licensed post office, two pubs, cafés, greengrocer, butcher, bookstore [Wikipedia]; R 7 consistent. Shops: no supermarket listed; Q 4 consistent. Transport: no station; bus 755 to Bayswater, Boronia and Ferntree Gully stations [Wikipedia]; S 3 consistent. Indian community: Vinayagar Hindu Temple is in the suburb [Wikipedia; Victorian Places 'a Hindu temple']; residents India-born 0.2%, Indian ancestry 0.9%, Hinduism 0.5% [ABS 2021 GCP SAL22496]; P 4 rests on the temple, not on residents. Hazards: 'topography causes strong wind which can fan severe fires'; 'much of the area is also flood prone' [Victorian Places]. City trip: 31 km [Wikipedia]; journey time not stated; V 4 estimate. NOT checked: GPs, bus frequency, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA25" s="16" t="inlineStr">
@@ -9868,6 +11011,51 @@
           <t>AVM house value ($845,187) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK25" s="22" t="inlineStr">
+        <is>
+          <t>SAL22496</t>
+        </is>
+      </c>
+      <c r="AL25" s="32" t="n">
+        <v>4497</v>
+      </c>
+      <c r="AM25" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AN25" s="33" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="AO25" s="33" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AP25" s="33" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="AQ25" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR25" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AS25" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AT25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" s="33" t="n">
+        <v>0.08199999999999999</v>
+      </c>
+      <c r="AV25" s="22" t="inlineStr">
+        <is>
+          <t>German 1.8%; Mandarin 1.1%; Italian 0.5%</t>
+        </is>
+      </c>
+      <c r="AW25" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="15">
       <c r="A26" s="18" t="inlineStr">
@@ -9970,7 +11158,7 @@
       </c>
       <c r="Z26" s="18" t="inlineStr">
         <is>
-          <t>Township shopping &amp; community hub; verify non-rail transport, fire exposure &amp; ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Township shopping &amp; community hub; verify non-rail transport, fire exposure &amp; ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 6,900; 33 km E of CBD at the foothills of Mount Dandenong, altitude 91-324 m [Wikipedia Montrose]. Nature: 'five bush reserves and two linear reserves'; government buy-back of steep land to protect bush; houses lost to fire in 1961 [Victorian Places]; N 8 consistent. Village: shopping area at Mount Dandenong and Swansea Rds with community centre and pioneer cottage; strong local preservation groups [Victorian Places]; R 6 consistent. Train: no station; 'not far from the Mooroolbark railway station' [Victorian Places]; S 3 consistent (bus not checked). Indian community: India-born 0.4%, Hinduism 0.2% [ABS 2021 GCP SAL21736]; P 3 generous (1-2 arguable). City trip: 33 km, no station; V 4 estimate. NOT checked: GPs, supermarket, bus. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA26" s="16" t="inlineStr">
@@ -10021,6 +11209,51 @@
           <t>AVM house value ($968,458) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK26" s="22" t="inlineStr">
+        <is>
+          <t>SAL21736</t>
+        </is>
+      </c>
+      <c r="AL26" s="32" t="n">
+        <v>6900</v>
+      </c>
+      <c r="AM26" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN26" s="33" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="AO26" s="33" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="AP26" s="33" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AQ26" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AR26" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AS26" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT26" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU26" s="33" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AV26" s="22" t="inlineStr">
+        <is>
+          <t>German 0.5%; Greek 0.3%; Italian 0.3%</t>
+        </is>
+      </c>
+      <c r="AW26" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="15">
       <c r="A27" s="18" t="inlineStr">
@@ -10123,7 +11356,7 @@
       </c>
       <c r="Z27" s="18" t="inlineStr">
         <is>
-          <t>Warburton Rail Trail &amp; Aqueduct Trail (no passenger rail); verify Maroondah ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Warburton Rail Trail &amp; Aqueduct Trail (no passenger rail); verify Maroondah ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 9,799; 37 km E of CBD, in a bend of Olinda Creek [Wikipedia Mount Evelyn]. Nature: Mount Evelyn Forest (part of Dandenong Ranges National Park) in the south; Warburton Rail Trail and Aqueduct Walk pass through [Wikipedia; Victorian Places]; N 8 consistent. Village: shopping centre west of the former station 'accompanied by several community meeting places and churches' [Victorian Places]; R 6 consistent. Train: railway closed 1965, now the rail trail [Wikipedia]; no station; S 3 consistent (bus not checked). Shops: supermarket not named; Q 5 estimate. Indian community: India-born 0.2%, Hinduism 0.2% [ABS 2021 GCP SAL21795]; P 2 consistent (1 arguable). City trip: 37 km, no rail; V 4 estimate. NOT checked: GPs, supermarket, bus, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA27" s="16" t="inlineStr">
@@ -10174,6 +11407,51 @@
           <t>AVM house value ($915,472) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK27" s="22" t="inlineStr">
+        <is>
+          <t>SAL21795</t>
+        </is>
+      </c>
+      <c r="AL27" s="32" t="n">
+        <v>9799</v>
+      </c>
+      <c r="AM27" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="AN27" s="33" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="AO27" s="33" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="AP27" s="33" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AQ27" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR27" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AS27" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT27" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU27" s="33" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AV27" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.4%; German 0.2%; French 0.2%</t>
+        </is>
+      </c>
+      <c r="AW27" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="15">
       <c r="A28" s="18" t="inlineStr">
@@ -10327,6 +11605,51 @@
           <t>AVM house value ($898,896) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK28" s="22" t="inlineStr">
+        <is>
+          <t>SAL20682</t>
+        </is>
+      </c>
+      <c r="AL28" s="32" t="n">
+        <v>28608</v>
+      </c>
+      <c r="AM28" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN28" s="33" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="AO28" s="33" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="AP28" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AQ28" s="33" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AR28" s="33" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="AS28" s="33" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AT28" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AU28" s="33" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="AV28" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 3.5%; Cantonese 1.2%; Hindi 0.8%</t>
+        </is>
+      </c>
+      <c r="AW28" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="15">
       <c r="A29" s="18" t="inlineStr">
@@ -10477,6 +11800,51 @@
       <c r="AJ29" s="22" t="inlineStr">
         <is>
           <t>Published house price ($620,000) is under $1.5M cap.</t>
+        </is>
+      </c>
+      <c r="AK29" s="22" t="inlineStr">
+        <is>
+          <t>SAL22698</t>
+        </is>
+      </c>
+      <c r="AL29" s="32" t="n">
+        <v>19856</v>
+      </c>
+      <c r="AM29" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AN29" s="33" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="AO29" s="33" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="AP29" s="33" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AQ29" s="33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AR29" s="33" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AS29" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AT29" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AU29" s="33" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="AV29" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 0.8%; Punjabi 0.4%; Italian 0.3%</t>
+        </is>
+      </c>
+      <c r="AW29" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -10612,6 +11980,51 @@
           <t>AVM house value ($1,610,862) is over the $1.5M cap; needs a documented search for 3+ bed homes under the cap.</t>
         </is>
       </c>
+      <c r="AK30" s="22" t="inlineStr">
+        <is>
+          <t>SAL21793</t>
+        </is>
+      </c>
+      <c r="AL30" s="32" t="n">
+        <v>18734</v>
+      </c>
+      <c r="AM30" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AN30" s="33" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="AO30" s="33" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="AP30" s="33" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AQ30" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AR30" s="33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AS30" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AT30" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU30" s="33" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="AV30" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 0.8%; Greek 0.7%; Italian 0.5%</t>
+        </is>
+      </c>
+      <c r="AW30" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="15">
       <c r="A31" s="18" t="inlineStr">
@@ -10763,6 +12176,51 @@
       <c r="AJ31" s="22" t="inlineStr">
         <is>
           <t>AVM house value ($1,096,505) is under $1.5M cap. Not a sale median.</t>
+        </is>
+      </c>
+      <c r="AK31" s="22" t="inlineStr">
+        <is>
+          <t>SAL21763</t>
+        </is>
+      </c>
+      <c r="AL31" s="32" t="n">
+        <v>25759</v>
+      </c>
+      <c r="AM31" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="AN31" s="33" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="AO31" s="33" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="AP31" s="33" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AQ31" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AR31" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AS31" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT31" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU31" s="33" t="n">
+        <v>0.05599999999999999</v>
+      </c>
+      <c r="AV31" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.7%; Greek 0.6%; Spanish 0.4%</t>
+        </is>
+      </c>
+      <c r="AW31" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -10897,6 +12355,51 @@
           <t>Published house price ($715,000) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK32" s="22" t="inlineStr">
+        <is>
+          <t>SAL20575</t>
+        </is>
+      </c>
+      <c r="AL32" s="32" t="n">
+        <v>7646</v>
+      </c>
+      <c r="AM32" s="22" t="n">
+        <v>48</v>
+      </c>
+      <c r="AN32" s="33" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="AO32" s="33" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="AP32" s="33" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AQ32" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR32" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AS32" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AT32" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" s="33" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="AV32" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.6%; Greek 0.4%; German 0.4%</t>
+        </is>
+      </c>
+      <c r="AW32" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="15">
       <c r="A33" s="18" t="inlineStr">
@@ -10998,7 +12501,7 @@
       </c>
       <c r="Z33" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 24.3% aged 65+, 8.1% non-Eng HH. Tough practicality test on winter comfort, fire risk &amp; distant ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>ABS 2021: 24.3% aged 65+, 8.1% non-Eng HH. Tough practicality test on winter comfort, fire risk &amp; distant ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 2,020; on the Yarra River, 76 km E of CBD [Wikipedia Warburton] (60 km per Victorian Places), foothills of the Great Dividing Range, adjoining Yarra State Forest via East Warburton [Victorian Places]. Nature: extensive walking trails, Warburton Bridges and River Walk, rail trail to Lilydale [Victorian Places]; N 10 consistent. Village: main street mostly retail, constrained by floodplain to the north; B&amp;Bs, health resorts, golf course, festivals [Victorian Places]; R 8 consistent. Train: line closed (now rail trail) [Victorian Places]; S 1 consistent. Indian community: India-born 0.3%, Hinduism 0.4% [ABS 2021 GCP SAL22689]; P 1 consistent. Older: median age 50; 13.7% birthplace not stated [ABS]. City trip: 60-76 km, no rail; V 1 consistent. NOT checked: GPs, supermarket, bus, flood overlay. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA33" s="16" t="inlineStr">
@@ -11047,6 +12550,51 @@
       <c r="AJ33" s="22" t="inlineStr">
         <is>
           <t>Published house price ($717,500) is under $1.5M cap.</t>
+        </is>
+      </c>
+      <c r="AK33" s="22" t="inlineStr">
+        <is>
+          <t>SAL22689</t>
+        </is>
+      </c>
+      <c r="AL33" s="32" t="n">
+        <v>2020</v>
+      </c>
+      <c r="AM33" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="AN33" s="33" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="AO33" s="33" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="AP33" s="33" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="AQ33" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AR33" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AS33" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AT33" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU33" s="33" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AV33" s="22" t="inlineStr">
+        <is>
+          <t>German 0.8%; Japanese 0.5%; Polish 0.3%</t>
+        </is>
+      </c>
+      <c r="AW33" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
     </row>
@@ -11181,6 +12729,51 @@
           <t>Published house price ($978,750) is under $1.5M cap.</t>
         </is>
       </c>
+      <c r="AK34" s="22" t="inlineStr">
+        <is>
+          <t>SAL22577</t>
+        </is>
+      </c>
+      <c r="AL34" s="32" t="n">
+        <v>1382</v>
+      </c>
+      <c r="AM34" s="22" t="n">
+        <v>56</v>
+      </c>
+      <c r="AN34" s="33" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="AO34" s="33" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="AP34" s="33" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="AQ34" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR34" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AS34" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT34" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU34" s="33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AV34" s="22" t="inlineStr">
+        <is>
+          <t>French 0.8%; Croatian 0.4%; Turkish 0.3%</t>
+        </is>
+      </c>
+      <c r="AW34" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="15">
       <c r="A35" s="18" t="inlineStr">
@@ -11283,7 +12876,7 @@
       </c>
       <c r="Z35" s="18" t="inlineStr">
         <is>
-          <t>Parks Vic documents severe-weather/fire closures; bus 694 to Belgrave; verify winter damp, slopes &amp; insurance. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count.</t>
+          <t>Parks Vic documents severe-weather/fire closures; bus 694 to Belgrave; verify winter damp, slopes &amp; insurance. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 1,773; Dandenong Ranges township at the southern foot of Mount Dandenong, 37 km E of Melbourne [Wikipedia Olinda; Victorian Places]. Nature: Dandenong Ranges Botanic Garden (National Rhododendron Garden), R.J. Hamer Arboretum, Olinda Falls and Cascade walk, many walking trails [Wikipedia; Victorian Places]; N 10 consistent. Village: 'the highest number of hospitality, gallery and garden attractions of any location in the Dandenongs'; cafés, galleries, craft shops; shopping centre with hotel and post office [Victorian Places]; R 9 consistent. Shops: small centre, no supermarket named; Q 3 consistent. Train: none named; S 2 consistent. Indian community: India-born 0.2%, Hinduism 0.6% [ABS 2021 GCP SAL22009]; P 2 consistent (1 arguable). City trip: 37 km, no rail; V 3 estimate. NOT checked: GPs, bus, bushfire overlay. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA35" s="16" t="inlineStr">
@@ -11334,6 +12927,51 @@
           <t>AVM house value ($1,020,069) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK35" s="22" t="inlineStr">
+        <is>
+          <t>SAL22009</t>
+        </is>
+      </c>
+      <c r="AL35" s="32" t="n">
+        <v>1773</v>
+      </c>
+      <c r="AM35" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AN35" s="33" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="AO35" s="33" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="AP35" s="33" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="AQ35" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR35" s="33" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AS35" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AT35" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU35" s="33" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="AV35" s="22" t="inlineStr">
+        <is>
+          <t>French 1.5%; Mandarin 0.8%; Japanese 0.5%</t>
+        </is>
+      </c>
+      <c r="AW35" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="15">
       <c r="A36" s="18" t="inlineStr">
@@ -11436,7 +13074,7 @@
       </c>
       <c r="Z36" s="18" t="inlineStr">
         <is>
-          <t>High tourism traffic on weekends; check everyday grocery/medical convenience &amp; bushfire overlay. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count.</t>
+          <t>High tourism traffic on weekends; check everyday grocery/medical convenience &amp; bushfire overlay. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 970; village ~500 m up in a saddle on the Dandenong Ranges ridgeline; much of the locality's west is Dandenong Ranges National Park; Sassafras Creek's banks almost entirely protected public land; Dandenong Ranges Tourist Track runs 15 km beside the creek [Wikipedia Sassafras]. N 10 consistent. Village: tourist village of boutique shops, cafés, Devonshire tea, toy and antique shops, nurseries [Wikipedia]; 'has a shopping centre, a hall, a school' [Victorian Places]; R 9 consistent. Shops: small centre only, no supermarket named; Q 3 consistent (estimate). Train: no station named in either source; S 2 consistent. Indian community: India-born 0, Hinduism 0.0% [ABS 2021 GCP SAL22239]; P 2 generous (1 arguable). City trip: 43 km E of CBD [Wikipedia]; journey time not stated; V 3 estimate. Hazard: area has burnt repeatedly since the 1850s, most recently 1962 [Wikipedia]. Small population: ABS perturbs small counts. NOT checked: GPs, supermarket, bus, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA36" s="16" t="inlineStr">
@@ -11487,6 +13125,51 @@
           <t>AVM house value ($1,006,318) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK36" s="22" t="inlineStr">
+        <is>
+          <t>SAL22239</t>
+        </is>
+      </c>
+      <c r="AL36" s="32" t="n">
+        <v>970</v>
+      </c>
+      <c r="AM36" s="22" t="n">
+        <v>47</v>
+      </c>
+      <c r="AN36" s="33" t="n">
+        <v>0.193</v>
+      </c>
+      <c r="AO36" s="33" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="AP36" s="33" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="AQ36" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR36" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AS36" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT36" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU36" s="33" t="n">
+        <v>0.07200000000000001</v>
+      </c>
+      <c r="AV36" s="22" t="inlineStr">
+        <is>
+          <t>German 1.0%; Japanese 0.9%; Russian 0.7%</t>
+        </is>
+      </c>
+      <c r="AW36" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="15">
       <c r="A37" s="18" t="inlineStr">
@@ -11589,7 +13272,7 @@
       </c>
       <c r="Z37" s="18" t="inlineStr">
         <is>
-          <t>Requires property-specific slope, tree-fall, insurance &amp; emergency egress verification. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count.</t>
+          <t>Requires property-specific slope, tree-fall, insurance &amp; emergency egress verification. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 1,271; 44 km E of CBD [Wikipedia Mount Dandenong] (35 km per Victorian Places); the 633 m peak is the highest in the Ranges. Nature: Doongalla Forest (Dandenong Ranges National Park) is in the suburb; William Ricketts Sanctuary; Burke's Lookout; fine gardens; light snow a few times most years [Victorian Places; Wikipedia]; N 10 consistent. Village: 'a small shopping centre and several restaurants' [Victorian Places]; R 7 consistent. Shops: Q 2 consistent. Train: none named; S 1 consistent. Indian community: India-born 0.6%, Hinduism 0.2% [ABS 2021 GCP SAL21787]; P 2 consistent. City trip: 35-44 km, no rail; V 3 estimate. Winter cold and snow are a consideration for older residents. NOT checked: GPs, bus. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA37" s="16" t="inlineStr">
@@ -11640,6 +13323,51 @@
           <t>AVM house value ($982,029) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK37" s="22" t="inlineStr">
+        <is>
+          <t>SAL21787</t>
+        </is>
+      </c>
+      <c r="AL37" s="32" t="n">
+        <v>1271</v>
+      </c>
+      <c r="AM37" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="AN37" s="33" t="n">
+        <v>0.218</v>
+      </c>
+      <c r="AO37" s="33" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AP37" s="33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AQ37" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AR37" s="33" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AS37" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT37" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU37" s="33" t="n">
+        <v>0.05599999999999999</v>
+      </c>
+      <c r="AV37" s="22" t="inlineStr">
+        <is>
+          <t>German 0.9%; Afrikaans 0.9%; Spanish 0.6%</t>
+        </is>
+      </c>
+      <c r="AW37" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="15">
       <c r="A38" s="18" t="inlineStr">
@@ -11742,7 +13470,7 @@
       </c>
       <c r="Z38" s="18" t="inlineStr">
         <is>
-          <t>Emerald Lake precinct; separate from ridge villages—verify routine services &amp; ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Emerald Lake precinct; separate from ridge villages—verify routine services &amp; ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 5,890; 44 km SE of CBD, Shires of Cardinia and Yarra Ranges [Wikipedia Emerald]. Nature: Emerald Lake park with walking tracks; Cardinia Reservoir Park (kangaroos, wombats); smaller reserves [Wikipedia; Victorian Places]; N 9 consistent. Village: 'an active shopping area', cooperative-owned hardware store, museum, golf club [Victorian Places]; R 8 consistent. Shops: Woolworths supermarket since 2011 [Victorian Places]; Q 6 consistent. Train: Puffing Billy heritage steam railway only (3 stations in Emerald) [Wikipedia]; S 2 consistent. Indian community: India-born 0.1%, Hinduism 0.0% [ABS 2021 GCP SAL20868]; P 2 generous (1 arguable). City trip: 44 km, no commuter rail; V 3 estimate. NOT checked: GPs, bus. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA38" s="16" t="inlineStr">
@@ -11793,6 +13521,51 @@
           <t>AVM house value ($980,699) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK38" s="22" t="inlineStr">
+        <is>
+          <t>SAL20868</t>
+        </is>
+      </c>
+      <c r="AL38" s="32" t="n">
+        <v>5890</v>
+      </c>
+      <c r="AM38" s="22" t="n">
+        <v>43</v>
+      </c>
+      <c r="AN38" s="33" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="AO38" s="33" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="AP38" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AQ38" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AR38" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AS38" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT38" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU38" s="33" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="AV38" s="22" t="inlineStr">
+        <is>
+          <t>Spanish 0.7%; German 0.5%; Japanese 0.5%</t>
+        </is>
+      </c>
+      <c r="AW38" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="15">
       <c r="A39" s="18" t="inlineStr">
@@ -11895,7 +13668,7 @@
       </c>
       <c r="Z39" s="18" t="inlineStr">
         <is>
-          <t>Belgrave line; compare flatter pockets and housing stock against Upper Ferntree Gully. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. OnTheHouse shows the same house AVM ($872,133) for Ferntree Gully and Upper Ferntree Gully (same postcode) — treat as postcode-level, weak. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price = postcode-level AVM shared with Upper FTG.</t>
+          <t>Belgrave line; compare flatter pockets and housing stock against Upper Ferntree Gully. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. OnTheHouse shows the same house AVM ($872,133) for Ferntree Gully and Upper Ferntree Gully (same postcode) — treat as postcode-level, weak. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price = postcode-level AVM shared with Upper FTG. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 27,398; foothills of the Dandenong Ranges, 30 km E of CBD [Wikipedia Ferntree Gully]. Nature: large part of Dandenong Ranges National Park forms the backdrop; eastern boundary is the National Park; One Tree Hill; 'high fire risk area' near the park [Wikipedia]; N 6 consistent (village end greener). Shops: Mountain Gate Shopping Centre; Ferntree Gully Village with supermarkets, greengrocers, butchers, cafés; two supermarkets on Burwood Hwy [Wikipedia; Victorian Places]; Q 8 consistent. Village: historic village at the station, rest is 'mostly a large suburban area' [Victorian Places]; R 4 consistent. Train: 'one of the busiest railway stations in the City of Knox' (Belgrave line) [Wikipedia]; S 8 consistent. Indian community: India-born 2.3%, Indian ancestry 3.1%, Hinduism 2.4% [ABS 2021 GCP SAL20917]; P 5 plausible (4 arguable). City trip: 30 km by train; V 6 estimate. NOT checked: GPs by name, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA39" s="16" t="inlineStr">
@@ -11946,6 +13719,51 @@
           <t>AVM house value ($872,133) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK39" s="22" t="inlineStr">
+        <is>
+          <t>SAL20917</t>
+        </is>
+      </c>
+      <c r="AL39" s="32" t="n">
+        <v>27398</v>
+      </c>
+      <c r="AM39" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AN39" s="33" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="AO39" s="33" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="AP39" s="33" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AQ39" s="33" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AR39" s="33" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="AS39" s="33" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AT39" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AU39" s="33" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="AV39" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 3.7%; Cantonese 1.5%; Sinhalese 1.2%</t>
+        </is>
+      </c>
+      <c r="AW39" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="15">
       <c r="A40" s="18" t="inlineStr">
@@ -12099,6 +13917,51 @@
           <t>AVM house value ($935,845) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK40" s="22" t="inlineStr">
+        <is>
+          <t>SAL20224</t>
+        </is>
+      </c>
+      <c r="AL40" s="32" t="n">
+        <v>50298</v>
+      </c>
+      <c r="AM40" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="AN40" s="33" t="n">
+        <v>0.142</v>
+      </c>
+      <c r="AO40" s="33" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="AP40" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AQ40" s="33" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="AR40" s="33" t="n">
+        <v>0.07400000000000001</v>
+      </c>
+      <c r="AS40" s="33" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AT40" s="33" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AU40" s="33" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="AV40" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 4.0%; Sinhalese 3.8%; Hindi 1.5%</t>
+        </is>
+      </c>
+      <c r="AW40" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="15">
       <c r="A41" s="18" t="inlineStr">
@@ -12201,7 +14064,7 @@
       </c>
       <c r="Z41" s="18" t="inlineStr">
         <is>
-          <t>Sweetwater Creek nature reserve; weaker station walk than central Frankston. Promoted to Active 26 Oct 2026 as a bush-plus-bay overlap candidate. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): No station; buses to Frankston. Olivers Hill bay views; Daveys Bay is in Mt Eliza, so beach access not in suburb: U lowered 7-&gt;6. No major shops, small strips only: Q lowered 6-&gt;5 (Wikipedia). GP: Baxter Park Medical Centre (healthdirect). Sweetwater Creek reserve. N, P, R, V remain estimates.</t>
+          <t>Sweetwater Creek nature reserve; weaker station walk than central Frankston. Promoted to Active 26 Oct 2026 as a bush-plus-bay overlap candidate. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): No station; buses to Frankston. Olivers Hill bay views; Daveys Bay is in Mt Eliza, so beach access not in suburb: U lowered 7-&gt;6. No major shops, small strips only: Q lowered 6-&gt;5 (Wikipedia). GP: Baxter Park Medical Centre (healthdirect). Sweetwater Creek reserve. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: elevated land where Sweetwater Creek descends from Mount Eliza; Frankston Reservoir; much stayed open country until postwar [Victorian Places Frankston South]; N 7 plausible. Village: 'no major shopping areas'; small strips on Norman Ave, Foot St and Overport Rd; south served by Mount Eliza village [Wikipedia Frankston South]; R 6 generous (5 arguable). Indian community: India-born 0.9%, Hinduism 0.4%; Malayalam 0.8% at home [ABS 2021 GCP SAL20949]; P 3 consistent (2 arguable). Older: median age 44, 22.0% aged 65+ [ABS]. City trip: 41-43 km SE, no station [Wikipedia; Victorian Places]; V 5 estimate. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA41" s="16" t="inlineStr">
@@ -12252,6 +14115,51 @@
           <t>AVM house value ($1,195,044) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK41" s="22" t="inlineStr">
+        <is>
+          <t>SAL20949</t>
+        </is>
+      </c>
+      <c r="AL41" s="32" t="n">
+        <v>18801</v>
+      </c>
+      <c r="AM41" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="AN41" s="33" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AO41" s="33" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="AP41" s="33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AQ41" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AR41" s="33" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AS41" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AT41" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU41" s="33" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AV41" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 1.2%; Greek 1.0%; Malayalam 0.8%</t>
+        </is>
+      </c>
+      <c r="AW41" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="15">
       <c r="A42" s="18" t="inlineStr">
@@ -12354,7 +14262,7 @@
       </c>
       <c r="Z42" s="18" t="inlineStr">
         <is>
-          <t>Hurstbridge rail terminus; test whether extra distance over Diamond Creek/Eltham adds value. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Hurstbridge rail terminus; test whether extra distance over Diamond Creek/Eltham adds value. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 3,554; 28 km NE of CBD, Shire of Nillumbik [Wikipedia Hurstbridge]. Train: terminus of the line from Melbourne via Eltham (1912; electrified 1926) [Victorian Places]; station opposite the post office [Wikipedia]; S 6 consistent (frequency not checked). Nature: 'two extensive parklands along the Diamond Creek and two native flora reserves', Ferguson's Paddock with monthly farmers' market [Victorian Places]; N 8 consistent. Village: 'The Main Road shops retain many original building elements'; Anzac Avenue avenue of honour [Victorian Places]; R 8 consistent. Shops: 'an active shopping centre' [Victorian Places]; supermarket not named; Q 5 estimate. Indian community: India-born 0.3%, Hinduism 0.3% [ABS 2021 GCP SAL21223]; 86.1% Australia-born [Wikipedia citing ABS]; P 1 consistent. City trip: 28 km by train; journey time not stated; V 5 estimate. NOT checked: GPs, supermarket, train frequency. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA42" s="16" t="inlineStr">
@@ -12403,6 +14311,51 @@
       <c r="AJ42" s="22" t="inlineStr">
         <is>
           <t>AVM house value ($980,767) is under $1.5M cap. Not a sale median.</t>
+        </is>
+      </c>
+      <c r="AK42" s="22" t="inlineStr">
+        <is>
+          <t>SAL21223</t>
+        </is>
+      </c>
+      <c r="AL42" s="32" t="n">
+        <v>3554</v>
+      </c>
+      <c r="AM42" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN42" s="33" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="AO42" s="33" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AP42" s="33" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AQ42" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AR42" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AS42" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT42" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU42" s="33" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AV42" s="22" t="inlineStr">
+        <is>
+          <t>Spanish 0.4%; Japanese 0.3%; Italian 0.3%</t>
+        </is>
+      </c>
+      <c r="AW42" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -12538,6 +14491,51 @@
           <t>AVM house value ($722,940) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK43" s="22" t="inlineStr">
+        <is>
+          <t>SAL20111</t>
+        </is>
+      </c>
+      <c r="AL43" s="32" t="n">
+        <v>5378</v>
+      </c>
+      <c r="AM43" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN43" s="33" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="AO43" s="33" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AP43" s="33" t="n">
+        <v>0.05400000000000001</v>
+      </c>
+      <c r="AQ43" s="33" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AR43" s="33" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AS43" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AT43" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AU43" s="33" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="AV43" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 0.8%; Punjabi 0.8%; Japanese 0.5%</t>
+        </is>
+      </c>
+      <c r="AW43" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. CAVEAT: Ballarat Central locality only (CBD, pop 5,378), not the whole city.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="15">
       <c r="A44" s="18" t="inlineStr">
@@ -12671,6 +14669,51 @@
           <t>AVM house value ($658,696) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK44" s="22" t="inlineStr">
+        <is>
+          <t>SAL20208</t>
+        </is>
+      </c>
+      <c r="AL44" s="32" t="n">
+        <v>5652</v>
+      </c>
+      <c r="AM44" s="22" t="n">
+        <v>43</v>
+      </c>
+      <c r="AN44" s="33" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="AO44" s="33" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="AP44" s="33" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AQ44" s="33" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="AR44" s="33" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AS44" s="33" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AT44" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AU44" s="33" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AV44" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 0.7%; Punjabi 0.6%; Malayalam 0.4%</t>
+        </is>
+      </c>
+      <c r="AW44" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. CAVEAT: Bendigo locality (central, pop 5,652), not the whole city.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="15">
       <c r="A45" s="18" t="inlineStr">
@@ -12773,7 +14816,7 @@
       </c>
       <c r="Z45" s="18" t="inlineStr">
         <is>
-          <t>Compare Rosebud vs Frankston ED access and year-round vs holiday-town feel. 27 Oct 2026: drive times, ED and AVM price added. ED: Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Compare Rosebud vs Frankston ED access and year-round vs holiday-town feel. 27 Oct 2026: drive times, ED and AVM price added. ED: Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 6,626; seaside suburb ~58 km S of Melbourne between Safety Beach, Rosebud and Red Hill; Arthurs Seat, the Peninsula's highest point, overlooks it [Wikipedia Dromana; Victorian Places]. Beach and pier [Victorian Places]; U 9 consistent. Nature: bay plus the Arthurs Seat backdrop; N 7 consistent. Village: historic local centre (pier 1862, Dromana Hotel 1857, heritage-listed Heronswood garden) [Victorian Places]; R 6 consistent. Train: no station named; S 2 consistent. Indian community: India-born 0.3%, Hinduism 0.2% [ABS 2021 GCP SAL20788]; P 2 generous (1 arguable). Older area: median age 50, 29.1% aged 65+ [ABS]. City trip: ~58 km, no rail; V 2 consistent. NOT checked: GPs, supermarket, bus. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA45" s="16" t="inlineStr">
@@ -12822,6 +14865,51 @@
       <c r="AJ45" s="22" t="inlineStr">
         <is>
           <t>AVM house value ($906,318) is under $1.5M cap. Not a sale median.</t>
+        </is>
+      </c>
+      <c r="AK45" s="22" t="inlineStr">
+        <is>
+          <t>SAL20788</t>
+        </is>
+      </c>
+      <c r="AL45" s="32" t="n">
+        <v>6626</v>
+      </c>
+      <c r="AM45" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="AN45" s="33" t="n">
+        <v>0.291</v>
+      </c>
+      <c r="AO45" s="33" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="AP45" s="33" t="n">
+        <v>0.08900000000000001</v>
+      </c>
+      <c r="AQ45" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AR45" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AS45" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT45" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU45" s="33" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="AV45" s="22" t="inlineStr">
+        <is>
+          <t>Greek 3.3%; Italian 1.8%; Spanish 0.4%</t>
+        </is>
+      </c>
+      <c r="AW45" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -12957,6 +15045,51 @@
           <t>AVM house value ($747,758) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK46" s="22" t="inlineStr">
+        <is>
+          <t>SAL20516</t>
+        </is>
+      </c>
+      <c r="AL46" s="32" t="n">
+        <v>7506</v>
+      </c>
+      <c r="AM46" s="22" t="n">
+        <v>52</v>
+      </c>
+      <c r="AN46" s="33" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="AO46" s="33" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="AP46" s="33" t="n">
+        <v>0.07200000000000001</v>
+      </c>
+      <c r="AQ46" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AR46" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AS46" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT46" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU46" s="33" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AV46" s="22" t="inlineStr">
+        <is>
+          <t>German 0.5%; Spanish 0.4%; French 0.3%</t>
+        </is>
+      </c>
+      <c r="AW46" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="15">
       <c r="A47" s="18" t="inlineStr">
@@ -13059,7 +15192,7 @@
       </c>
       <c r="Z47" s="18" t="inlineStr">
         <is>
-          <t>Bass Coast Health Wonthaggi Hospital; verify ED capability &amp; GW travel time before promoting. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. GW drive 88 min, 2 min under cap.</t>
+          <t>Bass Coast Health Wonthaggi Hospital; verify ED capability &amp; GW travel time before promoting. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. GW drive 88 min, 2 min under cap. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 5,215; 132 km SE of Melbourne by road (110 km straight line) between Western Port and Wilsons Promontory; largest town in South Gippsland [Wikipedia Wonthaggi; Victorian Places]. Shops: 'many large chain stores ... four major supermarkets, cafes, restaurants, pubs ... a hospital' [Wikipedia]; Q 7 consistent (8 arguable). Village: former coal-mining town, Union Community Arts Centre [Wikipedia]; R 5 consistent. Nature: coastal setting, Bunurong Marine and Coastal Park to the SE [Wikipedia]; N 6 consistent. Beach: town is inland; nearest coast Cape Paterson (not measured); U 6 plausible. Train: none (old Hicksborough station gone) [Victorian Places]; S 1 consistent. Indian community: India-born 0.8%, Hinduism 0.7% [ABS 2021 GCP SAL22829]; P 1 consistent. Oldest population on the list: median age 55, 35.2% aged 65+ [ABS]. City trip: 132 km road, no rail; V 1 consistent. NOT checked: GPs, beach distance. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA47" s="16" t="inlineStr">
@@ -13108,6 +15241,51 @@
       <c r="AJ47" s="22" t="inlineStr">
         <is>
           <t>AVM house value ($587,666) is under $1.5M cap. Not a sale median.</t>
+        </is>
+      </c>
+      <c r="AK47" s="22" t="inlineStr">
+        <is>
+          <t>SAL22829</t>
+        </is>
+      </c>
+      <c r="AL47" s="32" t="n">
+        <v>5215</v>
+      </c>
+      <c r="AM47" s="22" t="n">
+        <v>55</v>
+      </c>
+      <c r="AN47" s="33" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="AO47" s="33" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="AP47" s="33" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="AQ47" s="33" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AR47" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AS47" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AT47" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU47" s="33" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AV47" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.9%; Malayalam 0.6%; German 0.3%</t>
+        </is>
+      </c>
+      <c r="AW47" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
     </row>
@@ -13243,6 +15421,51 @@
           <t>AVM house value ($823,858) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK48" s="22" t="inlineStr">
+        <is>
+          <t>SAL21235</t>
+        </is>
+      </c>
+      <c r="AL48" s="32" t="n">
+        <v>6526</v>
+      </c>
+      <c r="AM48" s="22" t="n">
+        <v>54</v>
+      </c>
+      <c r="AN48" s="33" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="AO48" s="33" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="AP48" s="33" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="AQ48" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AR48" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AS48" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT48" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU48" s="33" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AV48" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.7%; German 0.3%; Mandarin 0.3%</t>
+        </is>
+      </c>
+      <c r="AW48" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="15">
       <c r="A49" s="18" t="inlineStr">
@@ -13377,6 +15600,11 @@
           <t>Synthetic test calibration model.</t>
         </is>
       </c>
+      <c r="AW49" t="inlineStr">
+        <is>
+          <t>Excluded test row: no demography.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="15">
       <c r="A50" s="18" t="inlineStr">
@@ -13511,6 +15739,11 @@
           <t>Synthetic test calibration model.</t>
         </is>
       </c>
+      <c r="AW50" t="inlineStr">
+        <is>
+          <t>Excluded test row: no demography.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="15">
       <c r="A51" s="16" t="inlineStr">
@@ -13613,7 +15846,7 @@
       </c>
       <c r="Z51" s="16" t="inlineStr">
         <is>
-          <t>OPEN-MIND VIEWING PICK (nominated by NJD): view for calibration. Verify year-round services vs holiday-town feel, local ED status and drive to a 24-hr public ED, GW drive and price. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Sand bars give safe swimming; pier; Rosebud Village and Port Phillip Plaza each with a supermarket: Q raised 8-&gt;9 (Victorian Places). GPs: Rosebud Medical Clinic and others (healthdirect). N, P, R, V remain estimates.</t>
+          <t>OPEN-MIND VIEWING PICK (nominated by NJD): view for calibration. Verify year-round services vs holiday-town feel, local ED status and drive to a 24-hr public ED, GW drive and price. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Sand bars give safe swimming; pier; Rosebud Village and Port Phillip Plaza each with a supermarket: Q raised 8-&gt;9 (Victorian Places). GPs: Rosebud Medical Clinic and others (healthdirect). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: between the lower slopes of Arthurs Seat, Port Phillip and the Boneo plains; sandy beaches, shallow water; one of the Peninsula's largest foreshore camping areas (summer population can double) [Wikipedia Rosebud]; N 6 consistent. Village: 'the largest and most commercially developed of the towns south of Mornington'; weekend markets; rebuilt pier [Victorian Places; Wikipedia]; R 4 consistent. Health: Rosebud Hospital on Point Nepean Rd; MICA ambulance unit in town [Wikipedia]. Indian community: India-born 0.4%, Hinduism 0.3% [ABS 2021 GCP SAL22198]; P 2 consistent. Older: median age 49, 29.5% aged 65+ [ABS]. City trip: ~60 km S, no rail [Wikipedia; Victorian Places]; V 2 consistent. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA51" s="16" t="inlineStr">
@@ -13664,6 +15897,51 @@
           <t>AVM house value ($753,965) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK51" s="22" t="inlineStr">
+        <is>
+          <t>SAL22198</t>
+        </is>
+      </c>
+      <c r="AL51" s="32" t="n">
+        <v>14381</v>
+      </c>
+      <c r="AM51" s="22" t="n">
+        <v>49</v>
+      </c>
+      <c r="AN51" s="33" t="n">
+        <v>0.295</v>
+      </c>
+      <c r="AO51" s="33" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="AP51" s="33" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="AQ51" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AR51" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AS51" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT51" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU51" s="33" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="AV51" s="22" t="inlineStr">
+        <is>
+          <t>Italian 1.3%; Greek 1.0%; Mandarin 0.3%</t>
+        </is>
+      </c>
+      <c r="AW51" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="15">
       <c r="A52" s="16" t="inlineStr">
@@ -13766,7 +16044,7 @@
       </c>
       <c r="Z52" s="16" t="inlineStr">
         <is>
-          <t>OPEN-MIND VIEWING PICK (nominated by NJD): view for calibration. Verify year-round services vs holiday-town feel, ED access (nearest 24-hr public ED likely Frankston/Peninsula Univ Hospital), GW drive and price. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Bay beach popular for swimming + unpatrolled ocean beach; pier (Wikipedia Rye). GP listing in Rye (healthdirect). Supermarket not confirmed; Q partly estimate. Bus not checked. N, P, R, V remain estimates.</t>
+          <t>OPEN-MIND VIEWING PICK (nominated by NJD): view for calibration. Verify year-round services vs holiday-town feel, ED access (nearest 24-hr public ED likely Frankston/Peninsula Univ Hospital), GW drive and price. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Bay beach popular for swimming + unpatrolled ocean beach; pier (Wikipedia Rye). GP listing in Rye (healthdirect). Supermarket not confirmed; Q partly estimate. Bus not checked. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: bay beach plus the unpatrolled ocean 'back beach' on Bass Strait; locality spans the peninsula [Wikipedia Rye; Victorian Places]; Moonah Links and The Dunes golf links; N 7 consistent. Village: commercial centre overlooking the bay; summer carnival; busy in holidays [Victorian Places; Wikipedia]; R 7 plausible (6 arguable given holiday swings). Indian community: India-born 0.2%, Hinduism 0.2% [ABS 2021 GCP SAL22220]; P 1 consistent. Older: median age 51, 29.2% aged 65+ [ABS]. City trip: 65 km S by straight line [Victorian Places] (Wikipedia gives 94.5 km, likely by road); no rail; V 1 consistent. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA52" s="16" t="inlineStr">
@@ -13817,6 +16095,51 @@
           <t>AVM house value ($918,392) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK52" s="22" t="inlineStr">
+        <is>
+          <t>SAL22220</t>
+        </is>
+      </c>
+      <c r="AL52" s="32" t="n">
+        <v>9438</v>
+      </c>
+      <c r="AM52" s="22" t="n">
+        <v>51</v>
+      </c>
+      <c r="AN52" s="33" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="AO52" s="33" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="AP52" s="33" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="AQ52" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AR52" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AS52" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AT52" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU52" s="33" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="AV52" s="22" t="inlineStr">
+        <is>
+          <t>Greek 2.0%; Italian 1.9%; Croatian 0.4%</t>
+        </is>
+      </c>
+      <c r="AW52" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="15">
       <c r="A53" s="16" t="inlineStr">
@@ -13919,7 +16242,7 @@
       </c>
       <c r="Z53" s="16" t="inlineStr">
         <is>
-          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify train access (nearest V/Line may be Riddells Creek), GW drive, price and nearest major public ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify train access (nearest V/Line may be Riddells Creek), GW drive, price and nearest major public ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Gisborne district pop 14,432 (June 2021) [Wikipedia Gisborne]; SAL pop 10,142 [ABS 2021 GCP SAL21001]; ~54 km NW of Melbourne. Train: station on the Bendigo line, built outside the township (the suburb New Gisborne); V/Line runs to Southern Cross; 'a 50-minute train ride'; 20 min to Sunbury for Metro; Gisborne Transit loop and on-demand bus to the station [Wikipedia]; resolves foundation-report item 14 (station exists, ~3 km out); S 4 low (5 arguable). Shops: town centre with cafés, theatre, galleries, monthly farmers' market and four supermarkets [Wikipedia]; Q 7 consistent (8 arguable). Village: 'country homesteads, tree-lined streets'; planning controls protect the town's character; fast growth [Wikipedia]; R 7 consistent. Nature: 'large leafy blocks' [Wikipedia]; N 7 consistent. Indian community: India-born 0.6%, Hinduism 0.3%, Sikhism 0.4% [ABS]; P 2 consistent. City trip: 45 min drive or 50 min train [Wikipedia]; V 5 consistent (6 arguable). NOT checked: GPs, train frequency. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA53" s="16" t="inlineStr">
@@ -13970,6 +16293,51 @@
           <t>AVM house value ($1,043,843) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK53" s="22" t="inlineStr">
+        <is>
+          <t>SAL21001</t>
+        </is>
+      </c>
+      <c r="AL53" s="32" t="n">
+        <v>10142</v>
+      </c>
+      <c r="AM53" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN53" s="33" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="AO53" s="33" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="AP53" s="33" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="AQ53" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AR53" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AS53" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AT53" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AU53" s="33" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AV53" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.6%; Punjabi 0.4%; Spanish 0.4%</t>
+        </is>
+      </c>
+      <c r="AW53" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="15">
       <c r="A54" s="16" t="inlineStr">
@@ -14072,7 +16440,7 @@
       </c>
       <c r="Z54" s="16" t="inlineStr">
         <is>
-          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify V/Line station and service frequency, GW drive, price and nearest major public ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify V/Line station and service frequency, GW drive, price and nearest major public ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 4,390; southern foothills of the Macedon Ranges, 15 km N of Sunbury, ~45 km from Melbourne [Wikipedia Riddells Creek; Victorian Places]. Nature: 'surrounded by natural bushland'; creek through Wybejong Park; Mount Charlie State Forest to the east [Wikipedia]; N 7 consistent. Village: shopping centre, mechanics' institute (1875), heritage railway bridge and goods shed; Dromkeen children's-literature homestead; shire plan to retain neighbourhood character [Victorian Places; Wikipedia]; R 7 consistent. Train: station on the Bendigo line; express services do not stop [Wikipedia]; S 5 consistent. Shops: supermarket and 12 shops were planned in 2013 [Victorian Places]; built status NOT confirmed; Q 4 estimate. Indian community: India-born 0.3%, Hinduism 0.0% [ABS 2021 GCP SAL22172]; P 2 generous (1 arguable). City trip: ~45 km by V/Line, stopping trains only; V 5 estimate. NOT checked: GPs, supermarket, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA54" s="16" t="inlineStr">
@@ -14123,6 +16491,51 @@
           <t>AVM house value ($994,380) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK54" s="22" t="inlineStr">
+        <is>
+          <t>SAL22172</t>
+        </is>
+      </c>
+      <c r="AL54" s="32" t="n">
+        <v>4390</v>
+      </c>
+      <c r="AM54" s="22" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN54" s="33" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="AO54" s="33" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="AP54" s="33" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="AQ54" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AR54" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AS54" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT54" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU54" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AV54" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.4%; Mandarin 0.3%; Greek 0.3%</t>
+        </is>
+      </c>
+      <c r="AW54" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="15">
       <c r="A55" s="16" t="inlineStr">
@@ -14225,7 +16638,7 @@
       </c>
       <c r="Z55" s="16" t="inlineStr">
         <is>
-          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Likely no train; verify GW drive, price and ED journey (Maroondah/Angliss). Compare with Healesville. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Likely no train; verify GW drive, price and ED journey (Maroondah/Angliss). Compare with Healesville. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 3,012; 55 km NE of CBD [Wikipedia Yarra Glen] (40 km per Victorian Places), just north of the Yarra River flood plain. Nature: open valley farmland and vineyards; heritage Gulf Station farm; Black Saturday 2009 fire killed at least 13 in the Yarra Glen-Steeles Creek area [Victorian Places]; N 8 plausible (open valley more than forest; 7 arguable). Village: 'substantial shopping centre', historic main street with the Grand Hotel (1888), racecourse, showground [Victorian Places]; R 7 consistent; Q 5 plausible (supermarket not named). Train: line closed 1980; tourist railway later disused [Victorian Places]; S 1 consistent. Indian community: India-born 0.1%, Hinduism 0.0% [ABS 2021 GCP SAL22910]; P 1 consistent. City trip: 40-55 km, no rail; V 2 consistent. NOT checked: GPs, bus, flood overlay. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA55" s="16" t="inlineStr">
@@ -14276,6 +16689,51 @@
           <t>AVM house value ($936,458) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK55" s="22" t="inlineStr">
+        <is>
+          <t>SAL22910</t>
+        </is>
+      </c>
+      <c r="AL55" s="32" t="n">
+        <v>3012</v>
+      </c>
+      <c r="AM55" s="22" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN55" s="33" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="AO55" s="33" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="AP55" s="33" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="AQ55" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AR55" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AS55" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT55" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU55" s="33" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AV55" s="22" t="inlineStr">
+        <is>
+          <t>Greek 0.3%; Italian 0.2%; German 0.2%</t>
+        </is>
+      </c>
+      <c r="AW55" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="15">
       <c r="A56" s="16" t="inlineStr">
@@ -14378,7 +16836,7 @@
       </c>
       <c r="Z56" s="16" t="inlineStr">
         <is>
-          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify V/Line station, GW drive, price and ED access (West Gippsland Hospital at Warragul). Compare with Warragul. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify V/Line station, GW drive, price and ED access (West Gippsland Hospital at Warragul). Compare with Warragul. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 15,287; West Gippsland, ~90 km E/SE of Melbourne on the Gippsland rail and road routes [Wikipedia Drouin, Victoria; Victorian Places]. Shops: Woolworths and Coles supermarkets [Wikipedia]; compact civic centre between the station and landscaped Civic Park [Victorian Places]; Q 7 consistent. Train: station beside the shopping precinct on Princes Way [Wikipedia]; Gippsland line [Victorian Places]; S 5 consistent (frequency not checked). Nature: Civic Park, other reserves and a botanic garden; Ficifolia avenue of honour [Victorian Places]; N 5 consistent. Village: growing town with new housing estates and a planned multi-storey retail complex [Wikipedia]; R 6 plausible. Indian community: India-born 0.5%, Hinduism 0.4% [ABS 2021 GCP SAL20790]; P 2 consistent. City trip: ~90 km by V/Line; V 4 estimate. NOT checked: GPs, train journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AA56" s="16" t="inlineStr">
@@ -14429,6 +16887,51 @@
           <t>AVM house value ($701,797) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK56" s="22" t="inlineStr">
+        <is>
+          <t>SAL20790</t>
+        </is>
+      </c>
+      <c r="AL56" s="32" t="n">
+        <v>15287</v>
+      </c>
+      <c r="AM56" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN56" s="33" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="AO56" s="33" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="AP56" s="33" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AQ56" s="33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AR56" s="33" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AS56" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AT56" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AU56" s="33" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AV56" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 0.3%; German 0.3%; Afrikaans 0.2%</t>
+        </is>
+      </c>
+      <c r="AW56" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="15">
       <c r="A57" s="16" t="inlineStr">
@@ -14531,7 +17034,7 @@
       </c>
       <c r="Z57" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Western Health: ED "always open". | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Western Health: ED "always open". | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 11,729; inner suburb 7 km W of CBD [Wikipedia West Footscray]. Indian community: Barkly Village strip has Indian-owned shops incl. 'a particularly large Indian grocery store, Bharat Traders' [Wikipedia]; India-born 3.7% (434), Indian ancestry 3.6%, Hinduism 3.5%; Telugu 1.4% at home (QuickStats, via Wikipedia) [ABS 2021 GCP SAL22756]; P 8 high next to Berwick 7 at 6.1% India-born, but the grocer is real (6-7 arguable). Nature: basalt plains, no bushland named [Wikipedia]; N 2 consistent. Village: Barkly Village strip with grocers, independent supermarket (Sims), new community centre and library [Wikipedia]; R 5 consistent; Q 8 consistent. Train: suburb split by the railway (Sunbury line) [Wikipedia]; S 8 consistent. Younger area: median age 35, 10.0% aged 65+ [ABS]. City trip: 7 km; V 9 consistent. NOT checked: GPs, station frequency. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB57" s="22" t="inlineStr">
@@ -14577,6 +17080,51 @@
           <t>AVM house value ($1,046,286) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK57" s="22" t="inlineStr">
+        <is>
+          <t>SAL22756</t>
+        </is>
+      </c>
+      <c r="AL57" s="32" t="n">
+        <v>11729</v>
+      </c>
+      <c r="AM57" s="22" t="n">
+        <v>35</v>
+      </c>
+      <c r="AN57" s="33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AO57" s="33" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="AP57" s="33" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AQ57" s="33" t="n">
+        <v>0.03700000000000001</v>
+      </c>
+      <c r="AR57" s="33" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="AS57" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AT57" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AU57" s="33" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AV57" s="22" t="inlineStr">
+        <is>
+          <t>Vietnamese 8.2%; Italian 1.8%; Cantonese 1.6%</t>
+        </is>
+      </c>
+      <c r="AW57" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="15">
       <c r="A58" s="16" t="inlineStr">
@@ -14679,7 +17227,7 @@
       </c>
       <c r="Z58" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 8,616; 12 km NE of CBD, ~2 km beyond Heidelberg, on the fringe of the Yarra Valley green belt [Wikipedia Rosanna; Victorian Places]. Nature: 'generous tree cover across hilly streets' (The Age 2019, via Wikipedia); Salt Creek open space on the former golf links, Banyule Creek linear park, Warringal parklands and Banyule Flats by the Yarra [Victorian Places]; N 6 consistent (7 arguable). Village: 'active shopping centre near the railway station'; Woolworths beside the library redevelopment [Victorian Places; Wikipedia]; R 6, Q 7 consistent. Train: recently updated station, Hurstbridge line [Wikipedia; Victorian Places]; S 8 consistent. Indian community: India-born 2.8%, Indian ancestry 3.8%, Hinduism 2.4% [ABS 2021 GCP SAL22194]; P 4 consistent. City trip: 12 km by train; V 8 consistent. NOT checked: GPs, journey time. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB58" s="22" t="inlineStr">
@@ -14725,6 +17273,51 @@
           <t>AVM house value ($1,242,201) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK58" s="22" t="inlineStr">
+        <is>
+          <t>SAL22194</t>
+        </is>
+      </c>
+      <c r="AL58" s="32" t="n">
+        <v>8616</v>
+      </c>
+      <c r="AM58" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN58" s="33" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="AO58" s="33" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="AP58" s="33" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="AQ58" s="33" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AR58" s="33" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AS58" s="33" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="AT58" s="33" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AU58" s="33" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="AV58" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 4.1%; Italian 4.1%; Cantonese 1.4%</t>
+        </is>
+      </c>
+      <c r="AW58" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="15">
       <c r="A59" s="16" t="inlineStr">
@@ -14827,7 +17420,7 @@
       </c>
       <c r="Z59" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two stations; beachside with foreshore reserve and 305 ha wetlands (Wikipedia Seaford). GPs: Seaford Central Medical Clinic, Seaford Beach Family Clinic (healthdirect). Supermarket in suburb NOT confirmed; Q partly estimate. N, P, R, V remain estimates.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two stations; beachside with foreshore reserve and 305 ha wetlands (Wikipedia Seaford). GPs: Seaford Central Medical Clinic, Seaford Beach Family Clinic (healthdirect). Supermarket in suburb NOT confirmed; Q partly estimate. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Seaford Foreshore Reserve is 'one of the few remaining substantial, continuous strands of natural coastal vegetation near Melbourne' along the whole suburb; Kananook walking trail [Wikipedia Seaford]; Edithvale-Seaford Wetland with walking trail and viewing platform; Kananook Creek linear reserve [Victorian Places]; N 5 looks low (6 arguable). Village: small shopping centre and pier near the station, a supermarket; largely cheap postwar housing [Victorian Places]; R 4 consistent. Indian community: India-born 0.6%, Hinduism 0.7% [ABS 2021 GCP SAL22249]; P 4 generous (2 arguable). City trip: 36 km SE on the Frankston line [Wikipedia]; journey time not stated; V 6 estimate. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB59" s="22" t="inlineStr">
@@ -14873,6 +17466,51 @@
           <t>AVM house value ($861,235) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK59" s="22" t="inlineStr">
+        <is>
+          <t>SAL22249</t>
+        </is>
+      </c>
+      <c r="AL59" s="32" t="n">
+        <v>17215</v>
+      </c>
+      <c r="AM59" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AN59" s="33" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="AO59" s="33" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="AP59" s="33" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AQ59" s="33" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="AR59" s="33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AS59" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AT59" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU59" s="33" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="AV59" s="22" t="inlineStr">
+        <is>
+          <t>Greek 0.9%; Russian 0.7%; Mandarin 0.7%</t>
+        </is>
+      </c>
+      <c r="AW59" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="15">
       <c r="A60" s="16" t="inlineStr">
@@ -14975,7 +17613,7 @@
       </c>
       <c r="Z60" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Dandenong and Monash Medical Centre Clayton both 23 min. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station; bay beach (Wikipedia Chelsea). GP: Chelsea Beach Medical Centre (healthdirect). Woolworths Chelsea (grocerize). N, P, R, V remain estimates.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Dandenong and Monash Medical Centre Clayton both 23 min. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station; bay beach (Wikipedia Chelsea). GP: Chelsea Beach Medical Centre (healthdirect). Woolworths Chelsea (grocerize). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: bay beach; Bicentennial Park on a former tip site [Wikipedia Chelsea]; no bushland named; N 4 consistent. Village: 'the most important bayside suburban centre between Mordialloc and Frankston'; much older housing replaced by single-storey units in the 1960s-70s; 'more elderly people than most other Melbourne suburbs' [Wikipedia]; R 5 consistent. Indian community: India-born 1.4%, Indian ancestry 1.8%, Hinduism 0.9% [ABS 2021 GCP SAL20537]; P 4 generous (2-3 arguable). City trip: 30 km SE on the Frankston line [Victorian Places]; V 7 plausible. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB60" s="22" t="inlineStr">
@@ -15021,6 +17659,51 @@
           <t>AVM house value ($1,161,160) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK60" s="22" t="inlineStr">
+        <is>
+          <t>SAL20537</t>
+        </is>
+      </c>
+      <c r="AL60" s="32" t="n">
+        <v>8347</v>
+      </c>
+      <c r="AM60" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="AN60" s="33" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AO60" s="33" t="n">
+        <v>0.244</v>
+      </c>
+      <c r="AP60" s="33" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AQ60" s="33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AR60" s="33" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AS60" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AT60" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU60" s="33" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="AV60" s="22" t="inlineStr">
+        <is>
+          <t>Greek 1.8%; Russian 1.1%; Mandarin 1.1%</t>
+        </is>
+      </c>
+      <c r="AW60" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="15">
       <c r="A61" s="16" t="inlineStr">
@@ -15140,6 +17823,51 @@
           <t>AVM house value ($744,355) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK61" s="22" t="inlineStr">
+        <is>
+          <t>SAL20697</t>
+        </is>
+      </c>
+      <c r="AL61" s="32" t="n">
+        <v>4175</v>
+      </c>
+      <c r="AM61" s="22" t="n">
+        <v>34</v>
+      </c>
+      <c r="AN61" s="33" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="AO61" s="33" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="AP61" s="33" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AQ61" s="33" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AR61" s="33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AS61" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AT61" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU61" s="33" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="AV61" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 0.6%; Tagalog 0.5%; Filipino 0.4%</t>
+        </is>
+      </c>
+      <c r="AW61" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="15">
       <c r="A62" s="16" t="inlineStr">
@@ -15242,7 +17970,7 @@
       </c>
       <c r="Z62" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 3,311; bayside suburb between Dromana and Rosebud, 59 km S of CBD [Wikipedia McCrae; Victorian Places]. Beach: foreshore reserve with camping and picnic areas, yacht club, Rosebud-McCrae Life Saving Club [Victorian Places]; U 9 consistent. Nature: housing climbs the slopes of Arthurs Seat [Victorian Places]; N 8 consistent. Village: shops near the lighthouse and a drive-in shopping plaza; heritage McCrae homestead (1844) and Eastern Lighthouse [Victorian Places]; R 6, Q 4 consistent. Holiday-house area: 43.3% of dwellings unoccupied on 2011 census night [Victorian Places]. Train: none; S 2 consistent. Indian community: India-born 0.0%, Hinduism 0.0% [ABS 2021 GCP SAL21625]; P 1 consistent. Older: median age 55, 34.6% aged 65+ [ABS]. City trip: 59 km, no rail; V 2 consistent. NOT checked: GPs, supermarket, bus. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB62" s="22" t="inlineStr">
@@ -15288,6 +18016,51 @@
           <t>AVM house value ($958,743) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK62" s="22" t="inlineStr">
+        <is>
+          <t>SAL21625</t>
+        </is>
+      </c>
+      <c r="AL62" s="32" t="n">
+        <v>3311</v>
+      </c>
+      <c r="AM62" s="22" t="n">
+        <v>55</v>
+      </c>
+      <c r="AN62" s="33" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="AO62" s="33" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="AP62" s="33" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AQ62" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR62" s="33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AS62" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT62" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU62" s="33" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AV62" s="22" t="inlineStr">
+        <is>
+          <t>Greek 1.1%; Italian 0.8%; Croatian 0.5%</t>
+        </is>
+      </c>
+      <c r="AW62" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="15">
       <c r="A63" s="16" t="inlineStr">
@@ -15390,7 +18163,7 @@
       </c>
       <c r="Z63" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Peninsula University Hospital 22 min. Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Peninsula University Hospital 22 min. Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 19,846; 6 km S of Mornington, 52 km S of Melbourne [Victorian Places Mount Martha]. Beach: bathing beach on Port Phillip [Wikipedia Mount Martha]; U 9 consistent. Nature: boardwalk along Balcombe Creek from the North Beach mouth to The Briars Historic Park [Wikipedia]; summit park (161 m) reserved 1929, with an ornamental conifer plantation [Victorian Places]; N 8 consistent (coast and creek, plantings partly exotic). Village: Mount Martha shopping centre; heritage holiday houses on the Esplanade [Victorian Places]; R 7 plausible. Train: no station named; S 2 consistent. Indian community: India-born 0.1%, Hinduism 0.1% [ABS 2021 GCP SAL21803]; P 2 generous (1 arguable). City trip: 52 km, no rail; V 2 consistent. NOT checked: GPs, supermarket, bus. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB63" s="22" t="inlineStr">
@@ -15436,6 +18209,51 @@
           <t>AVM house value ($1,344,095) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK63" s="22" t="inlineStr">
+        <is>
+          <t>SAL21803</t>
+        </is>
+      </c>
+      <c r="AL63" s="32" t="n">
+        <v>19846</v>
+      </c>
+      <c r="AM63" s="22" t="n">
+        <v>46</v>
+      </c>
+      <c r="AN63" s="33" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="AO63" s="33" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="AP63" s="33" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="AQ63" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AR63" s="33" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AS63" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AT63" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU63" s="33" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AV63" s="22" t="inlineStr">
+        <is>
+          <t>Italian 0.8%; German 0.6%; Greek 0.6%</t>
+        </is>
+      </c>
+      <c r="AW63" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="15">
       <c r="A64" s="16" t="inlineStr">
@@ -15538,7 +18356,7 @@
       </c>
       <c r="Z64" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Alfred Health: Sandringham ED 24 hrs, 7 days. Monash Medical Centre Clayton 18 min. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station on Frankston line; beach and pier (Wikipedia Mordialloc). GP: McDonald Street Medical Centre (healthdirect). Woolworths Mordialloc (grocerize). N, P, R, V remain estimates.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Alfred Health: Sandringham ED 24 hrs, 7 days. Monash Medical Centre Clayton 18 min. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station on Frankston line; beach and pier (Wikipedia Mordialloc). GP: McDonald Street Medical Centre (healthdirect). Woolworths Mordialloc (grocerize). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: tidal Mordialloc Creek mouth, beach with lifesaving and picnic facilities, numerous walking and cycling trails [Wikipedia Mordialloc; Victorian Places]; N 5 consistent. Village: shops within walking distance of the beach and station; pier and sailing club at the creek mouth [Victorian Places]; R 7 consistent. Indian community: India-born 1.4%, Indian ancestry 2.2%, Hinduism 1.4% [ABS 2021 GCP SAL21760]; P 5 generous (3 arguable). City trip: 24-25 km SE on the Frankston line [Wikipedia; Victorian Places]; V 7 plausible. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB64" s="22" t="inlineStr">
@@ -15584,6 +18402,51 @@
           <t>AVM house value ($1,401,241) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK64" s="22" t="inlineStr">
+        <is>
+          <t>SAL21760</t>
+        </is>
+      </c>
+      <c r="AL64" s="32" t="n">
+        <v>8886</v>
+      </c>
+      <c r="AM64" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AN64" s="33" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="AO64" s="33" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="AP64" s="33" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="AQ64" s="33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AR64" s="33" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AS64" s="33" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AT64" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU64" s="33" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="AV64" s="22" t="inlineStr">
+        <is>
+          <t>Greek 2.9%; Mandarin 2.3%; Italian 1.5%</t>
+        </is>
+      </c>
+      <c r="AW64" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="15">
       <c r="A65" s="16" t="inlineStr">
@@ -15686,7 +18549,7 @@
       </c>
       <c r="Z65" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Matches Williamstown row; Williamstown Hospital not checked. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two lines. No beach in suburb: The Strand foreshore and Altona Beach nearby; Newport Lakes 33 ha bushland (Wikipedia Newport). GP: Complete Family Care (healthdirect). Supermarket NOT confirmed; Q lowered 8-&gt;7. N, P, R, V remain estimates.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Matches Williamstown row; Williamstown Hospital not checked. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two lines. No beach in suburb: The Strand foreshore and Altona Beach nearby; Newport Lakes 33 ha bushland (Wikipedia Newport). GP: Complete Family Care (healthdirect). Supermarket NOT confirmed; Q lowered 8-&gt;7. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Newport Lakes Park, 33 ha 'bushland oasis' on a former quarry, 200+ plant and 85 bird species; Sandy Point Conservation Area; Greenwich Bay and The Strand [Wikipedia Newport]; N 4 low (5-6 arguable). Village: diverse mix; Substation arts centre beside the station; monthly artists' market; folk festival [Wikipedia]; residential and industrial suburb [Victorian Places]; R 6 consistent. Indian community: India-born 1.1%, Indian ancestry 1.8%, Hinduism 0.9% [ABS 2021 GCP SAL21934]; P 6 not supported (2-3 arguable). City trip: 7.5 km SW; 'a 20-minute train journey from Flinders Street' [Wikipedia]; V 9 consistent. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB65" s="22" t="inlineStr">
@@ -15732,6 +18595,51 @@
           <t>AVM house value ($1,150,951) is under $1.5M cap. Not a sale median.</t>
         </is>
       </c>
+      <c r="AK65" s="22" t="inlineStr">
+        <is>
+          <t>SAL21934</t>
+        </is>
+      </c>
+      <c r="AL65" s="32" t="n">
+        <v>13658</v>
+      </c>
+      <c r="AM65" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="AN65" s="33" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="AO65" s="33" t="n">
+        <v>0.232</v>
+      </c>
+      <c r="AP65" s="33" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AQ65" s="33" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AR65" s="33" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AS65" s="33" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="AT65" s="33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AU65" s="33" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="AV65" s="22" t="inlineStr">
+        <is>
+          <t>Arabic 2.4%; Greek 2.4%; Italian 1.5%</t>
+        </is>
+      </c>
+      <c r="AW65" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="15">
       <c r="A66" s="16" t="inlineStr">
@@ -15834,7 +18742,7 @@
       </c>
       <c r="Z66" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Peninsula University Hospital 30 min. Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price from 5 sales only (weak).</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Peninsula University Hospital 30 min. Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price from 5 sales only (weak). | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 414; small hill locality, 60 km S of CBD [Victorian Places] (Wikipedia's 85 km looks wrong); summit 304-314 m. Nature: Arthurs Seat State Park covers the western half with many walking tracks (Two Bays track, Kings Falls circuit); dry open eucalypt forest, burnt in 1973 and 1997; weeds on the NW face [Wikipedia; Victorian Places]; N 9 consistent. Village: no centre; residential area east of the summit 'shading into open country towards Main Ridge'; tourist attractions (Seawinds gardens, maze, restaurants) [Victorian Places; Wikipedia]; R 6 generous for a locality with no shops (4 arguable). Shops: none named; Q 2 consistent. Beach: Dromana and McCrae beaches below; U 6 plausible. Train: none; S 1 consistent. Indian community: 0 India-born, 0 Indian ancestry [ABS 2021 GCP SAL20072]; P 1 consistent. Very small population: ABS perturbs small counts. City trip: no rail; V 2 consistent. NOT checked: road access for older drivers, bushfire overlay. Scores unchanged.</t>
         </is>
       </c>
       <c r="AB66" s="22" t="inlineStr">
@@ -15878,6 +18786,51 @@
       <c r="AJ66" s="22" t="inlineStr">
         <is>
           <t>Sale median ($1,430,000) is under $1.5M cap, but based on only 5 sales. Treat as unreliable.</t>
+        </is>
+      </c>
+      <c r="AK66" s="22" t="inlineStr">
+        <is>
+          <t>SAL20072</t>
+        </is>
+      </c>
+      <c r="AL66" s="32" t="n">
+        <v>414</v>
+      </c>
+      <c r="AM66" s="22" t="n">
+        <v>48</v>
+      </c>
+      <c r="AN66" s="33" t="n">
+        <v>0.239</v>
+      </c>
+      <c r="AO66" s="33" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AP66" s="33" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="AQ66" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR66" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS66" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT66" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU66" s="33" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="AV66" s="22" t="inlineStr">
+        <is>
+          <t>Greek 2.2%; Italian 0.7%</t>
+        </is>
+      </c>
+      <c r="AW66" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
C3: re-score 13 nature/village/city-trip scores; P unchanged
- SuburbScorecard N/R/V: 13 changes, each sourced in col Z
  (Seaford, Newport, Frankston, Rosanna, Torquay, Mornington,
  Yarra Glen, Macedon, Arthurs Seat, Frankston South, Upwey, Gisborne).
- P unchanged pending a family decision; B4 now measures nearest
  Indian grocery, Hindu temple and church.
- AK-AW header comments moved one column left onto the right headers.
- Pointer: change log with top 15 and AQ/AU; Chrome prompt Task 7 and
  open-work list updated. Pre-change workbook archived.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013uWqdtxBL1QFjMDN6afhAy
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -442,22 +442,22 @@
         <t>27 Oct 2026: columns A–H and Z were Google-only formulas splitting column AA. Converted to plain values so they can be edited in Excel. Blank price (G) = not yet researched (was shown as 0).</t>
       </text>
     </comment>
-    <comment ref="AP1" authorId="1" shapeId="0">
+    <comment ref="AO1" authorId="1" shapeId="0">
       <text>
         <t>Born overseas / all people (ABS G01 Birthplace_Elsewhere_P / Tot_P). Not the same as 100 minus Australia-born: that also counts people who did not state a birthplace (see next column). This fixes foundation-report item 11.</t>
       </text>
     </comment>
-    <comment ref="AQ1" authorId="1" shapeId="0">
+    <comment ref="AP1" authorId="1" shapeId="0">
       <text>
         <t>All people minus Australia-born minus overseas-born, as a share of all people.</t>
       </text>
     </comment>
-    <comment ref="AS1" authorId="1" shapeId="0">
+    <comment ref="AR1" authorId="1" shapeId="0">
       <text>
         <t>Indian ancestry responses / all people (ABS G08). People can give two ancestries.</t>
       </text>
     </comment>
-    <comment ref="AW1" authorId="1" shapeId="0">
+    <comment ref="AV1" authorId="1" shapeId="0">
       <text>
         <t>From ABS GCP table G13 (about 45 named languages). Languages ABS groups as "other" there (e.g. Telugu, Burmese, Zomi) cannot appear; QuickStats top-responses may differ.</t>
       </text>
@@ -8193,7 +8193,7 @@
         <v/>
       </c>
       <c r="N11" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O11" s="19">
         <f>IF(K11="","",ROUND(MAX(0,10*(1-K11/Filters!$B$5)),1))</f>
@@ -8235,7 +8235,7 @@
       </c>
       <c r="Z11" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 22.5% overseas-born, 15.2% non-Eng HH. Peninsula Univ Hospital ED; ~66m train to CBD. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Rail terminus + bus hub to Mornington, Rosebud etc. (Wikipedia). GP: myhealth Bayside (healthdirect). Beach U and supermarket not individually checked. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: 'generally a leafy suburb'; natural reserves Bunarong Park, Frankston Foreshore Reserve, Lower Sweetwater Creek Reserve, Paratea Reserve; over 20 indigenous orchid species; McClelland Sculpture Park in 16 ha of park and reserve [Wikipedia Frankston]; N 5 consistent (6 arguable). Village: regional centre with Bayside (250+ stores) and Karingal Hub; several vacant highway buildings noted [Wikipedia; Victorian Places]; R 3 consistent. Health hub: four hospitals in the suburb [Wikipedia]. Indian community: India-born 1.1%, Hinduism 0.8%; Malayalam 0.5% at home [ABS 2021 GCP SAL20947; Wikipedia]; P 4 generous (2 arguable). City trip: 39-40 km SE, line terminus [Wikipedia; Victorian Places]; V 6 plausible. Scores unchanged.</t>
+          <t>ABS 2021: 22.5% overseas-born, 15.2% non-Eng HH. Peninsula Univ Hospital ED; ~66m train to CBD. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Rail terminus + bus hub to Mornington, Rosebud etc. (Wikipedia). GP: myhealth Bayside (healthdirect). Beach U and supermarket not individually checked. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: 'generally a leafy suburb'; natural reserves Bunarong Park, Frankston Foreshore Reserve, Lower Sweetwater Creek Reserve, Paratea Reserve; over 20 indigenous orchid species; McClelland Sculpture Park in 16 ha of park and reserve [Wikipedia Frankston]; N 5 consistent (6 arguable). Village: regional centre with Bayside (250+ stores) and Karingal Hub; several vacant highway buildings noted [Wikipedia; Victorian Places]; R 3 consistent. Health hub: four hospitals in the suburb [Wikipedia]. Indian community: India-born 1.1%, Hinduism 0.8%; Malayalam 0.5% at home [ABS 2021 GCP SAL20947; Wikipedia]; P 4 generous (2 arguable). City trip: 39-40 km SE, line terminus [Wikipedia; Victorian Places]; V 6 plausible. Scores unchanged. | C3 28 Oct 2026: N 5-&gt;6 (source: 'generally a leafy suburb'; Bunarong Park, Lower Sweetwater Creek and Paratea reserves [Wikipedia Frankston]).</t>
         </is>
       </c>
       <c r="AA11" s="16" t="inlineStr">
@@ -9357,7 +9357,7 @@
         <v/>
       </c>
       <c r="N17" s="19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O17" s="19">
         <f>IF(K17="","",ROUND(MAX(0,10*(1-K17/Filters!$B$5)),1))</f>
@@ -9399,7 +9399,7 @@
       </c>
       <c r="Z17" s="18" t="inlineStr">
         <is>
-          <t>Distinguish Macedon from Mount Macedon; check bushfire overlay, gradients &amp; major ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 2,073; foot of Mount Macedon, 58 km NW of Melbourne, on the Melbourne-Bendigo railway [Wikipedia Macedon; Victorian Places]. Nature: bushland foothills of the Mount Macedon range; vineyards nearby [Wikipedia]; N 10 plausible (9 arguable: town is at the foot, not on the mount). Village: rebuilt shops, churches and hall after the 1983 Ash Wednesday fire (499 houses, 8 lives lost in Macedon and Mount Macedon) [Victorian Places]; cafés and B&amp;Bs, new planning controls 'to protect the character' [Wikipedia]; R 8 consistent. Bushfire risk is real and documented. Shops: small; supermarket not named; Q 3 consistent. Train: station on the Bendigo line [Victorian Places]; S 5 consistent (frequency not checked). Indian community: India-born 0.2%, Hinduism 0.2% [ABS 2021 GCP SAL21562]; P 1 consistent. City trip: 58 km by V/Line; V 5 estimate. NOT checked: GPs, nearest ED, journey time. Scores unchanged.</t>
+          <t>Distinguish Macedon from Mount Macedon; check bushfire overlay, gradients &amp; major ED journey. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Low sales count. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 2,073; foot of Mount Macedon, 58 km NW of Melbourne, on the Melbourne-Bendigo railway [Wikipedia Macedon; Victorian Places]. Nature: bushland foothills of the Mount Macedon range; vineyards nearby [Wikipedia]; N 10 plausible (9 arguable: town is at the foot, not on the mount). Village: rebuilt shops, churches and hall after the 1983 Ash Wednesday fire (499 houses, 8 lives lost in Macedon and Mount Macedon) [Victorian Places]; cafés and B&amp;Bs, new planning controls 'to protect the character' [Wikipedia]; R 8 consistent. Bushfire risk is real and documented. Shops: small; supermarket not named; Q 3 consistent. Train: station on the Bendigo line [Victorian Places]; S 5 consistent (frequency not checked). Indian community: India-born 0.2%, Hinduism 0.2% [ABS 2021 GCP SAL21562]; P 1 consistent. City trip: 58 km by V/Line; V 5 estimate. NOT checked: GPs, nearest ED, journey time. Scores unchanged. | C3 28 Oct 2026: N 10-&gt;9 (source: town sits at the foot of Mount Macedon; surrounding bushland long harvested for timber [Wikipedia Macedon]; 10 kept for national-park settings).</t>
         </is>
       </c>
       <c r="AA17" s="16" t="inlineStr">
@@ -9554,7 +9554,7 @@
         <v/>
       </c>
       <c r="N18" s="19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O18" s="19">
         <f>IF(K18="","",ROUND(MAX(0,10*(1-K18/Filters!$B$5)),1))</f>
@@ -9567,7 +9567,7 @@
         <v>8</v>
       </c>
       <c r="R18" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S18" s="19" t="n">
         <v>4</v>
@@ -9596,7 +9596,7 @@
       </c>
       <c r="Z18" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 16.4% aged 65+, 7.4% non-Eng HH. Bus 54 to Marshall Station; relies on Univ Hospital Geelong for major public ED. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. GW drive 88 min, 2 min under cap. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Buses to Geelong/Marshall: S raised 3-&gt;4 (Bus News). GPs: Surfcoast Medical Centre, Orbit Medical, Banksia (healthdirect). Beach and supermarket not individually checked. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: surf beaches (Jan Juc, Bells Beach on the SW outskirts), Point Danger, Zeally Bay, Spring Creek on the western boundary [Wikipedia Torquay]; N 8 rests on coast, not bush (7 arguable). Village: population doubled 1991-2011 and 'some of its former holiday charm has been lost to redevelopment' [Victorian Places]; population triples in Jan-Feb; Surf Coast Plaza [Wikipedia]; R 6 generous (5 arguable). Indian community: India-born 0.2%, Hinduism 0.1% [ABS 2021 GCP SAL22551]; P 2 generous (1 arguable). City trip: 80 km W of Melbourne, 21 km S of Geelong [Victorian Places], no rail; V 3 plausible; journey time not checked. Scores unchanged.</t>
+          <t>ABS 2021: 16.4% aged 65+, 7.4% non-Eng HH. Bus 54 to Marshall Station; relies on Univ Hospital Geelong for major public ED. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. GW drive 88 min, 2 min under cap. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Buses to Geelong/Marshall: S raised 3-&gt;4 (Bus News). GPs: Surfcoast Medical Centre, Orbit Medical, Banksia (healthdirect). Beach and supermarket not individually checked. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: surf beaches (Jan Juc, Bells Beach on the SW outskirts), Point Danger, Zeally Bay, Spring Creek on the western boundary [Wikipedia Torquay]; N 8 rests on coast, not bush (7 arguable). Village: population doubled 1991-2011 and 'some of its former holiday charm has been lost to redevelopment' [Victorian Places]; population triples in Jan-Feb; Surf Coast Plaza [Wikipedia]; R 6 generous (5 arguable). Indian community: India-born 0.2%, Hinduism 0.1% [ABS 2021 GCP SAL22551]; P 2 generous (1 arguable). City trip: 80 km W of Melbourne, 21 km S of Geelong [Victorian Places], no rail; V 3 plausible; journey time not checked. Scores unchanged. | C3 28 Oct 2026: N 8-&gt;7 (source: nature is coastal and already scored under U (10); no bushland named [Wikipedia Torquay]). | C3 28 Oct 2026: R 6-&gt;5 (source: 'some of its former holiday charm has been lost to redevelopment' [Victorian Places Torquay]).</t>
         </is>
       </c>
       <c r="AA18" s="16" t="inlineStr">
@@ -10535,7 +10535,7 @@
         <v>5</v>
       </c>
       <c r="R23" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S23" s="19" t="n">
         <v>8</v>
@@ -10564,7 +10564,7 @@
       </c>
       <c r="Z23" s="18" t="inlineStr">
         <is>
-          <t>Belgrave rail line township; closer to foothills edge than Belgrave. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station beside Main St; medical centre on Main St; no supermarket mentioned: Q lowered 6-&gt;5. Adjoins Dandenong Ranges NP; Ferny, Monbulk creeks (Wikipedia Upwey). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Glenfern Valley Bushlands, 40 ha of remnant and rehabilitated forest down to Ferny Creek; ridge-top Glenfern Rd with views [Wikipedia Upwey]; N 9 consistent. Village: Main Street 'instilling a traditional community village nature', cafés with kerbside dining, medical and dental centre [Wikipedia]; R 7 consistent (8 arguable); medical centre on Main St supports Q. Indian community: India-born 0.6%, Hinduism 0.3%; 80.7% Australia-born [ABS 2021 GCP SAL22620; Wikipedia]; P 3 generous (1 arguable). City trip: 33 km E on the Belgrave line [Wikipedia]; V 5 estimate. Scores unchanged.</t>
+          <t>Belgrave rail line township; closer to foothills edge than Belgrave. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Station beside Main St; medical centre on Main St; no supermarket mentioned: Q lowered 6-&gt;5. Adjoins Dandenong Ranges NP; Ferny, Monbulk creeks (Wikipedia Upwey). N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Glenfern Valley Bushlands, 40 ha of remnant and rehabilitated forest down to Ferny Creek; ridge-top Glenfern Rd with views [Wikipedia Upwey]; N 9 consistent. Village: Main Street 'instilling a traditional community village nature', cafés with kerbside dining, medical and dental centre [Wikipedia]; R 7 consistent (8 arguable); medical centre on Main St supports Q. Indian community: India-born 0.6%, Hinduism 0.3%; 80.7% Australia-born [ABS 2021 GCP SAL22620; Wikipedia]; P 3 generous (1 arguable). City trip: 33 km E on the Belgrave line [Wikipedia]; V 5 estimate. Scores unchanged. | C3 28 Oct 2026: R 7-&gt;8 (source: Main Street 'instilling a traditional community village nature', kerbside cafés [Wikipedia Upwey]).</t>
         </is>
       </c>
       <c r="AA23" s="16" t="inlineStr">
@@ -12085,7 +12085,7 @@
         <v/>
       </c>
       <c r="N31" s="19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O31" s="19">
         <f>IF(K31="","",ROUND(MAX(0,10*(1-K31/Filters!$B$5)),1))</f>
@@ -12127,7 +12127,7 @@
       </c>
       <c r="Z31" s="18" t="inlineStr">
         <is>
-          <t>Substantial town services on bay; no passenger train (bus to Frankston); verify Frankston/Rosebud ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): No rail; bus to Frankston. Mothers Beach, Mills Beach patrolled (Visit Mornington Peninsula). GPs: Mornington Village Medical Centre, Mornington Medical Group (healthdirect). Supermarket not confirmed; Q partly estimate. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Indian community: India-born, Indian ancestry, Hinduism/Sikhism and Hindi/Punjabi are all absent from the ABS 2021 top responses (pop 25,759; 74.0% Australia-born) [ABS QuickStats SAL21763]; web search found no Indian grocer or temple (no result is not proof). Nature: sources name parks and gardens only (Botanical Rose Gardens, Alexandra Park, Dallas Brooks Park, Narambi Reserve), no bushland, creeks or trails [Wikipedia Mornington; Visit Mornington Peninsula], so N 7 is NOT supported by what was found; left at 7, consider 6. Village: 'cosmopolitan seaside village', 1 km+ of shopping, 370+ retail outlets, Wednesday main-street market [Visit Mornington Peninsula]; R 7 consistent. City trip: 46 km SE of CBD, 13 km to Frankston, no rail (heritage line only), buses 781/784/785/788 to Frankston [Wikipedia]; V 3 consistent. NOT checked: supermarket names, drive time to CBD. Scores unchanged.</t>
+          <t>Substantial town services on bay; no passenger train (bus to Frankston); verify Frankston/Rosebud ED drive. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): No rail; bus to Frankston. Mothers Beach, Mills Beach patrolled (Visit Mornington Peninsula). GPs: Mornington Village Medical Centre, Mornington Medical Group (healthdirect). Supermarket not confirmed; Q partly estimate. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Indian community: India-born, Indian ancestry, Hinduism/Sikhism and Hindi/Punjabi are all absent from the ABS 2021 top responses (pop 25,759; 74.0% Australia-born) [ABS QuickStats SAL21763]; web search found no Indian grocer or temple (no result is not proof). Nature: sources name parks and gardens only (Botanical Rose Gardens, Alexandra Park, Dallas Brooks Park, Narambi Reserve), no bushland, creeks or trails [Wikipedia Mornington; Visit Mornington Peninsula], so N 7 is NOT supported by what was found; left at 7, consider 6. Village: 'cosmopolitan seaside village', 1 km+ of shopping, 370+ retail outlets, Wednesday main-street market [Visit Mornington Peninsula]; R 7 consistent. City trip: 46 km SE of CBD, 13 km to Frankston, no rail (heritage line only), buses 781/784/785/788 to Frankston [Wikipedia]; V 3 consistent. NOT checked: supermarket names, drive time to CBD. Scores unchanged. | C3 28 Oct 2026: N 7-&gt;6 (source: earlier source run found parks and gardens only, no bushland named (flagged 'consider 6')).</t>
         </is>
       </c>
       <c r="AA31" s="16" t="inlineStr">
@@ -14035,7 +14035,7 @@
         <v>5</v>
       </c>
       <c r="R41" s="19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S41" s="19" t="n">
         <v>4</v>
@@ -14064,7 +14064,7 @@
       </c>
       <c r="Z41" s="18" t="inlineStr">
         <is>
-          <t>Sweetwater Creek nature reserve; weaker station walk than central Frankston. Promoted to Active 26 Oct 2026 as a bush-plus-bay overlap candidate. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): No station; buses to Frankston. Olivers Hill bay views; Daveys Bay is in Mt Eliza, so beach access not in suburb: U lowered 7-&gt;6. No major shops, small strips only: Q lowered 6-&gt;5 (Wikipedia). GP: Baxter Park Medical Centre (healthdirect). Sweetwater Creek reserve. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: elevated land where Sweetwater Creek descends from Mount Eliza; Frankston Reservoir; much stayed open country until postwar [Victorian Places Frankston South]; N 7 plausible. Village: 'no major shopping areas'; small strips on Norman Ave, Foot St and Overport Rd; south served by Mount Eliza village [Wikipedia Frankston South]; R 6 generous (5 arguable). Indian community: India-born 0.9%, Hinduism 0.4%; Malayalam 0.8% at home [ABS 2021 GCP SAL20949]; P 3 consistent (2 arguable). Older: median age 44, 22.0% aged 65+ [ABS]. City trip: 41-43 km SE, no station [Wikipedia; Victorian Places]; V 5 estimate. Scores unchanged.</t>
+          <t>Sweetwater Creek nature reserve; weaker station walk than central Frankston. Promoted to Active 26 Oct 2026 as a bush-plus-bay overlap candidate. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): No station; buses to Frankston. Olivers Hill bay views; Daveys Bay is in Mt Eliza, so beach access not in suburb: U lowered 7-&gt;6. No major shops, small strips only: Q lowered 6-&gt;5 (Wikipedia). GP: Baxter Park Medical Centre (healthdirect). Sweetwater Creek reserve. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: elevated land where Sweetwater Creek descends from Mount Eliza; Frankston Reservoir; much stayed open country until postwar [Victorian Places Frankston South]; N 7 plausible. Village: 'no major shopping areas'; small strips on Norman Ave, Foot St and Overport Rd; south served by Mount Eliza village [Wikipedia Frankston South]; R 6 generous (5 arguable). Indian community: India-born 0.9%, Hinduism 0.4%; Malayalam 0.8% at home [ABS 2021 GCP SAL20949]; P 3 consistent (2 arguable). Older: median age 44, 22.0% aged 65+ [ABS]. City trip: 41-43 km SE, no station [Wikipedia; Victorian Places]; V 5 estimate. Scores unchanged. | C3 28 Oct 2026: R 6-&gt;5 (source: 'no major shopping areas', only small strips [Wikipedia Frankston South]).</t>
         </is>
       </c>
       <c r="AA41" s="16" t="inlineStr">
@@ -15600,7 +15600,7 @@
           <t>Synthetic test calibration model.</t>
         </is>
       </c>
-      <c r="AW49" t="inlineStr">
+      <c r="AW49" s="22" t="inlineStr">
         <is>
           <t>Excluded test row: no demography.</t>
         </is>
@@ -15739,7 +15739,7 @@
           <t>Synthetic test calibration model.</t>
         </is>
       </c>
-      <c r="AW50" t="inlineStr">
+      <c r="AW50" s="22" t="inlineStr">
         <is>
           <t>Excluded test row: no demography.</t>
         </is>
@@ -16226,7 +16226,7 @@
         <v>0</v>
       </c>
       <c r="V53" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W53" s="16">
         <f>IF(M53="",0,COUNT(M53:V53))</f>
@@ -16242,7 +16242,7 @@
       </c>
       <c r="Z53" s="16" t="inlineStr">
         <is>
-          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify train access (nearest V/Line may be Riddells Creek), GW drive, price and nearest major public ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Gisborne district pop 14,432 (June 2021) [Wikipedia Gisborne]; SAL pop 10,142 [ABS 2021 GCP SAL21001]; ~54 km NW of Melbourne. Train: station on the Bendigo line, built outside the township (the suburb New Gisborne); V/Line runs to Southern Cross; 'a 50-minute train ride'; 20 min to Sunbury for Metro; Gisborne Transit loop and on-demand bus to the station [Wikipedia]; resolves foundation-report item 14 (station exists, ~3 km out); S 4 low (5 arguable). Shops: town centre with cafés, theatre, galleries, monthly farmers' market and four supermarkets [Wikipedia]; Q 7 consistent (8 arguable). Village: 'country homesteads, tree-lined streets'; planning controls protect the town's character; fast growth [Wikipedia]; R 7 consistent. Nature: 'large leafy blocks' [Wikipedia]; N 7 consistent. Indian community: India-born 0.6%, Hinduism 0.3%, Sikhism 0.4% [ABS]; P 2 consistent. City trip: 45 min drive or 50 min train [Wikipedia]; V 5 consistent (6 arguable). NOT checked: GPs, train frequency. Scores unchanged.</t>
+          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Verify train access (nearest V/Line may be Riddells Creek), GW drive, price and nearest major public ED. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Gisborne district pop 14,432 (June 2021) [Wikipedia Gisborne]; SAL pop 10,142 [ABS 2021 GCP SAL21001]; ~54 km NW of Melbourne. Train: station on the Bendigo line, built outside the township (the suburb New Gisborne); V/Line runs to Southern Cross; 'a 50-minute train ride'; 20 min to Sunbury for Metro; Gisborne Transit loop and on-demand bus to the station [Wikipedia]; resolves foundation-report item 14 (station exists, ~3 km out); S 4 low (5 arguable). Shops: town centre with cafés, theatre, galleries, monthly farmers' market and four supermarkets [Wikipedia]; Q 7 consistent (8 arguable). Village: 'country homesteads, tree-lined streets'; planning controls protect the town's character; fast growth [Wikipedia]; R 7 consistent. Nature: 'large leafy blocks' [Wikipedia]; N 7 consistent. Indian community: India-born 0.6%, Hinduism 0.3%, Sikhism 0.4% [ABS]; P 2 consistent. City trip: 45 min drive or 50 min train [Wikipedia]; V 5 consistent (6 arguable). NOT checked: GPs, train frequency. Scores unchanged. | C3 28 Oct 2026: V 5-&gt;6 (source: 'a 45-minute drive along the Calder Freeway or a 50-minute train ride' to the city [Wikipedia Gisborne]).</t>
         </is>
       </c>
       <c r="AA53" s="16" t="inlineStr">
@@ -16596,7 +16596,7 @@
         <v/>
       </c>
       <c r="N55" s="22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O55" s="16">
         <f>IF(K55="","",ROUND(MAX(0,10*(1-K55/Filters!$B$5)),1))</f>
@@ -16638,7 +16638,7 @@
       </c>
       <c r="Z55" s="16" t="inlineStr">
         <is>
-          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Likely no train; verify GW drive, price and ED journey (Maroondah/Angliss). Compare with Healesville. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 3,012; 55 km NE of CBD [Wikipedia Yarra Glen] (40 km per Victorian Places), just north of the Yarra River flood plain. Nature: open valley farmland and vineyards; heritage Gulf Station farm; Black Saturday 2009 fire killed at least 13 in the Yarra Glen-Steeles Creek area [Victorian Places]; N 8 plausible (open valley more than forest; 7 arguable). Village: 'substantial shopping centre', historic main street with the Grand Hotel (1888), racecourse, showground [Victorian Places]; R 7 consistent; Q 5 plausible (supermarket not named). Train: line closed 1980; tourist railway later disused [Victorian Places]; S 1 consistent. Indian community: India-born 0.1%, Hinduism 0.0% [ABS 2021 GCP SAL22910]; P 1 consistent. City trip: 40-55 km, no rail; V 2 consistent. NOT checked: GPs, bus, flood overlay. Scores unchanged.</t>
+          <t>Regional add (within about 1.5 hrs of Melbourne, from recall; verify). Likely no train; verify GW drive, price and ED journey (Maroondah/Angliss). Compare with Healesville. 27 Oct 2026 research pass: drive times/ED and/or AVM price added; L re-evaluated. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 3,012; 55 km NE of CBD [Wikipedia Yarra Glen] (40 km per Victorian Places), just north of the Yarra River flood plain. Nature: open valley farmland and vineyards; heritage Gulf Station farm; Black Saturday 2009 fire killed at least 13 in the Yarra Glen-Steeles Creek area [Victorian Places]; N 8 plausible (open valley more than forest; 7 arguable). Village: 'substantial shopping centre', historic main street with the Grand Hotel (1888), racecourse, showground [Victorian Places]; R 7 consistent; Q 5 plausible (supermarket not named). Train: line closed 1980; tourist railway later disused [Victorian Places]; S 1 consistent. Indian community: India-born 0.1%, Hinduism 0.0% [ABS 2021 GCP SAL22910]; P 1 consistent. City trip: 40-55 km, no rail; V 2 consistent. NOT checked: GPs, bus, flood overlay. Scores unchanged. | C3 28 Oct 2026: N 8-&gt;7 (source: open Yarra flood-plain farmland rather than forest [Victorian Places Yarra Glen]).</t>
         </is>
       </c>
       <c r="AA55" s="16" t="inlineStr">
@@ -17185,7 +17185,7 @@
         <v/>
       </c>
       <c r="N58" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O58" s="22">
         <f>IF(K58="","",ROUND(MAX(0,10*(1-K58/Filters!$B$5)),1))</f>
@@ -17227,7 +17227,7 @@
       </c>
       <c r="Z58" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 8,616; 12 km NE of CBD, ~2 km beyond Heidelberg, on the fringe of the Yarra Valley green belt [Wikipedia Rosanna; Victorian Places]. Nature: 'generous tree cover across hilly streets' (The Age 2019, via Wikipedia); Salt Creek open space on the former golf links, Banyule Creek linear park, Warringal parklands and Banyule Flats by the Yarra [Victorian Places]; N 6 consistent (7 arguable). Village: 'active shopping centre near the railway station'; Woolworths beside the library redevelopment [Victorian Places; Wikipedia]; R 6, Q 7 consistent. Train: recently updated station, Hurstbridge line [Wikipedia; Victorian Places]; S 8 consistent. Indian community: India-born 2.8%, Indian ancestry 3.8%, Hinduism 2.4% [ABS 2021 GCP SAL22194]; P 4 consistent. City trip: 12 km by train; V 8 consistent. NOT checked: GPs, journey time. Scores unchanged.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 8,616; 12 km NE of CBD, ~2 km beyond Heidelberg, on the fringe of the Yarra Valley green belt [Wikipedia Rosanna; Victorian Places]. Nature: 'generous tree cover across hilly streets' (The Age 2019, via Wikipedia); Salt Creek open space on the former golf links, Banyule Creek linear park, Warringal parklands and Banyule Flats by the Yarra [Victorian Places]; N 6 consistent (7 arguable). Village: 'active shopping centre near the railway station'; Woolworths beside the library redevelopment [Victorian Places; Wikipedia]; R 6, Q 7 consistent. Train: recently updated station, Hurstbridge line [Wikipedia; Victorian Places]; S 8 consistent. Indian community: India-born 2.8%, Indian ancestry 3.8%, Hinduism 2.4% [ABS 2021 GCP SAL22194]; P 4 consistent. City trip: 12 km by train; V 8 consistent. NOT checked: GPs, journey time. Scores unchanged. | C3 28 Oct 2026: N 6-&gt;7 (source: 'generous tree cover across hilly streets' (The Age 2019, via Wikipedia Rosanna); Banyule Flats Reserve and Warringal parklands [Victorian Places]).</t>
         </is>
       </c>
       <c r="AB58" s="22" t="inlineStr">
@@ -17378,7 +17378,7 @@
         <v/>
       </c>
       <c r="N59" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O59" s="22">
         <f>IF(K59="","",ROUND(MAX(0,10*(1-K59/Filters!$B$5)),1))</f>
@@ -17420,7 +17420,7 @@
       </c>
       <c r="Z59" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two stations; beachside with foreshore reserve and 305 ha wetlands (Wikipedia Seaford). GPs: Seaford Central Medical Clinic, Seaford Beach Family Clinic (healthdirect). Supermarket in suburb NOT confirmed; Q partly estimate. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Seaford Foreshore Reserve is 'one of the few remaining substantial, continuous strands of natural coastal vegetation near Melbourne' along the whole suburb; Kananook walking trail [Wikipedia Seaford]; Edithvale-Seaford Wetland with walking trail and viewing platform; Kananook Creek linear reserve [Victorian Places]; N 5 looks low (6 arguable). Village: small shopping centre and pier near the station, a supermarket; largely cheap postwar housing [Victorian Places]; R 4 consistent. Indian community: India-born 0.6%, Hinduism 0.7% [ABS 2021 GCP SAL22249]; P 4 generous (2 arguable). City trip: 36 km SE on the Frankston line [Wikipedia]; journey time not stated; V 6 estimate. Scores unchanged.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two stations; beachside with foreshore reserve and 305 ha wetlands (Wikipedia Seaford). GPs: Seaford Central Medical Clinic, Seaford Beach Family Clinic (healthdirect). Supermarket in suburb NOT confirmed; Q partly estimate. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Seaford Foreshore Reserve is 'one of the few remaining substantial, continuous strands of natural coastal vegetation near Melbourne' along the whole suburb; Kananook walking trail [Wikipedia Seaford]; Edithvale-Seaford Wetland with walking trail and viewing platform; Kananook Creek linear reserve [Victorian Places]; N 5 looks low (6 arguable). Village: small shopping centre and pier near the station, a supermarket; largely cheap postwar housing [Victorian Places]; R 4 consistent. Indian community: India-born 0.6%, Hinduism 0.7% [ABS 2021 GCP SAL22249]; P 4 generous (2 arguable). City trip: 36 km SE on the Frankston line [Wikipedia]; journey time not stated; V 6 estimate. Scores unchanged. | C3 28 Oct 2026: N 5-&gt;6 (source: Seaford Foreshore Reserve, 'one of the few remaining substantial, continuous strands of natural coastal vegetation near Melbourne' [Wikipedia Seaford]; Edithvale-Seaford Wetland [Victorian Places]).</t>
         </is>
       </c>
       <c r="AB59" s="22" t="inlineStr">
@@ -18507,7 +18507,7 @@
         <v/>
       </c>
       <c r="N65" s="22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O65" s="22">
         <f>IF(K65="","",ROUND(MAX(0,10*(1-K65/Filters!$B$5)),1))</f>
@@ -18549,7 +18549,7 @@
       </c>
       <c r="Z65" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Matches Williamstown row; Williamstown Hospital not checked. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two lines. No beach in suburb: The Strand foreshore and Altona Beach nearby; Newport Lakes 33 ha bushland (Wikipedia Newport). GP: Complete Family Care (healthdirect). Supermarket NOT confirmed; Q lowered 8-&gt;7. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Newport Lakes Park, 33 ha 'bushland oasis' on a former quarry, 200+ plant and 85 bird species; Sandy Point Conservation Area; Greenwich Bay and The Strand [Wikipedia Newport]; N 4 low (5-6 arguable). Village: diverse mix; Substation arts centre beside the station; monthly artists' market; folk festival [Wikipedia]; residential and industrial suburb [Victorian Places]; R 6 consistent. Indian community: India-born 1.1%, Indian ancestry 1.8%, Hinduism 0.9% [ABS 2021 GCP SAL21934]; P 6 not supported (2-3 arguable). City trip: 7.5 km SW; 'a 20-minute train journey from Flinders Street' [Wikipedia]; V 9 consistent. Scores unchanged.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Matches Williamstown row; Williamstown Hospital not checked. | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. | CHECKED 27 Oct 2026 (S train/bus, U beach, Q shops &amp; doctor; web sources, suburb level, not address level): Two lines. No beach in suburb: The Strand foreshore and Altona Beach nearby; Newport Lakes 33 ha bushland (Wikipedia Newport). GP: Complete Family Care (healthdirect). Supermarket NOT confirmed; Q lowered 8-&gt;7. N, P, R, V remain estimates. | CHECKED 27 Oct 2026, second pass (N, P, R, V; suburb level). Nature: Newport Lakes Park, 33 ha 'bushland oasis' on a former quarry, 200+ plant and 85 bird species; Sandy Point Conservation Area; Greenwich Bay and The Strand [Wikipedia Newport]; N 4 low (5-6 arguable). Village: diverse mix; Substation arts centre beside the station; monthly artists' market; folk festival [Wikipedia]; residential and industrial suburb [Victorian Places]; R 6 consistent. Indian community: India-born 1.1%, Indian ancestry 1.8%, Hinduism 0.9% [ABS 2021 GCP SAL21934]; P 6 not supported (2-3 arguable). City trip: 7.5 km SW; 'a 20-minute train journey from Flinders Street' [Wikipedia]; V 9 consistent. Scores unchanged. | C3 28 Oct 2026: N 4-&gt;5 (source: Newport Lakes Park, 33 ha 'bushland oasis', 200+ plant species; Sandy Point Conservation Area [Wikipedia Newport]).</t>
         </is>
       </c>
       <c r="AB65" s="22" t="inlineStr">
@@ -18713,7 +18713,7 @@
         <v>2</v>
       </c>
       <c r="R66" s="22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S66" s="22" t="n">
         <v>1</v>
@@ -18742,7 +18742,7 @@
       </c>
       <c r="Z66" s="16" t="inlineStr">
         <is>
-          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Peninsula University Hospital 30 min. Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price from 5 sales only (weak). | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 414; small hill locality, 60 km S of CBD [Victorian Places] (Wikipedia's 85 km looks wrong); summit 304-314 m. Nature: Arthurs Seat State Park covers the western half with many walking tracks (Two Bays track, Kings Falls circuit); dry open eucalypt forest, burnt in 1973 and 1997; weeds on the NW face [Wikipedia; Victorian Places]; N 9 consistent. Village: no centre; residential area east of the summit 'shading into open country towards Main Ridge'; tourist attractions (Seawinds gardens, maze, restaurants) [Victorian Places; Wikipedia]; R 6 generous for a locality with no shops (4 arguable). Shops: none named; Q 2 consistent. Beach: Dromana and McCrae beaches below; U 6 plausible. Train: none; S 1 consistent. Indian community: 0 India-born, 0 Indian ancestry [ABS 2021 GCP SAL20072]; P 1 consistent. Very small population: ABS perturbs small counts. City trip: no rail; V 2 consistent. NOT checked: road access for older drivers, bushfire overlay. Scores unchanged.</t>
+          <t>Added 27 Oct 2026 from realestate.com.au collection "Parents." (Listings tab). Fit ratings (P/Y/lens) not yet assessed. ED: Peninsula University Hospital 30 min. Rosebud ED is 24/7 but treats less serious cases; serious cases transfer to Frankston (Peninsula Health). | SCORES 27 Oct 2026: M (near family) and T (price) are formulas from J and G; O from K. N, P, Q, R, S, U, V are ESTIMATES (Claude, general knowledge, not site-checked); S also rests on train Yes/No marked 'verify'. Price from 5 sales only (weak). | CHECKED 27 Oct 2026, source run C1 (suburb level; Wikipedia, Victorian Places, ABS 2021 GCP DataPack). Pop 414; small hill locality, 60 km S of CBD [Victorian Places] (Wikipedia's 85 km looks wrong); summit 304-314 m. Nature: Arthurs Seat State Park covers the western half with many walking tracks (Two Bays track, Kings Falls circuit); dry open eucalypt forest, burnt in 1973 and 1997; weeds on the NW face [Wikipedia; Victorian Places]; N 9 consistent. Village: no centre; residential area east of the summit 'shading into open country towards Main Ridge'; tourist attractions (Seawinds gardens, maze, restaurants) [Victorian Places; Wikipedia]; R 6 generous for a locality with no shops (4 arguable). Shops: none named; Q 2 consistent. Beach: Dromana and McCrae beaches below; U 6 plausible. Train: none; S 1 consistent. Indian community: 0 India-born, 0 Indian ancestry [ABS 2021 GCP SAL20072]; P 1 consistent. Very small population: ABS perturbs small counts. City trip: no rail; V 2 consistent. NOT checked: road access for older drivers, bushfire overlay. Scores unchanged. | C3 28 Oct 2026: R 6-&gt;4 (source: no village centre or shops; residential area 'shading into open country towards Main Ridge' [Victorian Places Arthurs Seat]).</t>
         </is>
       </c>
       <c r="AB66" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Workbook: add six Community comparator rows (67-72), display-only band AX, DiscussionSummary list and rule
Rows are not ranked (no judgement scores; L avoids 'pass' so Y and the
Passing count are unchanged). Recalc: 0 errors; X/Y rows 2-66 unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013uWqdtxBL1QFjMDN6afhAy
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -157,7 +157,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -255,6 +255,9 @@
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -460,6 +463,11 @@
     <comment ref="AV1" authorId="1" shapeId="0">
       <text>
         <t>From ABS GCP table G13 (about 45 named languages). Languages ABS groups as "other" there (e.g. Telugu, Burmese, Zomi) cannot appear; QuickStats top-responses may differ.</t>
+      </text>
+    </comment>
+    <comment ref="AX1" authorId="1" shapeId="0">
+      <text>
+        <t>Comparison band, not a liveability score. Display-only: not used in X, Y or any weight, and does not change P. High: other language at home (AU) &gt;= 50% or born in India (AQ) &gt;= 8%. Medium: AU 30-49% or AQ 4-7.9%. Low: otherwise. Interim thresholds, family to confirm.</t>
       </text>
     </comment>
   </commentList>
@@ -788,7 +796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="15">
@@ -1228,6 +1236,103 @@
         <v/>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Community comparators (display-only; added 28 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Suburbs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Community comparators (approved)</t>
+        </is>
+      </c>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>Springvale, Clayton South, Keysborough, Clyde North (Diverse / lower-green); Endeavour Hills, Wheelers Hill (Potential both; Wheelers Hill community lighter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Nature-first anchors</t>
+        </is>
+      </c>
+      <c r="B34" s="34" t="inlineStr">
+        <is>
+          <t>Frankston, Mordialloc, Seaford</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B35" s="34" t="inlineStr">
+        <is>
+          <t>Rowville</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="B36" s="34" t="inlineStr">
+        <is>
+          <t>Point Cook: 08:00 Glen Waverley drive up to 1 hr 40 (fails 90-min cap at peak); 45–70 min off-peak. Family decision; not in scorecard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
+          <t>Tarneit (08:00 drive up to 1 hr 50); Mount Waverley (median over $1.5M cap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Viewing-shortlist rule (proposed)</t>
+        </is>
+      </c>
+      <c r="B38" s="34" t="inlineStr">
+        <is>
+          <t>The viewing shortlist includes at least 2 Community comparators, at least 1 nature-first anchor, and at least 1 verified Potential both suburb. Community comparators are not included for diversity figures alone; they must meet the purchase-price cap, verified Glen Waverley travel limit, and public 24-hour ED requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6135,7 +6240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AW90"/>
+  <dimension ref="A1:AX90"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="37" max="37"/>
@@ -6151,6 +6256,7 @@
     <col width="13" customWidth="1" style="15" min="47" max="47"/>
     <col width="30" customWidth="1" style="15" min="48" max="48"/>
     <col width="30" customWidth="1" style="15" min="49" max="49"/>
+    <col width="16" customWidth="1" style="15" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1" ht="41.75" customHeight="1" s="15">
@@ -6397,6 +6503,11 @@
       <c r="AW1" s="23" t="inlineStr">
         <is>
           <t>Demography source and caveats</t>
+        </is>
+      </c>
+      <c r="AX1" s="23" t="inlineStr">
+        <is>
+          <t>Community comparison band (display-only)</t>
         </is>
       </c>
     </row>
@@ -8331,6 +8442,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX11" s="22">
+        <f>IF(AU11="","",IF(OR(AU11&gt;=0.5,AQ11&gt;=0.08),"High",IF(OR(AU11&gt;=0.3,AQ11&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="15">
       <c r="A12" s="18" t="inlineStr">
@@ -17511,6 +17626,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX59" s="22">
+        <f>IF(AU59="","",IF(OR(AU59&gt;=0.5,AQ59&gt;=0.08),"High",IF(OR(AU59&gt;=0.3,AQ59&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="15">
       <c r="A60" s="16" t="inlineStr">
@@ -18447,6 +18566,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX64" s="22">
+        <f>IF(AU64="","",IF(OR(AU64&gt;=0.5,AQ64&gt;=0.08),"High",IF(OR(AU64&gt;=0.3,AQ64&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="15">
       <c r="A65" s="16" t="inlineStr">
@@ -18835,16 +18958,78 @@
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="15">
-      <c r="A67" s="16" t="n"/>
-      <c r="B67" s="16" t="n"/>
-      <c r="C67" s="16" t="n"/>
-      <c r="D67" s="16" t="n"/>
-      <c r="E67" s="16" t="n"/>
-      <c r="F67" s="16" t="n"/>
-      <c r="G67" s="16" t="n"/>
-      <c r="H67" s="16" t="n"/>
-      <c r="I67" s="16" t="str"/>
-      <c r="L67" s="16" t="n"/>
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>Springvale</t>
+        </is>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>South-East Melbourne</t>
+        </is>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator — Diverse / lower-green</t>
+        </is>
+      </c>
+      <c r="G67" s="16" t="n">
+        <v>942500</v>
+      </c>
+      <c r="H67" s="16" t="inlineStr">
+        <is>
+          <t>SOI median price, house, 1 Jul 2025–30 Jun 2026 (pricefinder), on SOI 24 Phillip Ave</t>
+        </is>
+      </c>
+      <c r="I67" s="16">
+        <f>G67*(1+Settings!$B$6)</f>
+        <v/>
+      </c>
+      <c r="J67" s="22" t="n">
+        <v>35</v>
+      </c>
+      <c r="K67" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="L67" s="16" t="inlineStr">
+        <is>
+          <t>Comparator: filters met (not ranked)</t>
+        </is>
+      </c>
+      <c r="M67" s="22">
+        <f>IF(J67="","",ROUND(MAX(0,10*(1-J67/Filters!$B$4)),1))</f>
+        <v/>
+      </c>
+      <c r="N67" s="22" t="n"/>
+      <c r="O67" s="22">
+        <f>IF(K67="","",ROUND(MAX(0,10*(1-K67/Filters!$B$5)),1))</f>
+        <v/>
+      </c>
+      <c r="P67" s="22" t="n"/>
+      <c r="Q67" s="22" t="n"/>
+      <c r="R67" s="22" t="n"/>
+      <c r="S67" s="22" t="n"/>
+      <c r="T67" s="22">
+        <f>IF(G67="","",ROUND(MAX(0,MIN(10,10*(Filters!$B$2-G67)/(Filters!$B$2-500000))),1))</f>
+        <v/>
+      </c>
+      <c r="U67" s="22" t="n"/>
+      <c r="V67" s="22" t="n"/>
       <c r="W67" s="16">
         <f>IF(M67="",0,COUNT(M67:V67))</f>
         <v/>
@@ -18857,19 +19042,177 @@
         <f>IF(AND(ISNUMBER(SEARCH("pass",L67)),ISNUMBER(X67)),COUNTIFS(L$2:L$90,"*pass*",X$2:X$90,"&gt;"&amp;X67)+1,"")</f>
         <v/>
       </c>
-      <c r="Z67" s="16" t="n"/>
+      <c r="Z67" s="16" t="inlineStr">
+        <is>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 10–35 min (top 35, passes 90-min cap), 8.3 km via Springvale Rd [https://www.google.com/maps/dir/Springvale%20VIC%203171/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 10–26 min. ED Monash Medical Centre Clayton 10–18 min. Price: SOI median $942,500 house (pricefinder, 1 Jul 2025–30 Jun 2026) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/b0b62daa-8691-4f3f-b21b-fc0a629845ff.pdf]; under-cap listings $700k–$790k. Indian grocery: India Town, 11b/310 Springvale Rd, 4 min (Google Business Profile). Hindu temple: Sankat Mochan Hanuman Mandir, 4 Margaret St, Oakleigh South, 10–20 min (Google, 602 reviews). Church: St Joseph's Catholic, cnr Buckingham Ave &amp; 7 St James Ave, 4 min (Google). ABS 2021: AQ 7.4%, AU 75.6%. Nature: none of real size (Wikipedia Springvale). ESTIMATE: train service (recall). NEEDS VERIFICATION: suitable property under cap; a 6-month SOI gives an outlier median $600k. Full sources: 'Community comparators — research (28 Oct 2026).md'.</t>
+        </is>
+      </c>
+      <c r="AB67" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC67" s="22" t="inlineStr">
+        <is>
+          <t>Springvale station, Cranbourne/Pakenham lines (recall; verify)</t>
+        </is>
+      </c>
+      <c r="AD67" s="22" t="inlineStr">
+        <is>
+          <t>Monash Medical Centre Clayton ED, 10–18 min; public hospital with 24-hour ED (Vic Dept of Health public-hospitals list; healthdirect "Open 24 hours"/"Mixed billing"); drive = top of Google Maps typical range, Depart at Wed 28 Oct 2026 10:00, suburb name not postcode</t>
+        </is>
+      </c>
+      <c r="AE67" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="AF67" s="22" t="inlineStr">
+        <is>
+          <t>Maximum purchase price, excluding transaction and moving costs</t>
+        </is>
+      </c>
+      <c r="AG67" s="22" t="inlineStr">
+        <is>
+          <t>SOI suburb median + under-cap listing</t>
+        </is>
+      </c>
+      <c r="AH67" s="22" t="inlineStr">
+        <is>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AI67" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AJ67" s="22" t="inlineStr">
+        <is>
+          <t>Median $942,500 under $1.5M cap. Houses also list/sell under cap: 24 Phillip Ave SOI range $700k–$770k; 15 Acacia Mews SOI range $720k–$790k with comparables 34 View Rd $730k (3 May 2026), 13 Acacia Mews $790k (27 Mar 2026). Suitable-property check (stairs, size) still needs data.</t>
+        </is>
+      </c>
+      <c r="AK67" s="22" t="inlineStr">
+        <is>
+          <t>SAL22328</t>
+        </is>
+      </c>
+      <c r="AL67" s="32" t="n">
+        <v>22174</v>
+      </c>
+      <c r="AM67" s="22" t="n">
+        <v>36</v>
+      </c>
+      <c r="AN67" s="33" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="AO67" s="33" t="n">
+        <v>0.6629999999999999</v>
+      </c>
+      <c r="AP67" s="33" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="AQ67" s="33" t="n">
+        <v>0.07400000000000001</v>
+      </c>
+      <c r="AR67" s="33" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="AS67" s="33" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="AT67" s="33" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AU67" s="33" t="n">
+        <v>0.7559999999999999</v>
+      </c>
+      <c r="AV67" s="22" t="inlineStr">
+        <is>
+          <t>Vietnamese 25.2%; Mandarin 6.7%; Cantonese 6.3%</t>
+        </is>
+      </c>
+      <c r="AW67" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
+      <c r="AX67" s="22">
+        <f>IF(AU67="","",IF(OR(AU67&gt;=0.5,AQ67&gt;=0.08),"High",IF(OR(AU67&gt;=0.3,AQ67&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="15">
-      <c r="A68" s="16" t="n"/>
-      <c r="B68" s="16" t="n"/>
-      <c r="C68" s="16" t="n"/>
-      <c r="D68" s="16" t="n"/>
-      <c r="E68" s="16" t="n"/>
-      <c r="F68" s="16" t="n"/>
-      <c r="G68" s="16" t="n"/>
-      <c r="H68" s="16" t="n"/>
-      <c r="I68" s="16" t="str"/>
-      <c r="L68" s="16" t="n"/>
+      <c r="A68" s="16" t="inlineStr">
+        <is>
+          <t>Clayton South</t>
+        </is>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>South-East Melbourne</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator — Diverse / lower-green</t>
+        </is>
+      </c>
+      <c r="G68" s="16" t="n">
+        <v>985000</v>
+      </c>
+      <c r="H68" s="16" t="inlineStr">
+        <is>
+          <t>SOI median price, house, 1 Apr 2025–31 Mar 2026 (pricefinder), on SOI 85 Osborne Ave</t>
+        </is>
+      </c>
+      <c r="I68" s="16">
+        <f>G68*(1+Settings!$B$6)</f>
+        <v/>
+      </c>
+      <c r="J68" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="K68" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="L68" s="16" t="inlineStr">
+        <is>
+          <t>Comparator: filters met (not ranked)</t>
+        </is>
+      </c>
+      <c r="M68" s="22">
+        <f>IF(J68="","",ROUND(MAX(0,10*(1-J68/Filters!$B$4)),1))</f>
+        <v/>
+      </c>
+      <c r="N68" s="22" t="n"/>
+      <c r="O68" s="22">
+        <f>IF(K68="","",ROUND(MAX(0,10*(1-K68/Filters!$B$5)),1))</f>
+        <v/>
+      </c>
+      <c r="P68" s="22" t="n"/>
+      <c r="Q68" s="22" t="n"/>
+      <c r="R68" s="22" t="n"/>
+      <c r="S68" s="22" t="n"/>
+      <c r="T68" s="22">
+        <f>IF(G68="","",ROUND(MAX(0,MIN(10,10*(Filters!$B$2-G68)/(Filters!$B$2-500000))),1))</f>
+        <v/>
+      </c>
+      <c r="U68" s="22" t="n"/>
+      <c r="V68" s="22" t="n"/>
       <c r="W68" s="16">
         <f>IF(M68="",0,COUNT(M68:V68))</f>
         <v/>
@@ -18882,19 +19225,177 @@
         <f>IF(AND(ISNUMBER(SEARCH("pass",L68)),ISNUMBER(X68)),COUNTIFS(L$2:L$90,"*pass*",X$2:X$90,"&gt;"&amp;X68)+1,"")</f>
         <v/>
       </c>
-      <c r="Z68" s="16" t="n"/>
+      <c r="Z68" s="16" t="inlineStr">
+        <is>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 16–40 min (top 40, passes), 11.4 km [https://www.google.com/maps/dir/Clayton%20South%20VIC%203169/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 14–35 min. ED Monash Medical Centre Clayton 8–12 min. Price: SOI median $985,000 house (pricefinder, Apr 2025–Mar 2026) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/daf40c18-47a7-4907-9f9a-1801cc782a35.pdf]; listing $1.00–1.08M and three comparables ~$1.0M. Indian grocery: Sarawan Spices, 335 Clayton Rd, Clayton, 5–8 min (Google Business Profile, confirmed operating); Little India Mart, 2/1310 Centre Rd, 4–6 min (Google). Hindu temple: Sankat Mochan Hanuman Mandir, Oakleigh South, 7–12 min (Google). Church: St Andrews Catholic, 76 Springs Rd, 5 min (Google). ABS 2021: AQ 14.9%, AU 67.1%. Nature: golf course and landfill; no named reserve (Victorian Places). ESTIMATE: Little India Mart's suburb (listing does not print it); train access (recall). NEEDS VERIFICATION: suitable property under cap.</t>
+        </is>
+      </c>
+      <c r="AB68" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC68" s="22" t="inlineStr">
+        <is>
+          <t>No station in suburb; Westall and Clayton stations nearby (recall; verify)</t>
+        </is>
+      </c>
+      <c r="AD68" s="22" t="inlineStr">
+        <is>
+          <t>Monash Medical Centre Clayton ED, 8–12 min; public hospital with 24-hour ED (Vic Dept of Health public-hospitals list; healthdirect "Open 24 hours"/"Mixed billing"); drive = top of Google Maps typical range, Depart at Wed 28 Oct 2026 10:00, suburb name not postcode</t>
+        </is>
+      </c>
+      <c r="AE68" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="AF68" s="22" t="inlineStr">
+        <is>
+          <t>Maximum purchase price, excluding transaction and moving costs</t>
+        </is>
+      </c>
+      <c r="AG68" s="22" t="inlineStr">
+        <is>
+          <t>SOI suburb median + under-cap listing</t>
+        </is>
+      </c>
+      <c r="AH68" s="22" t="inlineStr">
+        <is>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AI68" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AJ68" s="22" t="inlineStr">
+        <is>
+          <t>Median $985,000 under cap. 85 Osborne Ave SOI range $1.00M–$1.08M; comparables 37 Glenmorgan Cl $1.0M, 15 Clarevale St $1.033M, 3 Hadkinson St $1.045M (May 2026). Suitable-property check still needs data.</t>
+        </is>
+      </c>
+      <c r="AK68" s="22" t="inlineStr">
+        <is>
+          <t>SAL20570</t>
+        </is>
+      </c>
+      <c r="AL68" s="32" t="n">
+        <v>13381</v>
+      </c>
+      <c r="AM68" s="22" t="n">
+        <v>34</v>
+      </c>
+      <c r="AN68" s="33" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="AO68" s="33" t="n">
+        <v>0.628</v>
+      </c>
+      <c r="AP68" s="33" t="n">
+        <v>0.04099999999999999</v>
+      </c>
+      <c r="AQ68" s="33" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="AR68" s="33" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="AS68" s="33" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="AT68" s="33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AU68" s="33" t="n">
+        <v>0.6709999999999999</v>
+      </c>
+      <c r="AV68" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 10.7%; Greek 9.3%; Vietnamese 4.5%</t>
+        </is>
+      </c>
+      <c r="AW68" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
+      <c r="AX68" s="22">
+        <f>IF(AU68="","",IF(OR(AU68&gt;=0.5,AQ68&gt;=0.08),"High",IF(OR(AU68&gt;=0.3,AQ68&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="15">
-      <c r="A69" s="16" t="n"/>
-      <c r="B69" s="16" t="n"/>
-      <c r="C69" s="16" t="n"/>
-      <c r="D69" s="16" t="n"/>
-      <c r="E69" s="16" t="n"/>
-      <c r="F69" s="16" t="n"/>
-      <c r="G69" s="16" t="n"/>
-      <c r="H69" s="16" t="n"/>
-      <c r="I69" s="16" t="str"/>
-      <c r="L69" s="16" t="n"/>
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>Keysborough</t>
+        </is>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>South-East Melbourne</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator — Diverse / lower-green</t>
+        </is>
+      </c>
+      <c r="G69" s="16" t="n">
+        <v>975000</v>
+      </c>
+      <c r="H69" s="16" t="inlineStr">
+        <is>
+          <t>SOI median price, house, 1 Jul 2025–30 Jun 2026 (pricefinder), on SOI 7-9 Cascade Pl</t>
+        </is>
+      </c>
+      <c r="I69" s="16">
+        <f>G69*(1+Settings!$B$6)</f>
+        <v/>
+      </c>
+      <c r="J69" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="K69" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="L69" s="16" t="inlineStr">
+        <is>
+          <t>Comparator: filters met (not ranked)</t>
+        </is>
+      </c>
+      <c r="M69" s="22">
+        <f>IF(J69="","",ROUND(MAX(0,10*(1-J69/Filters!$B$4)),1))</f>
+        <v/>
+      </c>
+      <c r="N69" s="22" t="n"/>
+      <c r="O69" s="22">
+        <f>IF(K69="","",ROUND(MAX(0,10*(1-K69/Filters!$B$5)),1))</f>
+        <v/>
+      </c>
+      <c r="P69" s="22" t="n"/>
+      <c r="Q69" s="22" t="n"/>
+      <c r="R69" s="22" t="n"/>
+      <c r="S69" s="22" t="n"/>
+      <c r="T69" s="22">
+        <f>IF(G69="","",ROUND(MAX(0,MIN(10,10*(Filters!$B$2-G69)/(Filters!$B$2-500000))),1))</f>
+        <v/>
+      </c>
+      <c r="U69" s="22" t="n"/>
+      <c r="V69" s="22" t="n"/>
       <c r="W69" s="16">
         <f>IF(M69="",0,COUNT(M69:V69))</f>
         <v/>
@@ -18907,19 +19408,177 @@
         <f>IF(AND(ISNUMBER(SEARCH("pass",L69)),ISNUMBER(X69)),COUNTIFS(L$2:L$90,"*pass*",X$2:X$90,"&gt;"&amp;X69)+1,"")</f>
         <v/>
       </c>
-      <c r="Z69" s="16" t="n"/>
+      <c r="Z69" s="16" t="inlineStr">
+        <is>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 18–30 min (top 30, passes), 21.0 km via M3 [https://www.google.com/maps/dir/Keysborough%20VIC%203173/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 18–24 min. ED Dandenong Hospital 12–18 min. Price: SOI median $975,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/ca8cd377-fe5e-42cd-a3d6-525992dc0a9d.pdf]; under-cap listing 45 Weston St $1.05–1.155M [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/7b6728e4-a512-4e2d-b761-4e7595257093.pdf]. Indian grocery: India at Home, Parkmore Shopping Centre, 4–6 min (Google). Hindu temple: Shri Shiva Vishnu Temple, 52 Boundary Rd, Carrum Downs, 14–20 min (Google, 6,483 reviews); gurdwara at 198-206 Perry Rd in suburb. Church: Resurrection Parish, 402 Corrigan Rd, 5–6 min (Google). ABS 2021: AQ 6.6%, AU 61.1%. Nature: market gardens to the south; no named reserve (Wikipedia). ESTIMATE: no train (recall). NEEDS VERIFICATION: suitable property under cap.</t>
+        </is>
+      </c>
+      <c r="AB69" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC69" s="22" t="inlineStr">
+        <is>
+          <t>No passenger rail in suburb (recall; verify)</t>
+        </is>
+      </c>
+      <c r="AD69" s="22" t="inlineStr">
+        <is>
+          <t>Dandenong Hospital ED, 12–18 min; public hospital with 24-hour ED (Vic Dept of Health public-hospitals list; healthdirect "Open 24 hours"/"Mixed billing"); drive = top of Google Maps typical range, Depart at Wed 28 Oct 2026 10:00, suburb name not postcode</t>
+        </is>
+      </c>
+      <c r="AE69" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="AF69" s="22" t="inlineStr">
+        <is>
+          <t>Maximum purchase price, excluding transaction and moving costs</t>
+        </is>
+      </c>
+      <c r="AG69" s="22" t="inlineStr">
+        <is>
+          <t>SOI suburb median + under-cap listing</t>
+        </is>
+      </c>
+      <c r="AH69" s="22" t="inlineStr">
+        <is>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AI69" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AJ69" s="22" t="inlineStr">
+        <is>
+          <t>Median $975,000 under cap. 45 Weston St SOI range $1.05M–$1.155M; comparables 15 Petunia Dr $1.11M, 9 Annabelle Blvd $1.06M, 13 Sunflower Ct $1.128M (Feb–Jun 2026). Note the median SOI listing itself (7-9 Cascade Pl) is $1.75–1.85M, over cap. Suitable-property check still needs data.</t>
+        </is>
+      </c>
+      <c r="AK69" s="22" t="inlineStr">
+        <is>
+          <t>SAL21339</t>
+        </is>
+      </c>
+      <c r="AL69" s="32" t="n">
+        <v>30018</v>
+      </c>
+      <c r="AM69" s="22" t="n">
+        <v>36</v>
+      </c>
+      <c r="AN69" s="33" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="AO69" s="33" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="AP69" s="33" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AQ69" s="33" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="AR69" s="33" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="AS69" s="33" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="AT69" s="33" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AU69" s="33" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="AV69" s="22" t="inlineStr">
+        <is>
+          <t>Vietnamese 11.5%; Khmer 9.7%; Mandarin 6.8%</t>
+        </is>
+      </c>
+      <c r="AW69" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
+      <c r="AX69" s="22">
+        <f>IF(AU69="","",IF(OR(AU69&gt;=0.5,AQ69&gt;=0.08),"High",IF(OR(AU69&gt;=0.3,AQ69&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="15">
-      <c r="A70" s="16" t="n"/>
-      <c r="B70" s="16" t="n"/>
-      <c r="C70" s="16" t="n"/>
-      <c r="D70" s="16" t="n"/>
-      <c r="E70" s="16" t="n"/>
-      <c r="F70" s="16" t="n"/>
-      <c r="G70" s="16" t="n"/>
-      <c r="H70" s="16" t="n"/>
-      <c r="I70" s="16" t="str"/>
-      <c r="L70" s="16" t="n"/>
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>Clyde North</t>
+        </is>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>South-East Melbourne</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator</t>
+        </is>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F70" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator — Diverse / lower-green</t>
+        </is>
+      </c>
+      <c r="G70" s="16" t="n">
+        <v>752932</v>
+      </c>
+      <c r="H70" s="16" t="inlineStr">
+        <is>
+          <t>SOI median price, house, 1 Jun 2025–31 May 2026 (PropTrack), on SOI 24 Hollywell Rd</t>
+        </is>
+      </c>
+      <c r="I70" s="16">
+        <f>G70*(1+Settings!$B$6)</f>
+        <v/>
+      </c>
+      <c r="J70" s="22" t="n">
+        <v>70</v>
+      </c>
+      <c r="K70" s="22" t="n">
+        <v>24</v>
+      </c>
+      <c r="L70" s="16" t="inlineStr">
+        <is>
+          <t>Comparator: filters met (not ranked)</t>
+        </is>
+      </c>
+      <c r="M70" s="22">
+        <f>IF(J70="","",ROUND(MAX(0,10*(1-J70/Filters!$B$4)),1))</f>
+        <v/>
+      </c>
+      <c r="N70" s="22" t="n"/>
+      <c r="O70" s="22">
+        <f>IF(K70="","",ROUND(MAX(0,10*(1-K70/Filters!$B$5)),1))</f>
+        <v/>
+      </c>
+      <c r="P70" s="22" t="n"/>
+      <c r="Q70" s="22" t="n"/>
+      <c r="R70" s="22" t="n"/>
+      <c r="S70" s="22" t="n"/>
+      <c r="T70" s="22">
+        <f>IF(G70="","",ROUND(MAX(0,MIN(10,10*(Filters!$B$2-G70)/(Filters!$B$2-500000))),1))</f>
+        <v/>
+      </c>
+      <c r="U70" s="22" t="n"/>
+      <c r="V70" s="22" t="n"/>
       <c r="W70" s="16">
         <f>IF(M70="",0,COUNT(M70:V70))</f>
         <v/>
@@ -18932,19 +19591,177 @@
         <f>IF(AND(ISNUMBER(SEARCH("pass",L70)),ISNUMBER(X70)),COUNTIFS(L$2:L$90,"*pass*",X$2:X$90,"&gt;"&amp;X70)+1,"")</f>
         <v/>
       </c>
-      <c r="Z70" s="16" t="n"/>
+      <c r="Z70" s="16" t="inlineStr">
+        <is>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 35 min–1 hr 10 (top 70): passes the 90-min cap, but EXCEEDS A 60-MIN PREFERENCE if the family adopts one; 42.0 km via Thompsons Rd and M3 [https://www.google.com/maps/dir/Clyde%20North%20VIC%203978/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 28–50 min. ED Casey Hospital 12–24 min. Price: SOI median $752,932 house (PropTrack) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/a24be22a-1f37-4f59-820a-aeb288704b8c.pdf]; listing $790–860k and comparables ~$810k. Indian grocery: Wirsa Indian Groceries, 13/16 Selandra Blvd, 2 min (Google). Hindu temple: Shrinathji Haveli, 3-5 Princes Domain Dr, Hallam, 16–30 min (Google, confirmed operating). Church: St Thomas The Apostle Catholic, 5 Fiorelli Blvd, 4 min (Google; replaces the approximate GCatholic location). ABS 2021: AQ 18.2%, AU 53.6%. Nature: green-wedge farmland; regional park only proposed (Wikipedia). ESTIMATE: BAPS Mandir, 175-177 Smiths Ln, 8–12 min (listing does not print suburb); no train (recall). NEEDS VERIFICATION: suitable property under cap.</t>
+        </is>
+      </c>
+      <c r="AB70" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC70" s="22" t="inlineStr">
+        <is>
+          <t>No station in suburb; Cranbourne line nearby (recall; verify)</t>
+        </is>
+      </c>
+      <c r="AD70" s="22" t="inlineStr">
+        <is>
+          <t>Casey Hospital ED, Berwick, 12–24 min; public hospital with 24-hour ED (Vic Dept of Health public-hospitals list; healthdirect "Open 24 hours"/"Mixed billing"); drive = top of Google Maps typical range, Depart at Wed 28 Oct 2026 10:00, suburb name not postcode</t>
+        </is>
+      </c>
+      <c r="AE70" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="AF70" s="22" t="inlineStr">
+        <is>
+          <t>Maximum purchase price, excluding transaction and moving costs</t>
+        </is>
+      </c>
+      <c r="AG70" s="22" t="inlineStr">
+        <is>
+          <t>SOI suburb median + under-cap listing</t>
+        </is>
+      </c>
+      <c r="AH70" s="22" t="inlineStr">
+        <is>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AI70" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AJ70" s="22" t="inlineStr">
+        <is>
+          <t>Median $752,932 under cap. 24 Hollywell Rd SOI range $790k–$860k; comparables 20 &amp; 100 Deoro Pde, 55 Bazadaise Dr $810k–$827.5k (Feb–May 2026). Suitable-property check still needs data.</t>
+        </is>
+      </c>
+      <c r="AK70" s="22" t="inlineStr">
+        <is>
+          <t>SAL20582</t>
+        </is>
+      </c>
+      <c r="AL70" s="32" t="n">
+        <v>31681</v>
+      </c>
+      <c r="AM70" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="AN70" s="33" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="AO70" s="33" t="n">
+        <v>0.507</v>
+      </c>
+      <c r="AP70" s="33" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AQ70" s="33" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="AR70" s="33" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="AS70" s="33" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="AT70" s="33" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="AU70" s="33" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="AV70" s="22" t="inlineStr">
+        <is>
+          <t>Punjabi 11.5%; Sinhalese 7.9%; Malayalam 3.7%</t>
+        </is>
+      </c>
+      <c r="AW70" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
+      <c r="AX70" s="22">
+        <f>IF(AU70="","",IF(OR(AU70&gt;=0.5,AQ70&gt;=0.08),"High",IF(OR(AU70&gt;=0.3,AQ70&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="71" ht="15.75" customHeight="1" s="15">
-      <c r="A71" s="16" t="n"/>
-      <c r="B71" s="16" t="n"/>
-      <c r="C71" s="16" t="n"/>
-      <c r="D71" s="16" t="n"/>
-      <c r="E71" s="16" t="n"/>
-      <c r="F71" s="16" t="n"/>
-      <c r="G71" s="16" t="n"/>
-      <c r="H71" s="16" t="n"/>
-      <c r="I71" s="16" t="str"/>
-      <c r="L71" s="16" t="n"/>
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>Endeavour Hills</t>
+        </is>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>Dandenong Foothills</t>
+        </is>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator — Potential both</t>
+        </is>
+      </c>
+      <c r="G71" s="16" t="n">
+        <v>857000</v>
+      </c>
+      <c r="H71" s="16" t="inlineStr">
+        <is>
+          <t>SOI median price, house, 1 Aug 2025–1 Aug 2026 (Price Finder), on SOI 6 Isaac Smith Cres</t>
+        </is>
+      </c>
+      <c r="I71" s="16">
+        <f>G71*(1+Settings!$B$6)</f>
+        <v/>
+      </c>
+      <c r="J71" s="22" t="n">
+        <v>35</v>
+      </c>
+      <c r="K71" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="L71" s="16" t="inlineStr">
+        <is>
+          <t>Comparator: filters met (not ranked)</t>
+        </is>
+      </c>
+      <c r="M71" s="22">
+        <f>IF(J71="","",ROUND(MAX(0,10*(1-J71/Filters!$B$4)),1))</f>
+        <v/>
+      </c>
+      <c r="N71" s="22" t="n"/>
+      <c r="O71" s="22">
+        <f>IF(K71="","",ROUND(MAX(0,10*(1-K71/Filters!$B$5)),1))</f>
+        <v/>
+      </c>
+      <c r="P71" s="22" t="n"/>
+      <c r="Q71" s="22" t="n"/>
+      <c r="R71" s="22" t="n"/>
+      <c r="S71" s="22" t="n"/>
+      <c r="T71" s="22">
+        <f>IF(G71="","",ROUND(MAX(0,MIN(10,10*(Filters!$B$2-G71)/(Filters!$B$2-500000))),1))</f>
+        <v/>
+      </c>
+      <c r="U71" s="22" t="n"/>
+      <c r="V71" s="22" t="n"/>
       <c r="W71" s="16">
         <f>IF(M71="",0,COUNT(M71:V71))</f>
         <v/>
@@ -18957,19 +19774,177 @@
         <f>IF(AND(ISNUMBER(SEARCH("pass",L71)),ISNUMBER(X71)),COUNTIFS(L$2:L$90,"*pass*",X$2:X$90,"&gt;"&amp;X71)+1,"")</f>
         <v/>
       </c>
-      <c r="Z71" s="16" t="n"/>
+      <c r="Z71" s="16" t="inlineStr">
+        <is>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH (nature and community both realistic weekly). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 18–35 min (top 35, passes), 18.6 km via M3 [https://www.google.com/maps/dir/Endeavour%20Hills%20VIC%203802/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 16–26 min. ED Dandenong Hospital 7–12 min. Price: SOI median $857,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/8fc3f19f-6ab3-47ea-b801-9bbd2d72885f.pdf]; listing $760–820k. Indian grocery: India At Home – Dandenong, Dandenong Plaza, 49 McCrae St, 8–12 min (Google). Hindu temple: Shrinathji Haveli, Hallam, 8–14 min (Google, confirmed operating). Church: St Paul Apostle Catholic, 5 William Hovell Dr, 2 min (Google). Nature: Casuarina Forest / James Alexander Reserve 1.1 km, 3 min; Churchill National Park 8–10 min; Lysterfield Park 12 min. ABS 2021: AQ 4.6%, AU 51.3%. ESTIMATE: reserve walkable from central/northern streets (distance from suburb centre only); no train (recall). NEEDS VERIFICATION: Endeavour Spices (not found on Google Maps; not counted); Shri Sanatan Dharam Society, 126/128 Hallam N Rd (listing has no hours; 4–6 min if open); suitable property under cap.</t>
+        </is>
+      </c>
+      <c r="AB71" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC71" s="22" t="inlineStr">
+        <is>
+          <t>No passenger rail in suburb (recall; verify)</t>
+        </is>
+      </c>
+      <c r="AD71" s="22" t="inlineStr">
+        <is>
+          <t>Dandenong Hospital ED, 7–12 min; public hospital with 24-hour ED (Vic Dept of Health public-hospitals list; healthdirect "Open 24 hours"/"Mixed billing"); drive = top of Google Maps typical range, Depart at Wed 28 Oct 2026 10:00, suburb name not postcode</t>
+        </is>
+      </c>
+      <c r="AE71" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="AF71" s="22" t="inlineStr">
+        <is>
+          <t>Maximum purchase price, excluding transaction and moving costs</t>
+        </is>
+      </c>
+      <c r="AG71" s="22" t="inlineStr">
+        <is>
+          <t>SOI suburb median + under-cap listing</t>
+        </is>
+      </c>
+      <c r="AH71" s="22" t="inlineStr">
+        <is>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AI71" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="AJ71" s="22" t="inlineStr">
+        <is>
+          <t>Median $857,000 under cap. 6 Isaac Smith Cres SOI range $760k–$820k. Suitable-property check still needs data.</t>
+        </is>
+      </c>
+      <c r="AK71" s="22" t="inlineStr">
+        <is>
+          <t>SAL20871</t>
+        </is>
+      </c>
+      <c r="AL71" s="32" t="n">
+        <v>24455</v>
+      </c>
+      <c r="AM71" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="AN71" s="33" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AO71" s="33" t="n">
+        <v>0.492</v>
+      </c>
+      <c r="AP71" s="33" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="AQ71" s="33" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="AR71" s="33" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AS71" s="33" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AT71" s="33" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AU71" s="33" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="AV71" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 4.3%; Sinhalese 3.6%; Arabic 3.1%</t>
+        </is>
+      </c>
+      <c r="AW71" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
+      <c r="AX71" s="22">
+        <f>IF(AU71="","",IF(OR(AU71&gt;=0.5,AQ71&gt;=0.08),"High",IF(OR(AU71&gt;=0.3,AQ71&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="15">
-      <c r="A72" s="16" t="n"/>
-      <c r="B72" s="16" t="n"/>
-      <c r="C72" s="16" t="n"/>
-      <c r="D72" s="16" t="n"/>
-      <c r="E72" s="16" t="n"/>
-      <c r="F72" s="16" t="n"/>
-      <c r="G72" s="16" t="n"/>
-      <c r="H72" s="16" t="n"/>
-      <c r="I72" s="16" t="str"/>
-      <c r="L72" s="16" t="n"/>
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>Wheelers Hill</t>
+        </is>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>Dandenong Foothills</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>Community comparator — Potential both (community lighter)</t>
+        </is>
+      </c>
+      <c r="G72" s="16" t="n">
+        <v>1475000</v>
+      </c>
+      <c r="H72" s="16" t="inlineStr">
+        <is>
+          <t>SOI median price, house, 22 Jun 2025–21 Jun 2026 (Property Data), on SOI 9 Sunnybrook Dr</t>
+        </is>
+      </c>
+      <c r="I72" s="16">
+        <f>G72*(1+Settings!$B$6)</f>
+        <v/>
+      </c>
+      <c r="J72" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="K72" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="L72" s="16" t="inlineStr">
+        <is>
+          <t>Comparator: filters met on median only; suitable-property verification outstanding (not ranked)</t>
+        </is>
+      </c>
+      <c r="M72" s="22">
+        <f>IF(J72="","",ROUND(MAX(0,10*(1-J72/Filters!$B$4)),1))</f>
+        <v/>
+      </c>
+      <c r="N72" s="22" t="n"/>
+      <c r="O72" s="22">
+        <f>IF(K72="","",ROUND(MAX(0,10*(1-K72/Filters!$B$5)),1))</f>
+        <v/>
+      </c>
+      <c r="P72" s="22" t="n"/>
+      <c r="Q72" s="22" t="n"/>
+      <c r="R72" s="22" t="n"/>
+      <c r="S72" s="22" t="n"/>
+      <c r="T72" s="22">
+        <f>IF(G72="","",ROUND(MAX(0,MIN(10,10*(Filters!$B$2-G72)/(Filters!$B$2-500000))),1))</f>
+        <v/>
+      </c>
+      <c r="U72" s="22" t="n"/>
+      <c r="V72" s="22" t="n"/>
       <c r="W72" s="16">
         <f>IF(M72="",0,COUNT(M72:V72))</f>
         <v/>
@@ -18982,7 +19957,103 @@
         <f>IF(AND(ISNUMBER(SEARCH("pass",L72)),ISNUMBER(X72)),COUNTIFS(L$2:L$90,"*pass*",X$2:X$90,"&gt;"&amp;X72)+1,"")</f>
         <v/>
       </c>
-      <c r="Z72" s="16" t="n"/>
+      <c r="Z72" s="16" t="inlineStr">
+        <is>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH, with caveat: community access is lighter (Medium band; nearest Hindu temple 10–20 min). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 4–12 min (top 12, passes), 2.6 km [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 7–12 min. ED Dandenong Hospital 12–18 min. Price: SOI median $1,475,000 house (Property Data) [https://s3-ap-southeast-2.amazonaws.com/attach-property-clientvault-com/3868/11973436/S-13799066/1782296638-118760-9-Sunnybrook-WheelersHillSOI220626.pdf]. Indian grocery: The Heritage Spices, G15/580 Ferntree Gully Rd, 6–9 min (Google). Hindu temple: Shree Swaminarayan Temple, 69 Wadhurst Dr, Boronia, 10–20 min (Google, 253 reviews); Sankat Mochan 14–28; Vakrathunda 16–35. Church: St Justin's Catholic, 48 Whalley Dr, 4 min (Google). Nature: Jells Park (~127 ha) 2.6 km, 6 min. ABS 2021: AQ 4.1%, AU 46.0%. HARD FILTER: Pass on median only; suitable-property verification outstanding. ESTIMATE: budget (under-cap listings $1.28–1.38M and $1.32M from search text only); Jells Park walkable only from eastern streets; no train (recall). NEEDS VERIFICATION: open an under-cap SOI; suitable property under cap.</t>
+        </is>
+      </c>
+      <c r="AB72" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC72" s="22" t="inlineStr">
+        <is>
+          <t>No passenger rail in suburb (recall; verify)</t>
+        </is>
+      </c>
+      <c r="AD72" s="22" t="inlineStr">
+        <is>
+          <t>Dandenong Hospital ED, 12–18 min (MMC 14–30); public hospital with 24-hour ED (Vic Dept of Health public-hospitals list; healthdirect "Open 24 hours"/"Mixed billing"); drive = top of Google Maps typical range, Depart at Wed 28 Oct 2026 10:00, suburb name not postcode</t>
+        </is>
+      </c>
+      <c r="AE72" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="AF72" s="22" t="inlineStr">
+        <is>
+          <t>Maximum purchase price, excluding transaction and moving costs</t>
+        </is>
+      </c>
+      <c r="AG72" s="22" t="inlineStr">
+        <is>
+          <t>SOI suburb median only; under-cap listings ESTIMATE (search text)</t>
+        </is>
+      </c>
+      <c r="AH72" s="22" t="inlineStr">
+        <is>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AI72" s="22" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="AJ72" s="22" t="inlineStr">
+        <is>
+          <t>Pass on median only; suitable-property verification outstanding. Median $1,475,000 is 1.7% under cap (newer SOI medians in search text $1.46–1.494M). Under-cap listings 10 Dalkeith Cl $1.28–1.38M and 22 Darlington Ave $1.32M seen only in search-result text; PDFs not opened (HTTP 403). Not a verified budget pass.</t>
+        </is>
+      </c>
+      <c r="AK72" s="22" t="inlineStr">
+        <is>
+          <t>SAL22766</t>
+        </is>
+      </c>
+      <c r="AL72" s="32" t="n">
+        <v>20652</v>
+      </c>
+      <c r="AM72" s="22" t="n">
+        <v>48</v>
+      </c>
+      <c r="AN72" s="33" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="AO72" s="33" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="AP72" s="33" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AQ72" s="33" t="n">
+        <v>0.04099999999999999</v>
+      </c>
+      <c r="AR72" s="33" t="n">
+        <v>0.05599999999999999</v>
+      </c>
+      <c r="AS72" s="33" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AT72" s="33" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="AU72" s="33" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="AV72" s="22" t="inlineStr">
+        <is>
+          <t>Mandarin 15.4%; Cantonese 4.7%; Greek 4.5%</t>
+        </is>
+      </c>
+      <c r="AW72" s="22" t="inlineStr">
+        <is>
+          <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
+        </is>
+      </c>
+      <c r="AX72" s="22">
+        <f>IF(AU72="","",IF(OR(AU72&gt;=0.5,AQ72&gt;=0.08),"High",IF(OR(AU72&gt;=0.3,AQ72&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="15">
       <c r="A73" s="16" t="n"/>

</xml_diff>

<commit_message>
Pre-Phase-2 checks: Wheelers Hill budget Checked; Endeavour Spices and Sanatan Dharam remain Needs verification; Phase 2 readiness
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013uWqdtxBL1QFjMDN6afhAy
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -796,7 +796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="15">
@@ -1237,26 +1237,26 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>Community comparators (display-only; added 28 Oct 2026)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="22" t="inlineStr">
         <is>
           <t>Suburbs</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="22" t="inlineStr">
         <is>
           <t>Community comparators (approved)</t>
         </is>
@@ -1268,7 +1268,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>Nature-first anchors</t>
         </is>
@@ -1280,7 +1280,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
@@ -1292,7 +1292,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>Conditional</t>
         </is>
@@ -1304,7 +1304,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>Excluded</t>
         </is>
@@ -1316,7 +1316,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>Viewing-shortlist rule (proposed)</t>
         </is>
@@ -1327,12 +1327,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -19776,7 +19770,7 @@
       </c>
       <c r="Z71" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH (nature and community both realistic weekly). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 18–35 min (top 35, passes), 18.6 km via M3 [https://www.google.com/maps/dir/Endeavour%20Hills%20VIC%203802/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 16–26 min. ED Dandenong Hospital 7–12 min. Price: SOI median $857,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/8fc3f19f-6ab3-47ea-b801-9bbd2d72885f.pdf]; listing $760–820k. Indian grocery: India At Home – Dandenong, Dandenong Plaza, 49 McCrae St, 8–12 min (Google). Hindu temple: Shrinathji Haveli, Hallam, 8–14 min (Google, confirmed operating). Church: St Paul Apostle Catholic, 5 William Hovell Dr, 2 min (Google). Nature: Casuarina Forest / James Alexander Reserve 1.1 km, 3 min; Churchill National Park 8–10 min; Lysterfield Park 12 min. ABS 2021: AQ 4.6%, AU 51.3%. ESTIMATE: reserve walkable from central/northern streets (distance from suburb centre only); no train (recall). NEEDS VERIFICATION: Endeavour Spices (not found on Google Maps; not counted); Shri Sanatan Dharam Society, 126/128 Hallam N Rd (listing has no hours; 4–6 min if open); suitable property under cap.</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH (nature and community both realistic weekly). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 18–35 min (top 35, passes), 18.6 km via M3 [https://www.google.com/maps/dir/Endeavour%20Hills%20VIC%203802/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 16–26 min. ED Dandenong Hospital 7–12 min. Price: SOI median $857,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/8fc3f19f-6ab3-47ea-b801-9bbd2d72885f.pdf]; listing $760–820k. Indian grocery: India At Home – Dandenong, Dandenong Plaza, 49 McCrae St, 8–12 min (Google). Hindu temple: Shrinathji Haveli, Hallam, 8–14 min (Google, confirmed operating). Church: St Paul Apostle Catholic, 5 William Hovell Dr, 2 min (Google). Nature: Casuarina Forest / James Alexander Reserve 1.1 km, 3 min; Churchill National Park 8–10 min; Lysterfield Park 12 min. ABS 2021: AQ 4.6%, AU 51.3%. ESTIMATE: reserve walkable from central/northern streets (distance from suburb centre only); no train (recall). NEEDS VERIFICATION: Endeavour Spices (not found on Google Maps; not counted); Shri Sanatan Dharam Society, 126/128 Hallam N Rd (listing has no hours; 4–6 min if open); suitable property under cap. | UPDATE 28 Oct 2026: Endeavour Spices still NEEDS VERIFICATION (no Google Maps listing; web search found no listing, website or directory entry beyond the earlier onlymelbourne record); not counted as community access. Shri Sanatan Dharam Society: opening hours NEEDS VERIFICATION (Google listing shows none; web search found none). ACNC-linked register lists the society at Narre Warren North VIC 3804, so the 126/128 Hallam N Rd site may be in Narre Warren North, not Endeavour Hills; the 4–6 min drive (geocoded with "Endeavour Hills") is therefore an ESTIMATE. Source: https://civicgraph.app/charities/44400281254</t>
         </is>
       </c>
       <c r="AB71" s="22" t="inlineStr">
@@ -19959,7 +19953,7 @@
       </c>
       <c r="Z72" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH, with caveat: community access is lighter (Medium band; nearest Hindu temple 10–20 min). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 4–12 min (top 12, passes), 2.6 km [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 7–12 min. ED Dandenong Hospital 12–18 min. Price: SOI median $1,475,000 house (Property Data) [https://s3-ap-southeast-2.amazonaws.com/attach-property-clientvault-com/3868/11973436/S-13799066/1782296638-118760-9-Sunnybrook-WheelersHillSOI220626.pdf]. Indian grocery: The Heritage Spices, G15/580 Ferntree Gully Rd, 6–9 min (Google). Hindu temple: Shree Swaminarayan Temple, 69 Wadhurst Dr, Boronia, 10–20 min (Google, 253 reviews); Sankat Mochan 14–28; Vakrathunda 16–35. Church: St Justin's Catholic, 48 Whalley Dr, 4 min (Google). Nature: Jells Park (~127 ha) 2.6 km, 6 min. ABS 2021: AQ 4.1%, AU 46.0%. HARD FILTER: Pass on median only; suitable-property verification outstanding. ESTIMATE: budget (under-cap listings $1.28–1.38M and $1.32M from search text only); Jells Park walkable only from eastern streets; no train (recall). NEEDS VERIFICATION: open an under-cap SOI; suitable property under cap.</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH, with caveat: community access is lighter (Medium band; nearest Hindu temple 10–20 min). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 4–12 min (top 12, passes), 2.6 km [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 7–12 min. ED Dandenong Hospital 12–18 min. Price: SOI median $1,475,000 house (Property Data) [https://s3-ap-southeast-2.amazonaws.com/attach-property-clientvault-com/3868/11973436/S-13799066/1782296638-118760-9-Sunnybrook-WheelersHillSOI220626.pdf]. Indian grocery: The Heritage Spices, G15/580 Ferntree Gully Rd, 6–9 min (Google). Hindu temple: Shree Swaminarayan Temple, 69 Wadhurst Dr, Boronia, 10–20 min (Google, 253 reviews); Sankat Mochan 14–28; Vakrathunda 16–35. Church: St Justin's Catholic, 48 Whalley Dr, 4 min (Google). Nature: Jells Park (~127 ha) 2.6 km, 6 min. ABS 2021: AQ 4.1%, AU 46.0%. HARD FILTER: Pass on median only; suitable-property verification outstanding. ESTIMATE: budget (under-cap listings $1.28–1.38M and $1.32M from search text only); Jells Park walkable only from eastern streets; no train (recall). NEEDS VERIFICATION: open an under-cap SOI; suitable property under cap. | UPDATE 28 Oct 2026: budget evidence changed ESTIMATE -&gt; CHECKED. Jellis Craig Wheelers Hill Suburb Report Sep 2026 (data to 6 Sep 2026) lists houses sold under $1.5M, e.g. 8 Bottlebrush Ct 4-bed house $1,215,000 (27 Aug 2026), 4 Locum Ct 4-bed $1,224,500 (8 Aug 2026), 81 Cootamundra Dr 3-bed $1,130,000 (18 Jul 2026); report median $1.46M [https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf]. Agency sold-results report, not an SOI. Suitable-property verification still outstanding.</t>
         </is>
       </c>
       <c r="AB72" s="22" t="inlineStr">
@@ -19987,22 +19981,22 @@
       </c>
       <c r="AG72" s="22" t="inlineStr">
         <is>
-          <t>SOI suburb median only; under-cap listings ESTIMATE (search text)</t>
+          <t>Recorded house sales under cap (agency sold-results report) + SOI suburb median</t>
         </is>
       </c>
       <c r="AH72" s="22" t="inlineStr">
         <is>
-          <t>28 Oct 2026</t>
+          <t>28 Oct 2026 (report data current to 6 Sep 2026)</t>
         </is>
       </c>
       <c r="AI72" s="22" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Checked</t>
         </is>
       </c>
       <c r="AJ72" s="22" t="inlineStr">
         <is>
-          <t>Pass on median only; suitable-property verification outstanding. Median $1,475,000 is 1.7% under cap (newer SOI medians in search text $1.46–1.494M). Under-cap listings 10 Dalkeith Cl $1.28–1.38M and 22 Darlington Ave $1.32M seen only in search-result text; PDFs not opened (HTTP 403). Not a verified budget pass.</t>
+          <t>Budget evidence CHECKED 28 Oct 2026: Jellis Craig "Wheelers Hill Suburb Report" Sep 2026 (data current to 6 Sep 2026; Victorian sales data) lists houses SOLD under $1.5M, e.g. 8 Bottlebrush Ct, 4-bed house, $1,215,000, 27 Aug 2026; 4 Locum Ct, 4-bed house, $1,224,500, 8 Aug 2026; 21 Haversham Ave, 4-bed house, $1,140,000, 27 Jul 2026; 81 Cootamundra Dr, 3-bed house, $1,130,000, 18 Jul 2026; 25 Calderwood Ave $1,370,000; 1 Lanoma Ct $1,360,000; 1 Sean Cl $1,350,000; 58 The Deviation $1,120,000 (10 of the 16 disclosed house prices Jun–Sep 2026 are under cap). Report median house price $1.46M. Source: https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf. Document type: agency sold-results report, not a listing Statement of Information. Earlier search-text listings (10 Dalkeith Cl, 22 Darlington Ave) still not opened. Suitable-property check (stairs, size) still needs data.</t>
         </is>
       </c>
       <c r="AK72" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Wheelers Hill: accept sold-results budget evidence; update column L wording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013uWqdtxBL1QFjMDN6afhAy
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -19917,7 +19917,7 @@
       </c>
       <c r="L72" s="16" t="inlineStr">
         <is>
-          <t>Comparator: filters met on median only; suitable-property verification outstanding (not ranked)</t>
+          <t>Comparator: filters met; suitable-property verification outstanding (not ranked)</t>
         </is>
       </c>
       <c r="M72" s="22">
@@ -19953,7 +19953,7 @@
       </c>
       <c r="Z72" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH, with caveat: community access is lighter (Medium band; nearest Hindu temple 10–20 min). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 4–12 min (top 12, passes), 2.6 km [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 7–12 min. ED Dandenong Hospital 12–18 min. Price: SOI median $1,475,000 house (Property Data) [https://s3-ap-southeast-2.amazonaws.com/attach-property-clientvault-com/3868/11973436/S-13799066/1782296638-118760-9-Sunnybrook-WheelersHillSOI220626.pdf]. Indian grocery: The Heritage Spices, G15/580 Ferntree Gully Rd, 6–9 min (Google). Hindu temple: Shree Swaminarayan Temple, 69 Wadhurst Dr, Boronia, 10–20 min (Google, 253 reviews); Sankat Mochan 14–28; Vakrathunda 16–35. Church: St Justin's Catholic, 48 Whalley Dr, 4 min (Google). Nature: Jells Park (~127 ha) 2.6 km, 6 min. ABS 2021: AQ 4.1%, AU 46.0%. HARD FILTER: Pass on median only; suitable-property verification outstanding. ESTIMATE: budget (under-cap listings $1.28–1.38M and $1.32M from search text only); Jells Park walkable only from eastern streets; no train (recall). NEEDS VERIFICATION: open an under-cap SOI; suitable property under cap. | UPDATE 28 Oct 2026: budget evidence changed ESTIMATE -&gt; CHECKED. Jellis Craig Wheelers Hill Suburb Report Sep 2026 (data to 6 Sep 2026) lists houses sold under $1.5M, e.g. 8 Bottlebrush Ct 4-bed house $1,215,000 (27 Aug 2026), 4 Locum Ct 4-bed $1,224,500 (8 Aug 2026), 81 Cootamundra Dr 3-bed $1,130,000 (18 Jul 2026); report median $1.46M [https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf]. Agency sold-results report, not an SOI. Suitable-property verification still outstanding.</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH, with caveat: community access is lighter (Medium band; nearest Hindu temple 10–20 min). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 4–12 min (top 12, passes), 2.6 km [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 7–12 min. ED Dandenong Hospital 12–18 min. Price: SOI median $1,475,000 house (Property Data) [https://s3-ap-southeast-2.amazonaws.com/attach-property-clientvault-com/3868/11973436/S-13799066/1782296638-118760-9-Sunnybrook-WheelersHillSOI220626.pdf]. Indian grocery: The Heritage Spices, G15/580 Ferntree Gully Rd, 6–9 min (Google). Hindu temple: Shree Swaminarayan Temple, 69 Wadhurst Dr, Boronia, 10–20 min (Google, 253 reviews); Sankat Mochan 14–28; Vakrathunda 16–35. Church: St Justin's Catholic, 48 Whalley Dr, 4 min (Google). Nature: Jells Park (~127 ha) 2.6 km, 6 min. ABS 2021: AQ 4.1%, AU 46.0%. HARD FILTER: Pass on median only; suitable-property verification outstanding. ESTIMATE: budget (under-cap listings $1.28–1.38M and $1.32M from search text only); Jells Park walkable only from eastern streets; no train (recall). NEEDS VERIFICATION: open an under-cap SOI; suitable property under cap. | UPDATE 28 Oct 2026: budget evidence changed ESTIMATE -&gt; CHECKED. Jellis Craig Wheelers Hill Suburb Report Sep 2026 (data to 6 Sep 2026) lists houses sold under $1.5M, e.g. 8 Bottlebrush Ct 4-bed house $1,215,000 (27 Aug 2026), 4 Locum Ct 4-bed $1,224,500 (8 Aug 2026), 81 Cootamundra Dr 3-bed $1,130,000 (18 Jul 2026); report median $1.46M [https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf]. Agency sold-results report, not an SOI. Suitable-property verification still outstanding. | 28 Oct 2026: family accepted this report as Checked budget evidence. It shows recent sold houses under the cap; it does NOT verify that a specific suitable downsizing/family home is available. L updated to "filters met; suitable-property verification outstanding".</t>
         </is>
       </c>
       <c r="AB72" s="22" t="inlineStr">
@@ -19996,7 +19996,7 @@
       </c>
       <c r="AJ72" s="22" t="inlineStr">
         <is>
-          <t>Budget evidence CHECKED 28 Oct 2026: Jellis Craig "Wheelers Hill Suburb Report" Sep 2026 (data current to 6 Sep 2026; Victorian sales data) lists houses SOLD under $1.5M, e.g. 8 Bottlebrush Ct, 4-bed house, $1,215,000, 27 Aug 2026; 4 Locum Ct, 4-bed house, $1,224,500, 8 Aug 2026; 21 Haversham Ave, 4-bed house, $1,140,000, 27 Jul 2026; 81 Cootamundra Dr, 3-bed house, $1,130,000, 18 Jul 2026; 25 Calderwood Ave $1,370,000; 1 Lanoma Ct $1,360,000; 1 Sean Cl $1,350,000; 58 The Deviation $1,120,000 (10 of the 16 disclosed house prices Jun–Sep 2026 are under cap). Report median house price $1.46M. Source: https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf. Document type: agency sold-results report, not a listing Statement of Information. Earlier search-text listings (10 Dalkeith Cl, 22 Darlington Ave) still not opened. Suitable-property check (stairs, size) still needs data.</t>
+          <t>Budget evidence CHECKED 28 Oct 2026: Jellis Craig "Wheelers Hill Suburb Report" Sep 2026 (data current to 6 Sep 2026; Victorian sales data) lists houses SOLD under $1.5M, e.g. 8 Bottlebrush Ct, 4-bed house, $1,215,000, 27 Aug 2026; 4 Locum Ct, 4-bed house, $1,224,500, 8 Aug 2026; 21 Haversham Ave, 4-bed house, $1,140,000, 27 Jul 2026; 81 Cootamundra Dr, 3-bed house, $1,130,000, 18 Jul 2026; 25 Calderwood Ave $1,370,000; 1 Lanoma Ct $1,360,000; 1 Sean Cl $1,350,000; 58 The Deviation $1,120,000 (10 of the 16 disclosed house prices Jun–Sep 2026 are under cap). Report median house price $1.46M. Source: https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf. Document type: agency sold-results report, not a listing Statement of Information. Earlier search-text listings (10 Dalkeith Cl, 22 Darlington Ave) still not opened. Suitable-property check (stairs, size) still needs data. Accepted by family 28 Oct 2026 as Checked budget evidence; supports further suitable-property investigation only, not a verified suitable property.</t>
         </is>
       </c>
       <c r="AK72" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Comparator fixes: 10:00 drive basis in J, Tarneit family decision, AX on all rows, Q13d rows
J67-J72 now the top of the checked 10:00 weekday range (26, 35, 24, 50, 26,
12); 08:00 kept in Z as peak, not used in J. Tarneit reason recorded as the
family's decision (no filter failure). AX band filled on every row with ABS
data. Q13d added to RawResponses and CleanedAnswers, feeding no weight.
Recalc 0 errors; X/Y rows 2-66 unchanged; Passing 51.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013uWqdtxBL1QFjMDN6afhAy
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -436,6 +436,36 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="AN1" authorId="0" shapeId="0">
+      <text>
+        <t>Q13d (Round 4, reference-only; feeds no weight, ForcedChoiceCorrections or PriorityWeights). "If both options were within 30 minutes of family, which would you prefer for everyday living?" A = very green, peaceful village or bushland-edge suburb; Indian groceries, a Hindu temple and churches about 30 min away. B = more multicultural neighbourhood; Indian groceries, temples and churches close by, fewer trees and trails. Scale: A strongly / A slightly / No strong preference / B slightly / B strongly.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="A40" authorId="0" shapeId="0">
+      <text>
+        <t>Q13d (Round 4, reference-only; feeds no weight, ForcedChoiceCorrections or PriorityWeights). "If both options were within 30 minutes of family, which would you prefer for everyday living?" A = very green, peaceful village or bushland-edge suburb; Indian groceries, a Hindu temple and churches about 30 min away. B = more multicultural neighbourhood; Indian groceries, temples and churches close by, fewer trees and trails. Scale: A strongly / A slightly / No strong preference / B slightly / B strongly.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
     <author>Unknown Author</author>
     <author>Claude</author>
   </authors>
@@ -1311,7 +1341,7 @@
       </c>
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>Tarneit (08:00 drive up to 1 hr 50); Mount Waverley (median over $1.5M cap)</t>
+          <t>Tarneit: Excluded — family decision 28 Oct 2026 (stated reasons: safety concerns and not enough going for it). Mount Waverley (median over $1.5M cap)</t>
         </is>
       </c>
     </row>
@@ -1656,8 +1686,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AM15"/>
+  <dimension ref="A1:AN15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13" customWidth="1" style="15" min="39" max="39"/>
+    <col width="13" customWidth="1" style="15" min="40" max="40"/>
+  </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="15">
       <c r="A1" s="16" t="inlineStr">
@@ -1853,6 +1887,11 @@
       <c r="AM1" s="16" t="inlineStr">
         <is>
           <t>[Gap-form notes]</t>
+        </is>
+      </c>
+      <c r="AN1" s="16" t="inlineStr">
+        <is>
+          <t>[Q13d] Green village vs multicultural neighbourhood (reference-only)</t>
         </is>
       </c>
     </row>
@@ -3772,6 +3811,7 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3781,7 +3821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="15">
@@ -4845,10 +4885,42 @@
         <v/>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>[Q13d]</t>
+        </is>
+      </c>
+      <c r="B40" s="16">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$AN,$B$2,MATCH($A40&amp;"*",RawResponses!$A$1:$AN$1,0))="","",INDEX(RawResponses!$A:$AN,$B$2,MATCH($A40&amp;"*",RawResponses!$A$1:$AN$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C40" s="16">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$AN,$B$3,MATCH($A40&amp;"*",RawResponses!$A$1:$AN$1,0))="","",INDEX(RawResponses!$A:$AN,$B$3,MATCH($A40&amp;"*",RawResponses!$A$1:$AN$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D40" s="16">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$AN,$B$4,MATCH($A40&amp;"*",RawResponses!$A$1:$AN$1,0))="","",INDEX(RawResponses!$A:$AN,$B$4,MATCH($A40&amp;"*",RawResponses!$A$1:$AN$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E40" s="16">
+        <f>LEFT(B40,1)</f>
+        <v/>
+      </c>
+      <c r="F40" s="16">
+        <f>LEFT(C40,1)</f>
+        <v/>
+      </c>
+      <c r="G40" s="16">
+        <f>LEFT(D40,1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -6682,6 +6754,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX2" s="22">
+        <f>IF(AU2="","",IF(OR(AU2&gt;=0.5,AQ2&gt;=0.08),"High",IF(OR(AU2&gt;=0.3,AQ2&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="15">
       <c r="A3" s="18" t="inlineStr">
@@ -6879,6 +6955,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX3" s="22">
+        <f>IF(AU3="","",IF(OR(AU3&gt;=0.5,AQ3&gt;=0.08),"High",IF(OR(AU3&gt;=0.3,AQ3&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1" s="15">
       <c r="A4" s="18" t="inlineStr">
@@ -7076,6 +7156,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX4" s="22">
+        <f>IF(AU4="","",IF(OR(AU4&gt;=0.5,AQ4&gt;=0.08),"High",IF(OR(AU4&gt;=0.3,AQ4&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="15">
       <c r="A5" s="18" t="inlineStr">
@@ -7273,6 +7357,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX5" s="22">
+        <f>IF(AU5="","",IF(OR(AU5&gt;=0.5,AQ5&gt;=0.08),"High",IF(OR(AU5&gt;=0.3,AQ5&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="15">
       <c r="A6" s="18" t="inlineStr">
@@ -7469,6 +7557,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX6" s="22">
+        <f>IF(AU6="","",IF(OR(AU6&gt;=0.5,AQ6&gt;=0.08),"High",IF(OR(AU6&gt;=0.3,AQ6&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="15">
@@ -7647,6 +7739,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX7" s="22">
+        <f>IF(AU7="","",IF(OR(AU7&gt;=0.5,AQ7&gt;=0.08),"High",IF(OR(AU7&gt;=0.3,AQ7&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="15">
       <c r="A8" s="18" t="inlineStr">
@@ -7845,6 +7941,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX8" s="22">
+        <f>IF(AU8="","",IF(OR(AU8&gt;=0.5,AQ8&gt;=0.08),"High",IF(OR(AU8&gt;=0.3,AQ8&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="15">
       <c r="A9" s="18" t="inlineStr">
@@ -8042,6 +8142,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX9" s="22">
+        <f>IF(AU9="","",IF(OR(AU9&gt;=0.5,AQ9&gt;=0.08),"High",IF(OR(AU9&gt;=0.3,AQ9&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="15">
       <c r="A10" s="18" t="inlineStr">
@@ -8239,6 +8343,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX10" s="22">
+        <f>IF(AU10="","",IF(OR(AU10&gt;=0.5,AQ10&gt;=0.08),"High",IF(OR(AU10&gt;=0.3,AQ10&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="15">
       <c r="A11" s="18" t="inlineStr">
@@ -8636,6 +8744,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX12" s="22">
+        <f>IF(AU12="","",IF(OR(AU12&gt;=0.5,AQ12&gt;=0.08),"High",IF(OR(AU12&gt;=0.3,AQ12&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="15">
@@ -8814,6 +8926,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX13" s="22">
+        <f>IF(AU13="","",IF(OR(AU13&gt;=0.5,AQ13&gt;=0.08),"High",IF(OR(AU13&gt;=0.3,AQ13&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="15">
       <c r="A14" s="18" t="inlineStr">
@@ -9012,6 +9128,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX14" s="22">
+        <f>IF(AU14="","",IF(OR(AU14&gt;=0.5,AQ14&gt;=0.08),"High",IF(OR(AU14&gt;=0.3,AQ14&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="15">
       <c r="A15" s="18" t="inlineStr">
@@ -9209,6 +9329,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX15" s="22">
+        <f>IF(AU15="","",IF(OR(AU15&gt;=0.5,AQ15&gt;=0.08),"High",IF(OR(AU15&gt;=0.3,AQ15&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="15">
       <c r="A16" s="18" t="inlineStr">
@@ -9406,6 +9530,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX16" s="22">
+        <f>IF(AU16="","",IF(OR(AU16&gt;=0.5,AQ16&gt;=0.08),"High",IF(OR(AU16&gt;=0.3,AQ16&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="15">
       <c r="A17" s="18" t="inlineStr">
@@ -9604,6 +9732,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
+      <c r="AX17" s="22">
+        <f>IF(AU17="","",IF(OR(AU17&gt;=0.5,AQ17&gt;=0.08),"High",IF(OR(AU17&gt;=0.3,AQ17&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="15">
       <c r="A18" s="18" t="inlineStr">
@@ -9800,6 +9932,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX18" s="22">
+        <f>IF(AU18="","",IF(OR(AU18&gt;=0.5,AQ18&gt;=0.08),"High",IF(OR(AU18&gt;=0.3,AQ18&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="15">
@@ -9978,6 +10114,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX19" s="22">
+        <f>IF(AU19="","",IF(OR(AU19&gt;=0.5,AQ19&gt;=0.08),"High",IF(OR(AU19&gt;=0.3,AQ19&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="15">
       <c r="A20" s="18" t="inlineStr">
@@ -10176,6 +10316,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Newtown (Greater Geelong), SAL21938.</t>
         </is>
       </c>
+      <c r="AX20" s="22">
+        <f>IF(AU20="","",IF(OR(AU20&gt;=0.5,AQ20&gt;=0.08),"High",IF(OR(AU20&gt;=0.3,AQ20&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="15">
       <c r="A21" s="18" t="inlineStr">
@@ -10374,6 +10518,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX21" s="22">
+        <f>IF(AU21="","",IF(OR(AU21&gt;=0.5,AQ21&gt;=0.08),"High",IF(OR(AU21&gt;=0.3,AQ21&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="15">
       <c r="A22" s="18" t="inlineStr">
@@ -10572,6 +10720,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX22" s="22">
+        <f>IF(AU22="","",IF(OR(AU22&gt;=0.5,AQ22&gt;=0.08),"High",IF(OR(AU22&gt;=0.3,AQ22&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="15">
       <c r="A23" s="18" t="inlineStr">
@@ -10769,6 +10921,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX23" s="22">
+        <f>IF(AU23="","",IF(OR(AU23&gt;=0.5,AQ23&gt;=0.08),"High",IF(OR(AU23&gt;=0.3,AQ23&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="15">
       <c r="A24" s="18" t="inlineStr">
@@ -10967,6 +11123,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
+      <c r="AX24" s="22">
+        <f>IF(AU24="","",IF(OR(AU24&gt;=0.5,AQ24&gt;=0.08),"High",IF(OR(AU24&gt;=0.3,AQ24&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="15">
       <c r="A25" s="18" t="inlineStr">
@@ -11165,6 +11325,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX25" s="22">
+        <f>IF(AU25="","",IF(OR(AU25&gt;=0.5,AQ25&gt;=0.08),"High",IF(OR(AU25&gt;=0.3,AQ25&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="15">
       <c r="A26" s="18" t="inlineStr">
@@ -11363,6 +11527,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX26" s="22">
+        <f>IF(AU26="","",IF(OR(AU26&gt;=0.5,AQ26&gt;=0.08),"High",IF(OR(AU26&gt;=0.3,AQ26&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="15">
       <c r="A27" s="18" t="inlineStr">
@@ -11561,6 +11729,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX27" s="22">
+        <f>IF(AU27="","",IF(OR(AU27&gt;=0.5,AQ27&gt;=0.08),"High",IF(OR(AU27&gt;=0.3,AQ27&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="15">
       <c r="A28" s="18" t="inlineStr">
@@ -11759,6 +11931,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX28" s="22">
+        <f>IF(AU28="","",IF(OR(AU28&gt;=0.5,AQ28&gt;=0.08),"High",IF(OR(AU28&gt;=0.3,AQ28&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="15">
       <c r="A29" s="18" t="inlineStr">
@@ -11955,6 +12131,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX29" s="22">
+        <f>IF(AU29="","",IF(OR(AU29&gt;=0.5,AQ29&gt;=0.08),"High",IF(OR(AU29&gt;=0.3,AQ29&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="15">
@@ -12134,6 +12314,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX30" s="22">
+        <f>IF(AU30="","",IF(OR(AU30&gt;=0.5,AQ30&gt;=0.08),"High",IF(OR(AU30&gt;=0.3,AQ30&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="15">
       <c r="A31" s="18" t="inlineStr">
@@ -12331,6 +12515,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX31" s="22">
+        <f>IF(AU31="","",IF(OR(AU31&gt;=0.5,AQ31&gt;=0.08),"High",IF(OR(AU31&gt;=0.3,AQ31&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="15">
@@ -12509,6 +12697,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX32" s="22">
+        <f>IF(AU32="","",IF(OR(AU32&gt;=0.5,AQ32&gt;=0.08),"High",IF(OR(AU32&gt;=0.3,AQ32&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="15">
       <c r="A33" s="18" t="inlineStr">
@@ -12705,6 +12897,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
+      </c>
+      <c r="AX33" s="22">
+        <f>IF(AU33="","",IF(OR(AU33&gt;=0.5,AQ33&gt;=0.08),"High",IF(OR(AU33&gt;=0.3,AQ33&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="15">
@@ -12883,6 +13079,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
+      <c r="AX34" s="22">
+        <f>IF(AU34="","",IF(OR(AU34&gt;=0.5,AQ34&gt;=0.08),"High",IF(OR(AU34&gt;=0.3,AQ34&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="15">
       <c r="A35" s="18" t="inlineStr">
@@ -13081,6 +13281,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
+      <c r="AX35" s="22">
+        <f>IF(AU35="","",IF(OR(AU35&gt;=0.5,AQ35&gt;=0.08),"High",IF(OR(AU35&gt;=0.3,AQ35&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="15">
       <c r="A36" s="18" t="inlineStr">
@@ -13279,6 +13483,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
+      <c r="AX36" s="22">
+        <f>IF(AU36="","",IF(OR(AU36&gt;=0.5,AQ36&gt;=0.08),"High",IF(OR(AU36&gt;=0.3,AQ36&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="15">
       <c r="A37" s="18" t="inlineStr">
@@ -13477,6 +13685,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
+      <c r="AX37" s="22">
+        <f>IF(AU37="","",IF(OR(AU37&gt;=0.5,AQ37&gt;=0.08),"High",IF(OR(AU37&gt;=0.3,AQ37&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="15">
       <c r="A38" s="18" t="inlineStr">
@@ -13675,6 +13887,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX38" s="22">
+        <f>IF(AU38="","",IF(OR(AU38&gt;=0.5,AQ38&gt;=0.08),"High",IF(OR(AU38&gt;=0.3,AQ38&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="15">
       <c r="A39" s="18" t="inlineStr">
@@ -13873,6 +14089,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX39" s="22">
+        <f>IF(AU39="","",IF(OR(AU39&gt;=0.5,AQ39&gt;=0.08),"High",IF(OR(AU39&gt;=0.3,AQ39&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="15">
       <c r="A40" s="18" t="inlineStr">
@@ -14071,6 +14291,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX40" s="22">
+        <f>IF(AU40="","",IF(OR(AU40&gt;=0.5,AQ40&gt;=0.08),"High",IF(OR(AU40&gt;=0.3,AQ40&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="15">
       <c r="A41" s="18" t="inlineStr">
@@ -14269,6 +14493,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX41" s="22">
+        <f>IF(AU41="","",IF(OR(AU41&gt;=0.5,AQ41&gt;=0.08),"High",IF(OR(AU41&gt;=0.3,AQ41&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="15">
       <c r="A42" s="18" t="inlineStr">
@@ -14466,6 +14694,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX42" s="22">
+        <f>IF(AU42="","",IF(OR(AU42&gt;=0.5,AQ42&gt;=0.08),"High",IF(OR(AU42&gt;=0.3,AQ42&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="15">
@@ -14645,6 +14877,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. CAVEAT: Ballarat Central locality only (CBD, pop 5,378), not the whole city.</t>
         </is>
       </c>
+      <c r="AX43" s="22">
+        <f>IF(AU43="","",IF(OR(AU43&gt;=0.5,AQ43&gt;=0.08),"High",IF(OR(AU43&gt;=0.3,AQ43&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="15">
       <c r="A44" s="18" t="inlineStr">
@@ -14823,6 +15059,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. CAVEAT: Bendigo locality (central, pop 5,652), not the whole city.</t>
         </is>
       </c>
+      <c r="AX44" s="22">
+        <f>IF(AU44="","",IF(OR(AU44&gt;=0.5,AQ44&gt;=0.08),"High",IF(OR(AU44&gt;=0.3,AQ44&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="15">
       <c r="A45" s="18" t="inlineStr">
@@ -15020,6 +15260,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX45" s="22">
+        <f>IF(AU45="","",IF(OR(AU45&gt;=0.5,AQ45&gt;=0.08),"High",IF(OR(AU45&gt;=0.3,AQ45&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="15">
@@ -15199,6 +15443,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX46" s="22">
+        <f>IF(AU46="","",IF(OR(AU46&gt;=0.5,AQ46&gt;=0.08),"High",IF(OR(AU46&gt;=0.3,AQ46&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="15">
       <c r="A47" s="18" t="inlineStr">
@@ -15396,6 +15644,10 @@
         <is>
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
+      </c>
+      <c r="AX47" s="22">
+        <f>IF(AU47="","",IF(OR(AU47&gt;=0.5,AQ47&gt;=0.08),"High",IF(OR(AU47&gt;=0.3,AQ47&gt;=0.04),"Medium","Low")))</f>
+        <v/>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="15">
@@ -15575,6 +15827,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX48" s="22">
+        <f>IF(AU48="","",IF(OR(AU48&gt;=0.5,AQ48&gt;=0.08),"High",IF(OR(AU48&gt;=0.3,AQ48&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="15">
       <c r="A49" s="18" t="inlineStr">
@@ -16051,6 +16307,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX51" s="22">
+        <f>IF(AU51="","",IF(OR(AU51&gt;=0.5,AQ51&gt;=0.08),"High",IF(OR(AU51&gt;=0.3,AQ51&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="15">
       <c r="A52" s="16" t="inlineStr">
@@ -16249,6 +16509,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX52" s="22">
+        <f>IF(AU52="","",IF(OR(AU52&gt;=0.5,AQ52&gt;=0.08),"High",IF(OR(AU52&gt;=0.3,AQ52&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="15">
       <c r="A53" s="16" t="inlineStr">
@@ -16447,6 +16711,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX53" s="22">
+        <f>IF(AU53="","",IF(OR(AU53&gt;=0.5,AQ53&gt;=0.08),"High",IF(OR(AU53&gt;=0.3,AQ53&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="15">
       <c r="A54" s="16" t="inlineStr">
@@ -16645,6 +16913,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX54" s="22">
+        <f>IF(AU54="","",IF(OR(AU54&gt;=0.5,AQ54&gt;=0.08),"High",IF(OR(AU54&gt;=0.3,AQ54&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="15">
       <c r="A55" s="16" t="inlineStr">
@@ -16843,6 +17115,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX55" s="22">
+        <f>IF(AU55="","",IF(OR(AU55&gt;=0.5,AQ55&gt;=0.08),"High",IF(OR(AU55&gt;=0.3,AQ55&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="15">
       <c r="A56" s="16" t="inlineStr">
@@ -17041,6 +17317,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX56" s="22">
+        <f>IF(AU56="","",IF(OR(AU56&gt;=0.5,AQ56&gt;=0.08),"High",IF(OR(AU56&gt;=0.3,AQ56&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="15">
       <c r="A57" s="16" t="inlineStr">
@@ -17234,6 +17514,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX57" s="22">
+        <f>IF(AU57="","",IF(OR(AU57&gt;=0.5,AQ57&gt;=0.08),"High",IF(OR(AU57&gt;=0.3,AQ57&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="15">
       <c r="A58" s="16" t="inlineStr">
@@ -17427,6 +17711,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX58" s="22">
+        <f>IF(AU58="","",IF(OR(AU58&gt;=0.5,AQ58&gt;=0.08),"High",IF(OR(AU58&gt;=0.3,AQ58&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="15">
       <c r="A59" s="16" t="inlineStr">
@@ -17817,6 +18105,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX60" s="22">
+        <f>IF(AU60="","",IF(OR(AU60&gt;=0.5,AQ60&gt;=0.08),"High",IF(OR(AU60&gt;=0.3,AQ60&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="15">
       <c r="A61" s="16" t="inlineStr">
@@ -17981,6 +18273,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX61" s="22">
+        <f>IF(AU61="","",IF(OR(AU61&gt;=0.5,AQ61&gt;=0.08),"High",IF(OR(AU61&gt;=0.3,AQ61&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="15">
       <c r="A62" s="16" t="inlineStr">
@@ -18174,6 +18470,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX62" s="22">
+        <f>IF(AU62="","",IF(OR(AU62&gt;=0.5,AQ62&gt;=0.08),"High",IF(OR(AU62&gt;=0.3,AQ62&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="15">
       <c r="A63" s="16" t="inlineStr">
@@ -18367,6 +18667,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX63" s="22">
+        <f>IF(AU63="","",IF(OR(AU63&gt;=0.5,AQ63&gt;=0.08),"High",IF(OR(AU63&gt;=0.3,AQ63&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="15">
       <c r="A64" s="16" t="inlineStr">
@@ -18757,6 +19061,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence.</t>
         </is>
       </c>
+      <c r="AX65" s="22">
+        <f>IF(AU65="","",IF(OR(AU65&gt;=0.5,AQ65&gt;=0.08),"High",IF(OR(AU65&gt;=0.3,AQ65&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="15">
       <c r="A66" s="16" t="inlineStr">
@@ -18950,6 +19258,10 @@
           <t>ABS 2021 Census General Community Profile DataPack, Suburbs and Localities (SAL), Victoria (tables G01, G02, G08, G09, G13, G14); downloaded 27 Oct 2026 from abs.gov.au. Place of usual residence. Small population: ABS randomly adjusts small counts, so treat shares under 1% as noise.</t>
         </is>
       </c>
+      <c r="AX66" s="22">
+        <f>IF(AU66="","",IF(OR(AU66&gt;=0.5,AQ66&gt;=0.08),"High",IF(OR(AU66&gt;=0.3,AQ66&gt;=0.04),"Medium","Low")))</f>
+        <v/>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="15">
       <c r="A67" s="16" t="inlineStr">
@@ -18995,7 +19307,7 @@
         <v/>
       </c>
       <c r="J67" s="22" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K67" s="22" t="n">
         <v>18</v>
@@ -19038,7 +19350,7 @@
       </c>
       <c r="Z67" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 10–35 min (top 35, passes 90-min cap), 8.3 km via Springvale Rd [https://www.google.com/maps/dir/Springvale%20VIC%203171/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 10–26 min. ED Monash Medical Centre Clayton 10–18 min. Price: SOI median $942,500 house (pricefinder, 1 Jul 2025–30 Jun 2026) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/b0b62daa-8691-4f3f-b21b-fc0a629845ff.pdf]; under-cap listings $700k–$790k. Indian grocery: India Town, 11b/310 Springvale Rd, 4 min (Google Business Profile). Hindu temple: Sankat Mochan Hanuman Mandir, 4 Margaret St, Oakleigh South, 10–20 min (Google, 602 reviews). Church: St Joseph's Catholic, cnr Buckingham Ave &amp; 7 St James Ave, 4 min (Google). ABS 2021: AQ 7.4%, AU 75.6%. Nature: none of real size (Wikipedia Springvale). ESTIMATE: train service (recall). NEEDS VERIFICATION: suitable property under cap; a 6-month SOI gives an outlier median $600k. Full sources: 'Community comparators — research (28 Oct 2026).md'.</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive peak (08:00), not used in J: typical 10–35 min (top 35, passes 90-min cap), 8.3 km via Springvale Rd [https://www.google.com/maps/dir/Springvale%20VIC%203171/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; GW drive 10:00 weekday (Wed 28 Oct 2026) typical 10–26 min, top 26 = J from 28 Oct 2026 (off-peak basis, closest checked figure to the Filters tab's "leave now") [https://www.google.com/maps/dir/Springvale%20VIC%203171/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793181600!3e0]. ED Monash Medical Centre Clayton 10–18 min. Price: SOI median $942,500 house (pricefinder, 1 Jul 2025–30 Jun 2026) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/b0b62daa-8691-4f3f-b21b-fc0a629845ff.pdf]; under-cap listings $700k–$790k. Indian grocery: India Town, 11b/310 Springvale Rd, 4 min (Google Business Profile). Hindu temple: Sankat Mochan Hanuman Mandir, 4 Margaret St, Oakleigh South, 10–20 min (Google, 602 reviews). Church: St Joseph's Catholic, cnr Buckingham Ave &amp; 7 St James Ave, 4 min (Google). ABS 2021: AQ 7.4%, AU 75.6%. Nature: none of real size (Wikipedia Springvale). ESTIMATE: train service (recall). NEEDS VERIFICATION: suitable property under cap; a 6-month SOI gives an outlier median $600k. Full sources: 'Community comparators — research (28 Oct 2026).md'.</t>
         </is>
       </c>
       <c r="AB67" s="22" t="inlineStr">
@@ -19178,7 +19490,7 @@
         <v/>
       </c>
       <c r="J68" s="22" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K68" s="22" t="n">
         <v>12</v>
@@ -19221,7 +19533,7 @@
       </c>
       <c r="Z68" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 16–40 min (top 40, passes), 11.4 km [https://www.google.com/maps/dir/Clayton%20South%20VIC%203169/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 14–35 min. ED Monash Medical Centre Clayton 8–12 min. Price: SOI median $985,000 house (pricefinder, Apr 2025–Mar 2026) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/daf40c18-47a7-4907-9f9a-1801cc782a35.pdf]; listing $1.00–1.08M and three comparables ~$1.0M. Indian grocery: Sarawan Spices, 335 Clayton Rd, Clayton, 5–8 min (Google Business Profile, confirmed operating); Little India Mart, 2/1310 Centre Rd, 4–6 min (Google). Hindu temple: Sankat Mochan Hanuman Mandir, Oakleigh South, 7–12 min (Google). Church: St Andrews Catholic, 76 Springs Rd, 5 min (Google). ABS 2021: AQ 14.9%, AU 67.1%. Nature: golf course and landfill; no named reserve (Victorian Places). ESTIMATE: Little India Mart's suburb (listing does not print it); train access (recall). NEEDS VERIFICATION: suitable property under cap.</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive peak (08:00), not used in J: typical 16–40 min (top 40, passes), 11.4 km [https://www.google.com/maps/dir/Clayton%20South%20VIC%203169/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; GW drive 10:00 weekday (Wed 28 Oct 2026) typical 14–35 min, top 35 = J from 28 Oct 2026 (off-peak basis, closest checked figure to the Filters tab's "leave now") [https://www.google.com/maps/dir/Clayton%20South%20VIC%203169/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793181600!3e0]. ED Monash Medical Centre Clayton 8–12 min. Price: SOI median $985,000 house (pricefinder, Apr 2025–Mar 2026) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/daf40c18-47a7-4907-9f9a-1801cc782a35.pdf]; listing $1.00–1.08M and three comparables ~$1.0M. Indian grocery: Sarawan Spices, 335 Clayton Rd, Clayton, 5–8 min (Google Business Profile, confirmed operating); Little India Mart, 2/1310 Centre Rd, 4–6 min (Google). Hindu temple: Sankat Mochan Hanuman Mandir, Oakleigh South, 7–12 min (Google). Church: St Andrews Catholic, 76 Springs Rd, 5 min (Google). ABS 2021: AQ 14.9%, AU 67.1%. Nature: golf course and landfill; no named reserve (Victorian Places). ESTIMATE: Little India Mart's suburb (listing does not print it); train access (recall). NEEDS VERIFICATION: suitable property under cap.</t>
         </is>
       </c>
       <c r="AB68" s="22" t="inlineStr">
@@ -19361,7 +19673,7 @@
         <v/>
       </c>
       <c r="J69" s="22" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="K69" s="22" t="n">
         <v>18</v>
@@ -19404,7 +19716,7 @@
       </c>
       <c r="Z69" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 18–30 min (top 30, passes), 21.0 km via M3 [https://www.google.com/maps/dir/Keysborough%20VIC%203173/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 18–24 min. ED Dandenong Hospital 12–18 min. Price: SOI median $975,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/ca8cd377-fe5e-42cd-a3d6-525992dc0a9d.pdf]; under-cap listing 45 Weston St $1.05–1.155M [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/7b6728e4-a512-4e2d-b761-4e7595257093.pdf]. Indian grocery: India at Home, Parkmore Shopping Centre, 4–6 min (Google). Hindu temple: Shri Shiva Vishnu Temple, 52 Boundary Rd, Carrum Downs, 14–20 min (Google, 6,483 reviews); gurdwara at 198-206 Perry Rd in suburb. Church: Resurrection Parish, 402 Corrigan Rd, 5–6 min (Google). ABS 2021: AQ 6.6%, AU 61.1%. Nature: market gardens to the south; no named reserve (Wikipedia). ESTIMATE: no train (recall). NEEDS VERIFICATION: suitable property under cap.</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive peak (08:00), not used in J: typical 18–30 min (top 30, passes), 21.0 km via M3 [https://www.google.com/maps/dir/Keysborough%20VIC%203173/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; GW drive 10:00 weekday (Wed 28 Oct 2026) typical 18–24 min, top 24 = J from 28 Oct 2026 (off-peak basis, closest checked figure to the Filters tab's "leave now") [https://www.google.com/maps/dir/Keysborough%20VIC%203173/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793181600!3e0]. ED Dandenong Hospital 12–18 min. Price: SOI median $975,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/ca8cd377-fe5e-42cd-a3d6-525992dc0a9d.pdf]; under-cap listing 45 Weston St $1.05–1.155M [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/7b6728e4-a512-4e2d-b761-4e7595257093.pdf]. Indian grocery: India at Home, Parkmore Shopping Centre, 4–6 min (Google). Hindu temple: Shri Shiva Vishnu Temple, 52 Boundary Rd, Carrum Downs, 14–20 min (Google, 6,483 reviews); gurdwara at 198-206 Perry Rd in suburb. Church: Resurrection Parish, 402 Corrigan Rd, 5–6 min (Google). ABS 2021: AQ 6.6%, AU 61.1%. Nature: market gardens to the south; no named reserve (Wikipedia). ESTIMATE: no train (recall). NEEDS VERIFICATION: suitable property under cap.</t>
         </is>
       </c>
       <c r="AB69" s="22" t="inlineStr">
@@ -19544,7 +19856,7 @@
         <v/>
       </c>
       <c r="J70" s="22" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="K70" s="22" t="n">
         <v>24</v>
@@ -19587,7 +19899,7 @@
       </c>
       <c r="Z70" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 35 min–1 hr 10 (top 70): passes the 90-min cap, but EXCEEDS A 60-MIN PREFERENCE if the family adopts one; 42.0 km via Thompsons Rd and M3 [https://www.google.com/maps/dir/Clyde%20North%20VIC%203978/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 28–50 min. ED Casey Hospital 12–24 min. Price: SOI median $752,932 house (PropTrack) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/a24be22a-1f37-4f59-820a-aeb288704b8c.pdf]; listing $790–860k and comparables ~$810k. Indian grocery: Wirsa Indian Groceries, 13/16 Selandra Blvd, 2 min (Google). Hindu temple: Shrinathji Haveli, 3-5 Princes Domain Dr, Hallam, 16–30 min (Google, confirmed operating). Church: St Thomas The Apostle Catholic, 5 Fiorelli Blvd, 4 min (Google; replaces the approximate GCatholic location). ABS 2021: AQ 18.2%, AU 53.6%. Nature: green-wedge farmland; regional park only proposed (Wikipedia). ESTIMATE: BAPS Mandir, 175-177 Smiths Ln, 8–12 min (listing does not print suburb); no train (recall). NEEDS VERIFICATION: suitable property under cap.</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: Diverse / lower-green. CHECKED (checked 28 Oct 2026 AEDT): GW drive peak (08:00), not used in J: typical 35 min–1 hr 10 (top 70): passes the 90-min cap, but EXCEEDS A 60-MIN PREFERENCE if the family adopts one; 42.0 km via Thompsons Rd and M3 [https://www.google.com/maps/dir/Clyde%20North%20VIC%203978/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; GW drive 10:00 weekday (Wed 28 Oct 2026) typical 28–50 min, top 50 = J from 28 Oct 2026 (off-peak basis, closest checked figure to the Filters tab's "leave now") [https://www.google.com/maps/dir/Clyde%20North%20VIC%203978/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793181600!3e0]. ED Casey Hospital 12–24 min. Price: SOI median $752,932 house (PropTrack) [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/a24be22a-1f37-4f59-820a-aeb288704b8c.pdf]; listing $790–860k and comparables ~$810k. Indian grocery: Wirsa Indian Groceries, 13/16 Selandra Blvd, 2 min (Google). Hindu temple: Shrinathji Haveli, 3-5 Princes Domain Dr, Hallam, 16–30 min (Google, confirmed operating). Church: St Thomas The Apostle Catholic, 5 Fiorelli Blvd, 4 min (Google; replaces the approximate GCatholic location). ABS 2021: AQ 18.2%, AU 53.6%. Nature: green-wedge farmland; regional park only proposed (Wikipedia). ESTIMATE: BAPS Mandir, 175-177 Smiths Ln, 8–12 min (listing does not print suburb); no train (recall). NEEDS VERIFICATION: suitable property under cap.</t>
         </is>
       </c>
       <c r="AB70" s="22" t="inlineStr">
@@ -19727,7 +20039,7 @@
         <v/>
       </c>
       <c r="J71" s="22" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K71" s="22" t="n">
         <v>12</v>
@@ -19770,7 +20082,7 @@
       </c>
       <c r="Z71" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH (nature and community both realistic weekly). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 18–35 min (top 35, passes), 18.6 km via M3 [https://www.google.com/maps/dir/Endeavour%20Hills%20VIC%203802/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 16–26 min. ED Dandenong Hospital 7–12 min. Price: SOI median $857,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/8fc3f19f-6ab3-47ea-b801-9bbd2d72885f.pdf]; listing $760–820k. Indian grocery: India At Home – Dandenong, Dandenong Plaza, 49 McCrae St, 8–12 min (Google). Hindu temple: Shrinathji Haveli, Hallam, 8–14 min (Google, confirmed operating). Church: St Paul Apostle Catholic, 5 William Hovell Dr, 2 min (Google). Nature: Casuarina Forest / James Alexander Reserve 1.1 km, 3 min; Churchill National Park 8–10 min; Lysterfield Park 12 min. ABS 2021: AQ 4.6%, AU 51.3%. ESTIMATE: reserve walkable from central/northern streets (distance from suburb centre only); no train (recall). NEEDS VERIFICATION: Endeavour Spices (not found on Google Maps; not counted); Shri Sanatan Dharam Society, 126/128 Hallam N Rd (listing has no hours; 4–6 min if open); suitable property under cap. | UPDATE 28 Oct 2026: Endeavour Spices still NEEDS VERIFICATION (no Google Maps listing; web search found no listing, website or directory entry beyond the earlier onlymelbourne record); not counted as community access. Shri Sanatan Dharam Society: opening hours NEEDS VERIFICATION (Google listing shows none; web search found none). ACNC-linked register lists the society at Narre Warren North VIC 3804, so the 126/128 Hallam N Rd site may be in Narre Warren North, not Endeavour Hills; the 4–6 min drive (geocoded with "Endeavour Hills") is therefore an ESTIMATE. Source: https://civicgraph.app/charities/44400281254</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH (nature and community both realistic weekly). CHECKED (checked 28 Oct 2026 AEDT): GW drive peak (08:00), not used in J: typical 18–35 min (top 35, passes), 18.6 km via M3 [https://www.google.com/maps/dir/Endeavour%20Hills%20VIC%203802/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; GW drive 10:00 weekday (Wed 28 Oct 2026) typical 16–26 min, top 26 = J from 28 Oct 2026 (off-peak basis, closest checked figure to the Filters tab's "leave now") [https://www.google.com/maps/dir/Endeavour%20Hills%20VIC%203802/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793181600!3e0]. ED Dandenong Hospital 7–12 min. Price: SOI median $857,000 house [https://s3-ap-southeast-2.amazonaws.com/zenu/soi/8fc3f19f-6ab3-47ea-b801-9bbd2d72885f.pdf]; listing $760–820k. Indian grocery: India At Home – Dandenong, Dandenong Plaza, 49 McCrae St, 8–12 min (Google). Hindu temple: Shrinathji Haveli, Hallam, 8–14 min (Google, confirmed operating). Church: St Paul Apostle Catholic, 5 William Hovell Dr, 2 min (Google). Nature: Casuarina Forest / James Alexander Reserve 1.1 km, 3 min; Churchill National Park 8–10 min; Lysterfield Park 12 min. ABS 2021: AQ 4.6%, AU 51.3%. ESTIMATE: reserve walkable from central/northern streets (distance from suburb centre only); no train (recall). NEEDS VERIFICATION: Endeavour Spices (not found on Google Maps; not counted); Shri Sanatan Dharam Society, 126/128 Hallam N Rd (listing has no hours; 4–6 min if open); suitable property under cap. | UPDATE 28 Oct 2026: Endeavour Spices still NEEDS VERIFICATION (no Google Maps listing; web search found no listing, website or directory entry beyond the earlier onlymelbourne record); not counted as community access. Shri Sanatan Dharam Society: opening hours NEEDS VERIFICATION (Google listing shows none; web search found none). ACNC-linked register lists the society at Narre Warren North VIC 3804, so the 126/128 Hallam N Rd site may be in Narre Warren North, not Endeavour Hills; the 4–6 min drive (geocoded with "Endeavour Hills") is therefore an ESTIMATE. Source: https://civicgraph.app/charities/44400281254</t>
         </is>
       </c>
       <c r="AB71" s="22" t="inlineStr">
@@ -19953,7 +20265,7 @@
       </c>
       <c r="Z72" s="16" t="inlineStr">
         <is>
-          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH, with caveat: community access is lighter (Medium band; nearest Hindu temple 10–20 min). CHECKED (checked 28 Oct 2026 AEDT): GW drive 08:00 typical 4–12 min (top 12, passes), 2.6 km [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; 10:00 7–12 min. ED Dandenong Hospital 12–18 min. Price: SOI median $1,475,000 house (Property Data) [https://s3-ap-southeast-2.amazonaws.com/attach-property-clientvault-com/3868/11973436/S-13799066/1782296638-118760-9-Sunnybrook-WheelersHillSOI220626.pdf]. Indian grocery: The Heritage Spices, G15/580 Ferntree Gully Rd, 6–9 min (Google). Hindu temple: Shree Swaminarayan Temple, 69 Wadhurst Dr, Boronia, 10–20 min (Google, 253 reviews); Sankat Mochan 14–28; Vakrathunda 16–35. Church: St Justin's Catholic, 48 Whalley Dr, 4 min (Google). Nature: Jells Park (~127 ha) 2.6 km, 6 min. ABS 2021: AQ 4.1%, AU 46.0%. HARD FILTER: Pass on median only; suitable-property verification outstanding. ESTIMATE: budget (under-cap listings $1.28–1.38M and $1.32M from search text only); Jells Park walkable only from eastern streets; no train (recall). NEEDS VERIFICATION: open an under-cap SOI; suitable property under cap. | UPDATE 28 Oct 2026: budget evidence changed ESTIMATE -&gt; CHECKED. Jellis Craig Wheelers Hill Suburb Report Sep 2026 (data to 6 Sep 2026) lists houses sold under $1.5M, e.g. 8 Bottlebrush Ct 4-bed house $1,215,000 (27 Aug 2026), 4 Locum Ct 4-bed $1,224,500 (8 Aug 2026), 81 Cootamundra Dr 3-bed $1,130,000 (18 Jul 2026); report median $1.46M [https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf]. Agency sold-results report, not an SOI. Suitable-property verification still outstanding. | 28 Oct 2026: family accepted this report as Checked budget evidence. It shows recent sold houses under the cap; it does NOT verify that a specific suitable downsizing/family home is available. L updated to "filters met; suitable-property verification outstanding".</t>
+          <t>COMMUNITY COMPARATOR added 28 Oct 2026 (display-only; not ranked; no judgement scores). Corner: POTENTIAL BOTH, with caveat: community access is lighter (Medium band; nearest Hindu temple 10–20 min). CHECKED (checked 28 Oct 2026 AEDT): GW drive peak (08:00), not used in J: typical 4–12 min (top 12, passes), 2.6 km [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793174400!3e0]; GW drive 10:00 weekday (Wed 28 Oct 2026) typical 7–12 min, top 12 = J from 28 Oct 2026 (off-peak basis, closest checked figure to the Filters tab's "leave now") [https://www.google.com/maps/dir/Wheelers%20Hill%20VIC%203150/Glen%20Waverley%20VIC%203150/data=!4m6!4m5!2m3!6e0!7e2!8j1793181600!3e0]. ED Dandenong Hospital 12–18 min. Price: SOI median $1,475,000 house (Property Data) [https://s3-ap-southeast-2.amazonaws.com/attach-property-clientvault-com/3868/11973436/S-13799066/1782296638-118760-9-Sunnybrook-WheelersHillSOI220626.pdf]. Indian grocery: The Heritage Spices, G15/580 Ferntree Gully Rd, 6–9 min (Google). Hindu temple: Shree Swaminarayan Temple, 69 Wadhurst Dr, Boronia, 10–20 min (Google, 253 reviews); Sankat Mochan 14–28; Vakrathunda 16–35. Church: St Justin's Catholic, 48 Whalley Dr, 4 min (Google). Nature: Jells Park (~127 ha) 2.6 km, 6 min. ABS 2021: AQ 4.1%, AU 46.0%. HARD FILTER: Pass on median only; suitable-property verification outstanding. ESTIMATE: budget (under-cap listings $1.28–1.38M and $1.32M from search text only); Jells Park walkable only from eastern streets; no train (recall). NEEDS VERIFICATION: open an under-cap SOI; suitable property under cap. | UPDATE 28 Oct 2026: budget evidence changed ESTIMATE -&gt; CHECKED. Jellis Craig Wheelers Hill Suburb Report Sep 2026 (data to 6 Sep 2026) lists houses sold under $1.5M, e.g. 8 Bottlebrush Ct 4-bed house $1,215,000 (27 Aug 2026), 4 Locum Ct 4-bed $1,224,500 (8 Aug 2026), 81 Cootamundra Dr 3-bed $1,130,000 (18 Jul 2026); report median $1.46M [https://helpers.jelliscraig.com.au/suburbreportsdownloads/Wheelers_Hill_Suburb_Reports_Sep_2026.pdf]. Agency sold-results report, not an SOI. Suitable-property verification still outstanding. | 28 Oct 2026: family accepted this report as Checked budget evidence. It shows recent sold houses under the cap; it does NOT verify that a specific suitable downsizing/family home is available. L updated to "filters met; suitable-property verification outstanding".</t>
         </is>
       </c>
       <c r="AB72" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Workbook: Glen Waverley house median from realestate.com.au
SuburbScorecard row 7: G7 $1,763,500 -> $1,675,000; H7 442 sales, all
bedrooms, 12 months; I7 1,775,500 (G7 x 1.06, plain value as before);
Z7 source and cross-checks (REIV $1.75m via 5 Northam St SOI, Jellis
Craig $1.68m, 4-bed median $1,603,000); AH7 29 Oct 2026; AJ7 note.
Recalc test pre and post: 0 errors, X numeric 53, Y ranked 51; only
these six cells changed; no score or rank moved. Pre-change copy in
Archive.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013uWqduC6UkfLJbJZE4E3Dw
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -7595,15 +7595,15 @@
         </is>
       </c>
       <c r="G7" s="18" t="n">
-        <v>1763500</v>
+        <v>1675000</v>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>Sale median, rolling 12m (454 sales); unit $930k</t>
+          <t>Sale median, all bedrooms, 12 months (442 sales); unit $930k</t>
         </is>
       </c>
       <c r="I7" s="18" t="n">
-        <v>1869310</v>
+        <v>1775500</v>
       </c>
       <c r="J7" s="19" t="n">
         <v>0</v>
@@ -7643,7 +7643,7 @@
       </c>
       <c r="Z7" s="18" t="inlineStr">
         <is>
-          <t>ABS 2021: 58.7% overseas-born, 63.0% non-Eng HH. Baseline benchmark for family proximity.</t>
+          <t>ABS 2021: 58.7% overseas-born, 63.0% non-Eng HH. Baseline benchmark for family proximity. C 29 Oct 2026: G7 $1,675,000 and H7 442 sales from the realestate.com.au Glen Waverley suburb profile (house median, all bedrooms, past 12 months; figure read by the user 29 Oct 2026), CHECKED. Replaces $1,763,500 (454 sales; no source named). Cross-checks: REIV $1,750,000 (1 Jul 2025-30 Jun 2026, via the 5 Northam St Statement of Information); Jellis Craig $1.68m (rolling 12 months, read 28 Oct 2026); realestate.com.au 4-bed median $1,603,000 (Oct 2025-Sep 2026, 175 sales).</t>
         </is>
       </c>
       <c r="AA7" s="16" t="inlineStr">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="AH7" s="22" t="inlineStr">
         <is>
-          <t>26 Oct 2026</t>
+          <t>29 Oct 2026</t>
         </is>
       </c>
       <c r="AI7" s="22" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="AJ7" s="22" t="inlineStr">
         <is>
-          <t>House median $1.76M (454 sales) exceeds $1.5M cap; unit median $930k. Awaiting documented search for suitable single-level homes/units under $1.5M.</t>
+          <t>House median $1.68M (442 sales, realestate.com.au) exceeds $1.5M cap; unit median $930k. Awaiting documented search for suitable single-level homes/units under $1.5M.</t>
         </is>
       </c>
       <c r="AK7" s="22" t="inlineStr">

</xml_diff>

<commit_message>
N2: rounds 5–7 workbook intake (empty structure); recalc and diff passed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StartHere" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RawResponses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CleanedAnswers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filters" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PriorityWeights" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForcedChoiceCorrections" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SuburbScorecard" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listings" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DiscussionSummary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="StartHere" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="RawResponses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CleanedAnswers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Filters" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PriorityWeights" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ForcedChoiceCorrections" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SuburbScorecard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Listings" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DiscussionSummary" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Listings'!$A$1:$U$33</definedName>
@@ -826,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="15">
@@ -1354,6 +1354,171 @@
       <c r="B38" s="34" t="inlineStr">
         <is>
           <t>The viewing shortlist includes at least 2 Community comparators, at least 1 nature-first anchor, and at least 1 verified Potential both suburb. Community comparators are not included for diversity figures alone; they must meet the purchase-price cap, verified Glen Waverley travel limit, and public 24-hour ED requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Rounds 5–6 answers (display-only; added 30 Oct 2026; no pass count until N4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>GW firm limit (min)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>GW preferred (min)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ED firm limit (min)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>R5.7 church denomination</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Answer check</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mum</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>CleanedAnswers!B59</f>
+        <v/>
+      </c>
+      <c r="C42">
+        <f>CleanedAnswers!B60</f>
+        <v/>
+      </c>
+      <c r="D42">
+        <f>IF(CleanedAnswers!E44="E","No limit",CleanedAnswers!B61)</f>
+        <v/>
+      </c>
+      <c r="E42">
+        <f>CleanedAnswers!B47</f>
+        <v/>
+      </c>
+      <c r="F42">
+        <f>CleanedAnswers!B71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Dad</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>CleanedAnswers!C59</f>
+        <v/>
+      </c>
+      <c r="C43">
+        <f>CleanedAnswers!C60</f>
+        <v/>
+      </c>
+      <c r="D43">
+        <f>IF(CleanedAnswers!F44="E","No limit",CleanedAnswers!C61)</f>
+        <v/>
+      </c>
+      <c r="E43">
+        <f>CleanedAnswers!C47</f>
+        <v/>
+      </c>
+      <c r="F43">
+        <f>CleanedAnswers!C71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Me</t>
+        </is>
+      </c>
+      <c r="B44">
+        <f>CleanedAnswers!D59</f>
+        <v/>
+      </c>
+      <c r="C44">
+        <f>CleanedAnswers!D60</f>
+        <v/>
+      </c>
+      <c r="D44">
+        <f>IF(CleanedAnswers!G44="E","No limit",CleanedAnswers!D61)</f>
+        <v/>
+      </c>
+      <c r="E44">
+        <f>CleanedAnswers!D47</f>
+        <v/>
+      </c>
+      <c r="F44">
+        <f>CleanedAnswers!D71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Household (strictest)</t>
+        </is>
+      </c>
+      <c r="B45">
+        <f>CleanedAnswers!E59</f>
+        <v/>
+      </c>
+      <c r="C45">
+        <f>CleanedAnswers!E60</f>
+        <v/>
+      </c>
+      <c r="D45">
+        <f>CleanedAnswers!E61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Separation (household floor / ceiling / check)</t>
+        </is>
+      </c>
+      <c r="B47">
+        <f>CleanedAnswers!E64</f>
+        <v/>
+      </c>
+      <c r="C47">
+        <f>CleanedAnswers!E65</f>
+        <v/>
+      </c>
+      <c r="D47">
+        <f>CleanedAnswers!F65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Household cells stay blank until all three have answered. GW preferred (R5.3) is a preference only: never a filter or score. Filters change only at G2, with approval.</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="15">
@@ -1669,6 +1834,215 @@
         <v>0</v>
       </c>
       <c r="C25" s="18" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Property fit parameters (rounds 5–6)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Value (approved)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Survey reference</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>B blank until approved (G5; B38/B39 at G3). Intake changes no fit result</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Separation floor (1–4)</t>
+        </is>
+      </c>
+      <c r="C28">
+        <f>CleanedAnswers!E64</f>
+        <v/>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>R6.1, household MAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Separation ceiling (1–4)</t>
+        </is>
+      </c>
+      <c r="C29">
+        <f>CleanedAnswers!E65</f>
+        <v/>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>R6.2, household MIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Separation importance (3 Essential / 2 Important / 1 Nice to have)</t>
+        </is>
+      </c>
+      <c r="C30">
+        <f>CleanedAnswers!E66</f>
+        <v/>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>R6.3, household MAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Mobility must-have (0–3)</t>
+        </is>
+      </c>
+      <c r="C31">
+        <f>CleanedAnswers!E67</f>
+        <v/>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>R6.4, household MAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Garden preferred band (1–4)</t>
+        </is>
+      </c>
+      <c r="C32">
+        <f>CleanedAnswers!E68</f>
+        <v/>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>R6.5a, household MEDIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Garden capacity band (1–4)</t>
+        </is>
+      </c>
+      <c r="C33">
+        <f>CleanedAnswers!E69</f>
+        <v/>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>R6.5b, household MEDIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Front-door access (1–4)</t>
+        </is>
+      </c>
+      <c r="C34">
+        <f>CleanedAnswers!E70</f>
+        <v/>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>R6.6, household MIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Land-size band: courtyard (m², up to)</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>400</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Land-size band: small garden (m², up to)</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>650</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Land-size band: medium garden (m², up to)</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Estimate; above = large</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>M scale (min)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>90</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Proposed; B set at G3 (M/O decoupling)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>O scale (min)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>90</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Proposed; B set at G3 (M/O decoupling)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1686,7 +2060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN15"/>
+  <dimension ref="A1:BE15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="39" max="39"/>
@@ -1892,6 +2266,91 @@
       <c r="AN1" s="16" t="inlineStr">
         <is>
           <t>[Q13d] Green village vs multicultural neighbourhood (reference-only)</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>[R5.1] Time in Glen Waverley in person</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>[R5.2] GW drive: firm limit</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>[R5.3] GW drive: preferred</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>[R5.4] ED drive: firm limit</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>[R5.5] Community place used most</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>[R5.6] Community place: longest regular drive</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>[R5.7] Church: particular denomination</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>[R5 Notes]</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>[R6.1] Separation: least that would work</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>[R6.2] Separation: most that still feels like one household</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>[R6.3] Separation: importance of having it already</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>[R6.4] Mobility: must-have in 10-15 years</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>[R6.5a] Outdoor space wanted</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>[R6.5b] Garden upkeep capacity</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>[R6.6] Supermarket and GP from the front door</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>[R6.7] Privacy: one thing that matters most</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>[R6 Notes]</t>
         </is>
       </c>
     </row>
@@ -3821,7 +4280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="15">
@@ -4913,6 +5372,807 @@
       </c>
       <c r="G40" s="16">
         <f>LEFT(D40,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>[R5.1] Time in Glen Waverley in person</t>
+        </is>
+      </c>
+      <c r="B41">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C41">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D41">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E41">
+        <f>LEFT(B41,1)</f>
+        <v/>
+      </c>
+      <c r="F41">
+        <f>LEFT(C41,1)</f>
+        <v/>
+      </c>
+      <c r="G41">
+        <f>LEFT(D41,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>[R5.2] GW drive: firm limit</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C42">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D42">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E42">
+        <f>LEFT(B42,1)</f>
+        <v/>
+      </c>
+      <c r="F42">
+        <f>LEFT(C42,1)</f>
+        <v/>
+      </c>
+      <c r="G42">
+        <f>LEFT(D42,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>[R5.3] GW drive: preferred</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C43">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D43">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E43">
+        <f>LEFT(B43,1)</f>
+        <v/>
+      </c>
+      <c r="F43">
+        <f>LEFT(C43,1)</f>
+        <v/>
+      </c>
+      <c r="G43">
+        <f>LEFT(D43,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>[R5.4] ED drive: firm limit</t>
+        </is>
+      </c>
+      <c r="B44">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C44">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D44">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E44">
+        <f>LEFT(B44,1)</f>
+        <v/>
+      </c>
+      <c r="F44">
+        <f>LEFT(C44,1)</f>
+        <v/>
+      </c>
+      <c r="G44">
+        <f>LEFT(D44,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>[R5.5] Community place used most</t>
+        </is>
+      </c>
+      <c r="B45">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C45">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D45">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E45">
+        <f>LEFT(B45,1)</f>
+        <v/>
+      </c>
+      <c r="F45">
+        <f>LEFT(C45,1)</f>
+        <v/>
+      </c>
+      <c r="G45">
+        <f>LEFT(D45,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>[R5.6] Community place: longest regular drive</t>
+        </is>
+      </c>
+      <c r="B46">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C46">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D46">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E46">
+        <f>LEFT(B46,1)</f>
+        <v/>
+      </c>
+      <c r="F46">
+        <f>LEFT(C46,1)</f>
+        <v/>
+      </c>
+      <c r="G46">
+        <f>LEFT(D46,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>[R5.7] Church: particular denomination</t>
+        </is>
+      </c>
+      <c r="B47">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C47">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D47">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E47">
+        <f>LEFT(B47,1)</f>
+        <v/>
+      </c>
+      <c r="F47">
+        <f>LEFT(C47,1)</f>
+        <v/>
+      </c>
+      <c r="G47">
+        <f>LEFT(D47,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>[R5 Notes]</t>
+        </is>
+      </c>
+      <c r="B48">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C48">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D48">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>[R6.1] Separation: least that would work</t>
+        </is>
+      </c>
+      <c r="B49">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C49">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D49">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E49">
+        <f>LEFT(B49,1)</f>
+        <v/>
+      </c>
+      <c r="F49">
+        <f>LEFT(C49,1)</f>
+        <v/>
+      </c>
+      <c r="G49">
+        <f>LEFT(D49,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>[R6.2] Separation: most that still feels like one household</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C50">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D50">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E50">
+        <f>LEFT(B50,1)</f>
+        <v/>
+      </c>
+      <c r="F50">
+        <f>LEFT(C50,1)</f>
+        <v/>
+      </c>
+      <c r="G50">
+        <f>LEFT(D50,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>[R6.3] Separation: importance of having it already</t>
+        </is>
+      </c>
+      <c r="B51">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C51">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D51">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E51">
+        <f>LEFT(B51,1)</f>
+        <v/>
+      </c>
+      <c r="F51">
+        <f>LEFT(C51,1)</f>
+        <v/>
+      </c>
+      <c r="G51">
+        <f>LEFT(D51,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>[R6.4] Mobility: must-have in 10-15 years</t>
+        </is>
+      </c>
+      <c r="B52">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C52">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D52">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E52">
+        <f>LEFT(B52,1)</f>
+        <v/>
+      </c>
+      <c r="F52">
+        <f>LEFT(C52,1)</f>
+        <v/>
+      </c>
+      <c r="G52">
+        <f>LEFT(D52,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>[R6.5a] Outdoor space wanted</t>
+        </is>
+      </c>
+      <c r="B53">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C53">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D53">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E53">
+        <f>LEFT(B53,1)</f>
+        <v/>
+      </c>
+      <c r="F53">
+        <f>LEFT(C53,1)</f>
+        <v/>
+      </c>
+      <c r="G53">
+        <f>LEFT(D53,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>[R6.5b] Garden upkeep capacity</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C54">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D54">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E54">
+        <f>LEFT(B54,1)</f>
+        <v/>
+      </c>
+      <c r="F54">
+        <f>LEFT(C54,1)</f>
+        <v/>
+      </c>
+      <c r="G54">
+        <f>LEFT(D54,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>[R6.6] Supermarket and GP from the front door</t>
+        </is>
+      </c>
+      <c r="B55">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C55">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D55">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E55">
+        <f>LEFT(B55,1)</f>
+        <v/>
+      </c>
+      <c r="F55">
+        <f>LEFT(C55,1)</f>
+        <v/>
+      </c>
+      <c r="G55">
+        <f>LEFT(D55,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>[R6.7] Privacy: one thing that matters most</t>
+        </is>
+      </c>
+      <c r="B56">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C56">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D56">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E56">
+        <f>LEFT(B56,1)</f>
+        <v/>
+      </c>
+      <c r="F56">
+        <f>LEFT(C56,1)</f>
+        <v/>
+      </c>
+      <c r="G56">
+        <f>LEFT(D56,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>[R6 Notes]</t>
+        </is>
+      </c>
+      <c r="B57">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="C57">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D57">
+        <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Derived (B–D per person; E household)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>GW firm limit (min)</t>
+        </is>
+      </c>
+      <c r="B59">
+        <f>IFERROR(IF(E42="","",CHOOSE(FIND(E42,"ABCDE"),25,35,45,60,90)),"")</f>
+        <v/>
+      </c>
+      <c r="C59">
+        <f>IFERROR(IF(F42="","",CHOOSE(FIND(F42,"ABCDE"),25,35,45,60,90)),"")</f>
+        <v/>
+      </c>
+      <c r="D59">
+        <f>IFERROR(IF(G42="","",CHOOSE(FIND(G42,"ABCDE"),25,35,45,60,90)),"")</f>
+        <v/>
+      </c>
+      <c r="E59">
+        <f>IF(COUNTIF(E42:G42,"?")&lt;3,"",MIN(B59:D59))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>GW preferred (min)</t>
+        </is>
+      </c>
+      <c r="B60">
+        <f>IFERROR(IF(E43="","",CHOOSE(FIND(E43,"ABCDE"),25,35,45,60,90)),"")</f>
+        <v/>
+      </c>
+      <c r="C60">
+        <f>IFERROR(IF(F43="","",CHOOSE(FIND(F43,"ABCDE"),25,35,45,60,90)),"")</f>
+        <v/>
+      </c>
+      <c r="D60">
+        <f>IFERROR(IF(G43="","",CHOOSE(FIND(G43,"ABCDE"),25,35,45,60,90)),"")</f>
+        <v/>
+      </c>
+      <c r="E60">
+        <f>IF(COUNTIF(E43:G43,"?")&lt;3,"",MIN(B60:D60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ED firm limit (min; blank = no limit)</t>
+        </is>
+      </c>
+      <c r="B61">
+        <f>IFERROR(IF(E44="","",CHOOSE(FIND(E44,"ABCDE"),15,20,30,45,"")),"")</f>
+        <v/>
+      </c>
+      <c r="C61">
+        <f>IFERROR(IF(F44="","",CHOOSE(FIND(F44,"ABCDE"),15,20,30,45,"")),"")</f>
+        <v/>
+      </c>
+      <c r="D61">
+        <f>IFERROR(IF(G44="","",CHOOSE(FIND(G44,"ABCDE"),15,20,30,45,"")),"")</f>
+        <v/>
+      </c>
+      <c r="E61">
+        <f>IF(COUNTIF(E44:G44,"?")&lt;3,"",IF(COUNT(B61:D61)=0,"No cap",MIN(B61:D61)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Community place index (grocery 1, temple 2, church 3, none 0)</t>
+        </is>
+      </c>
+      <c r="B62">
+        <f>IFERROR(IF(E45="","",CHOOSE(FIND(E45,"ABCDE"),1,2,3,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C62">
+        <f>IFERROR(IF(F45="","",CHOOSE(FIND(F45,"ABCDE"),1,2,3,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D62">
+        <f>IFERROR(IF(G45="","",CHOOSE(FIND(G45,"ABCDE"),1,2,3,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Community drive limit (min)</t>
+        </is>
+      </c>
+      <c r="B63">
+        <f>IFERROR(IF(E46="","",CHOOSE(FIND(E46,"ABCDE"),10,20,30,45,"")),"")</f>
+        <v/>
+      </c>
+      <c r="C63">
+        <f>IFERROR(IF(F46="","",CHOOSE(FIND(F46,"ABCDE"),10,20,30,45,"")),"")</f>
+        <v/>
+      </c>
+      <c r="D63">
+        <f>IFERROR(IF(G46="","",CHOOSE(FIND(G46,"ABCDE"),10,20,30,45,"")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Separation floor (1–4)</t>
+        </is>
+      </c>
+      <c r="B64">
+        <f>IFERROR(IF(E49="","",CHOOSE(FIND(E49,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="C64">
+        <f>IFERROR(IF(F49="","",CHOOSE(FIND(F49,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="D64">
+        <f>IFERROR(IF(G49="","",CHOOSE(FIND(G49,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="E64">
+        <f>IF(COUNTIF(E49:G49,"?")&lt;3,"",MAX(B64:D64))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Separation ceiling (1–4)</t>
+        </is>
+      </c>
+      <c r="B65">
+        <f>IFERROR(IF(E50="","",CHOOSE(FIND(E50,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="C65">
+        <f>IFERROR(IF(F50="","",CHOOSE(FIND(F50,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="D65">
+        <f>IFERROR(IF(G50="","",CHOOSE(FIND(G50,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="E65">
+        <f>IF(COUNTIF(E50:G50,"?")&lt;3,"",MIN(B65:D65))</f>
+        <v/>
+      </c>
+      <c r="F65">
+        <f>IF(OR(E64="",E65=""),"",IF(E64&gt;E65,"CONFLICT: no layout suits everyone","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Separation importance (3 Essential, 2 Important, 1 Nice to have)</t>
+        </is>
+      </c>
+      <c r="B66">
+        <f>IFERROR(IF(E51="","",CHOOSE(FIND(E51,"ABCDE"),3,2,1)),"")</f>
+        <v/>
+      </c>
+      <c r="C66">
+        <f>IFERROR(IF(F51="","",CHOOSE(FIND(F51,"ABCDE"),3,2,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D66">
+        <f>IFERROR(IF(G51="","",CHOOSE(FIND(G51,"ABCDE"),3,2,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E66">
+        <f>IF(COUNTIF(E51:G51,"?")&lt;3,"",MAX(B66:D66))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Mobility must-have (0–3)</t>
+        </is>
+      </c>
+      <c r="B67">
+        <f>IFERROR(IF(E52="","",CHOOSE(FIND(E52,"ABCDE"),0,1,2,3)),"")</f>
+        <v/>
+      </c>
+      <c r="C67">
+        <f>IFERROR(IF(F52="","",CHOOSE(FIND(F52,"ABCDE"),0,1,2,3)),"")</f>
+        <v/>
+      </c>
+      <c r="D67">
+        <f>IFERROR(IF(G52="","",CHOOSE(FIND(G52,"ABCDE"),0,1,2,3)),"")</f>
+        <v/>
+      </c>
+      <c r="E67">
+        <f>IF(COUNTIF(E52:G52,"?")&lt;3,"",MAX(B67:D67))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Garden preferred band (1–4)</t>
+        </is>
+      </c>
+      <c r="B68">
+        <f>IFERROR(IF(E53="","",CHOOSE(FIND(E53,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="C68">
+        <f>IFERROR(IF(F53="","",CHOOSE(FIND(F53,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="D68">
+        <f>IFERROR(IF(G53="","",CHOOSE(FIND(G53,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="E68">
+        <f>IF(COUNTIF(E53:G53,"?")&lt;3,"",MEDIAN(B68:D68))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Garden capacity band (1–4)</t>
+        </is>
+      </c>
+      <c r="B69">
+        <f>IFERROR(IF(E54="","",CHOOSE(FIND(E54,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="C69">
+        <f>IFERROR(IF(F54="","",CHOOSE(FIND(F54,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="D69">
+        <f>IFERROR(IF(G54="","",CHOOSE(FIND(G54,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="E69">
+        <f>IF(COUNTIF(E54:G54,"?")&lt;3,"",MEDIAN(B69:D69))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Front-door access (1 must walk … 4 drive up to 20 min)</t>
+        </is>
+      </c>
+      <c r="B70">
+        <f>IFERROR(IF(E55="","",CHOOSE(FIND(E55,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="C70">
+        <f>IFERROR(IF(F55="","",CHOOSE(FIND(F55,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="D70">
+        <f>IFERROR(IF(G55="","",CHOOSE(FIND(G55,"ABCDE"),1,2,3,4)),"")</f>
+        <v/>
+      </c>
+      <c r="E70">
+        <f>IF(COUNTIF(E55:G55,"?")&lt;3,"",MIN(B70:D70))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Validation (R6.2 ≥ R6.1; R5.5/R5.6 and R5.5/R5.7 consistent)</t>
+        </is>
+      </c>
+      <c r="B71">
+        <f>IFERROR(IF(E45&amp;E46&amp;E47&amp;E49&amp;E50="","",IF(AND(LEN(E45&amp;E46&amp;E47&amp;E49&amp;E50)=5,E50&gt;=E49,IF(E45="D",E46="E",E46&lt;&gt;"E"),IF(E45="C",E47&lt;&gt;"C",E47="C")),"OK","Check")),"Check")</f>
+        <v/>
+      </c>
+      <c r="C71">
+        <f>IFERROR(IF(F45&amp;F46&amp;F47&amp;F49&amp;F50="","",IF(AND(LEN(F45&amp;F46&amp;F47&amp;F49&amp;F50)=5,F50&gt;=F49,IF(F45="D",F46="E",F46&lt;&gt;"E"),IF(F45="C",F47&lt;&gt;"C",F47="C")),"OK","Check")),"Check")</f>
+        <v/>
+      </c>
+      <c r="D71">
+        <f>IFERROR(IF(G45&amp;G46&amp;G47&amp;G49&amp;G50="","",IF(AND(LEN(G45&amp;G46&amp;G47&amp;G49&amp;G50)=5,G50&gt;=G49,IF(G45="D",G46="E",G46&lt;&gt;"E"),IF(G45="C",G47&lt;&gt;"C",G47="C")),"OK","Check")),"Check")</f>
         <v/>
       </c>
     </row>
@@ -6306,7 +7566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AX90"/>
+  <dimension ref="A1:BF90"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="15" min="37" max="37"/>
@@ -6576,6 +7836,31 @@
           <t>Community comparison band (display-only)</t>
         </is>
       </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>Drive to nearest Indian grocery (min; 10:00 weekday, top of range)</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>Drive to nearest Hindu temple (min; 10:00 weekday, top of range)</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>Drive to nearest church (min; 10:00 weekday, top of range)</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>Community drive basis and evidence (Checked / Estimate / Needs verification)</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>Slope/stairs risk (display-only, Estimate; feeds nothing)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" s="15">
       <c r="A2" s="18" t="inlineStr">
@@ -20828,7 +22113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:W33"/>
+  <dimension ref="A1:AG33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="22" min="1" max="1"/>
@@ -20967,6 +22252,56 @@
           <t>Source: realestate.com.au collection 'Parents.', read from browser 27 Oct 2026 (copied from the Google Sheet version of this tab). A–F, H–O, U are pasted values; G and P–T are formulas. Prices are agent guides (purchase price, before costs), compared with Filters!B2 purchase cap. Drive times and train are suburb-level from SuburbScorecard, not per address. Inspection times go stale after 31 Oct. Refresh = re-read the collection and overwrite pasted columns only.</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Separation tier now (A–D / Unknown; R6.1 ladder, from floorplan)</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Mobility level met now (0–3 / Unknown; R6.4 ladder)</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Mobility gap (None / Minor works / Major / Unknown)</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Garden band 1–4 (formula: K vs Settings B35:B37; photos override, note in AF)</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Walk to supermarket (min; basis named)</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Walk to GP (min; basis named)</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Noise flag (Highway / Rail / Flight path / None)</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Overlay (Bushfire / Flood / Heritage / None; task B3)</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Evidence basis + date (Floorplan seen / Photos only / Not checked)</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Home fit (formula: first matching rule, design doc section 5)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="15">
       <c r="A2" s="22" t="n">
@@ -21054,6 +22389,14 @@
           <t>https://www.realestate.com.au/property-house-vic-torquay-152666740</t>
         </is>
       </c>
+      <c r="AA2">
+        <f>IF(OR(NOT(ISNUMBER(K2)),Settings!$B$35=""),"",IF(K2&lt;=Settings!$B$35,1,IF(K2&lt;=Settings!$B$36,2,IF(K2&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG2">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T2="Under offer",LEFT(T2,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X2="",X2="Unknown",Y2="",Y2="Unknown",AND(AND(ISNUMBER(Y2),Y2&lt;Settings!$B$31),OR(Z2="",Z2="Unknown"))),"Needs data: floorplan",IF(FIND(X2,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X2,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y2),Y2&lt;Settings!$B$31),Z2="Major"),"Not suitable: mobility",IF(FIND(X2,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y2),Y2&lt;Settings!$B$31),Z2="Minor works"),"Watchlist: minor mobility works",IF(T2="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA2),AA2&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA2),ABS(AA2-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD2&lt;&gt;"",AD2&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE2&lt;&gt;"",AE2&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB2),AB2&gt;10),AND(ISNUMBER(AC2),AC2&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="15">
       <c r="A3" s="22" t="n">
@@ -21139,6 +22482,14 @@
           <t>https://www.realestate.com.au/property-house-vic-west+footscray-152623144</t>
         </is>
       </c>
+      <c r="AA3">
+        <f>IF(OR(NOT(ISNUMBER(K3)),Settings!$B$35=""),"",IF(K3&lt;=Settings!$B$35,1,IF(K3&lt;=Settings!$B$36,2,IF(K3&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG3">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T3="Under offer",LEFT(T3,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X3="",X3="Unknown",Y3="",Y3="Unknown",AND(AND(ISNUMBER(Y3),Y3&lt;Settings!$B$31),OR(Z3="",Z3="Unknown"))),"Needs data: floorplan",IF(FIND(X3,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X3,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y3),Y3&lt;Settings!$B$31),Z3="Major"),"Not suitable: mobility",IF(FIND(X3,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y3),Y3&lt;Settings!$B$31),Z3="Minor works"),"Watchlist: minor mobility works",IF(T3="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA3),AA3&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA3),ABS(AA3-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD3&lt;&gt;"",AD3&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE3&lt;&gt;"",AE3&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB3),AB3&gt;10),AND(ISNUMBER(AC3),AC3&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="15">
       <c r="A4" s="22" t="n">
@@ -21231,6 +22582,14 @@
           <t>https://www.realestate.com.au/property-house-vic-warburton-150763740</t>
         </is>
       </c>
+      <c r="AA4">
+        <f>IF(OR(NOT(ISNUMBER(K4)),Settings!$B$35=""),"",IF(K4&lt;=Settings!$B$35,1,IF(K4&lt;=Settings!$B$36,2,IF(K4&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG4">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T4="Under offer",LEFT(T4,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X4="",X4="Unknown",Y4="",Y4="Unknown",AND(AND(ISNUMBER(Y4),Y4&lt;Settings!$B$31),OR(Z4="",Z4="Unknown"))),"Needs data: floorplan",IF(FIND(X4,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X4,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y4),Y4&lt;Settings!$B$31),Z4="Major"),"Not suitable: mobility",IF(FIND(X4,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y4),Y4&lt;Settings!$B$31),Z4="Minor works"),"Watchlist: minor mobility works",IF(T4="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA4),AA4&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA4),ABS(AA4-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD4&lt;&gt;"",AD4&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE4&lt;&gt;"",AE4&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB4),AB4&gt;10),AND(ISNUMBER(AC4),AC4&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="15">
       <c r="A5" s="22" t="n">
@@ -21315,6 +22674,14 @@
           <t>https://www.realestate.com.au/property-house-vic-williamstown-152686328</t>
         </is>
       </c>
+      <c r="AA5">
+        <f>IF(OR(NOT(ISNUMBER(K5)),Settings!$B$35=""),"",IF(K5&lt;=Settings!$B$35,1,IF(K5&lt;=Settings!$B$36,2,IF(K5&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG5">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T5="Under offer",LEFT(T5,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X5="",X5="Unknown",Y5="",Y5="Unknown",AND(AND(ISNUMBER(Y5),Y5&lt;Settings!$B$31),OR(Z5="",Z5="Unknown"))),"Needs data: floorplan",IF(FIND(X5,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X5,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y5),Y5&lt;Settings!$B$31),Z5="Major"),"Not suitable: mobility",IF(FIND(X5,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y5),Y5&lt;Settings!$B$31),Z5="Minor works"),"Watchlist: minor mobility works",IF(T5="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA5),AA5&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA5),ABS(AA5-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD5&lt;&gt;"",AD5&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE5&lt;&gt;"",AE5&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB5),AB5&gt;10),AND(ISNUMBER(AC5),AC5&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="15">
       <c r="A6" s="22" t="n">
@@ -21403,6 +22770,14 @@
           <t>https://www.realestate.com.au/property-house-vic-rosanna-152574468</t>
         </is>
       </c>
+      <c r="AA6">
+        <f>IF(OR(NOT(ISNUMBER(K6)),Settings!$B$35=""),"",IF(K6&lt;=Settings!$B$35,1,IF(K6&lt;=Settings!$B$36,2,IF(K6&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG6">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T6="Under offer",LEFT(T6,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X6="",X6="Unknown",Y6="",Y6="Unknown",AND(AND(ISNUMBER(Y6),Y6&lt;Settings!$B$31),OR(Z6="",Z6="Unknown"))),"Needs data: floorplan",IF(FIND(X6,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X6,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y6),Y6&lt;Settings!$B$31),Z6="Major"),"Not suitable: mobility",IF(FIND(X6,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y6),Y6&lt;Settings!$B$31),Z6="Minor works"),"Watchlist: minor mobility works",IF(T6="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA6),AA6&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA6),ABS(AA6-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD6&lt;&gt;"",AD6&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE6&lt;&gt;"",AE6&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB6),AB6&gt;10),AND(ISNUMBER(AC6),AC6&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="15">
       <c r="A7" s="22" t="n">
@@ -21490,6 +22865,14 @@
           <t>https://www.realestate.com.au/property-house-vic-diamond+creek-152290624</t>
         </is>
       </c>
+      <c r="AA7">
+        <f>IF(OR(NOT(ISNUMBER(K7)),Settings!$B$35=""),"",IF(K7&lt;=Settings!$B$35,1,IF(K7&lt;=Settings!$B$36,2,IF(K7&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG7">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T7="Under offer",LEFT(T7,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X7="",X7="Unknown",Y7="",Y7="Unknown",AND(AND(ISNUMBER(Y7),Y7&lt;Settings!$B$31),OR(Z7="",Z7="Unknown"))),"Needs data: floorplan",IF(FIND(X7,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X7,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y7),Y7&lt;Settings!$B$31),Z7="Major"),"Not suitable: mobility",IF(FIND(X7,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y7),Y7&lt;Settings!$B$31),Z7="Minor works"),"Watchlist: minor mobility works",IF(T7="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA7),AA7&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA7),ABS(AA7-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD7&lt;&gt;"",AD7&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE7&lt;&gt;"",AE7&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB7),AB7&gt;10),AND(ISNUMBER(AC7),AC7&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="15">
       <c r="A8" s="22" t="n">
@@ -21578,6 +22961,14 @@
           <t>https://www.realestate.com.au/property-house-vic-mordialloc-152622844</t>
         </is>
       </c>
+      <c r="AA8">
+        <f>IF(OR(NOT(ISNUMBER(K8)),Settings!$B$35=""),"",IF(K8&lt;=Settings!$B$35,1,IF(K8&lt;=Settings!$B$36,2,IF(K8&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG8">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T8="Under offer",LEFT(T8,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X8="",X8="Unknown",Y8="",Y8="Unknown",AND(AND(ISNUMBER(Y8),Y8&lt;Settings!$B$31),OR(Z8="",Z8="Unknown"))),"Needs data: floorplan",IF(FIND(X8,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X8,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y8),Y8&lt;Settings!$B$31),Z8="Major"),"Not suitable: mobility",IF(FIND(X8,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y8),Y8&lt;Settings!$B$31),Z8="Minor works"),"Watchlist: minor mobility works",IF(T8="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA8),AA8&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA8),ABS(AA8-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD8&lt;&gt;"",AD8&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE8&lt;&gt;"",AE8&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB8),AB8&gt;10),AND(ISNUMBER(AC8),AC8&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="15">
       <c r="A9" s="22" t="n">
@@ -21666,6 +23057,14 @@
           <t>https://www.realestate.com.au/property-house-vic-seaford-152011424</t>
         </is>
       </c>
+      <c r="AA9">
+        <f>IF(OR(NOT(ISNUMBER(K9)),Settings!$B$35=""),"",IF(K9&lt;=Settings!$B$35,1,IF(K9&lt;=Settings!$B$36,2,IF(K9&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG9">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T9="Under offer",LEFT(T9,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X9="",X9="Unknown",Y9="",Y9="Unknown",AND(AND(ISNUMBER(Y9),Y9&lt;Settings!$B$31),OR(Z9="",Z9="Unknown"))),"Needs data: floorplan",IF(FIND(X9,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X9,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y9),Y9&lt;Settings!$B$31),Z9="Major"),"Not suitable: mobility",IF(FIND(X9,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y9),Y9&lt;Settings!$B$31),Z9="Minor works"),"Watchlist: minor mobility works",IF(T9="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA9),AA9&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA9),ABS(AA9-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD9&lt;&gt;"",AD9&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE9&lt;&gt;"",AE9&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB9),AB9&gt;10),AND(ISNUMBER(AC9),AC9&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="15">
       <c r="A10" s="22" t="n">
@@ -21754,6 +23153,14 @@
           <t>https://www.realestate.com.au/property-house-vic-seaford-151815440</t>
         </is>
       </c>
+      <c r="AA10">
+        <f>IF(OR(NOT(ISNUMBER(K10)),Settings!$B$35=""),"",IF(K10&lt;=Settings!$B$35,1,IF(K10&lt;=Settings!$B$36,2,IF(K10&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG10">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T10="Under offer",LEFT(T10,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X10="",X10="Unknown",Y10="",Y10="Unknown",AND(AND(ISNUMBER(Y10),Y10&lt;Settings!$B$31),OR(Z10="",Z10="Unknown"))),"Needs data: floorplan",IF(FIND(X10,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X10,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y10),Y10&lt;Settings!$B$31),Z10="Major"),"Not suitable: mobility",IF(FIND(X10,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y10),Y10&lt;Settings!$B$31),Z10="Minor works"),"Watchlist: minor mobility works",IF(T10="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA10),AA10&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA10),ABS(AA10-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD10&lt;&gt;"",AD10&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE10&lt;&gt;"",AE10&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB10),AB10&gt;10),AND(ISNUMBER(AC10),AC10&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="22" t="n">
@@ -21841,6 +23248,14 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-151176748</t>
         </is>
       </c>
+      <c r="AA11">
+        <f>IF(OR(NOT(ISNUMBER(K11)),Settings!$B$35=""),"",IF(K11&lt;=Settings!$B$35,1,IF(K11&lt;=Settings!$B$36,2,IF(K11&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG11">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T11="Under offer",LEFT(T11,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X11="",X11="Unknown",Y11="",Y11="Unknown",AND(AND(ISNUMBER(Y11),Y11&lt;Settings!$B$31),OR(Z11="",Z11="Unknown"))),"Needs data: floorplan",IF(FIND(X11,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X11,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y11),Y11&lt;Settings!$B$31),Z11="Major"),"Not suitable: mobility",IF(FIND(X11,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y11),Y11&lt;Settings!$B$31),Z11="Minor works"),"Watchlist: minor mobility works",IF(T11="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA11),AA11&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA11),ABS(AA11-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD11&lt;&gt;"",AD11&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE11&lt;&gt;"",AE11&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB11),AB11&gt;10),AND(ISNUMBER(AC11),AC11&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="15">
       <c r="A12" s="22" t="n">
@@ -21928,6 +23343,14 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-152450032</t>
         </is>
       </c>
+      <c r="AA12">
+        <f>IF(OR(NOT(ISNUMBER(K12)),Settings!$B$35=""),"",IF(K12&lt;=Settings!$B$35,1,IF(K12&lt;=Settings!$B$36,2,IF(K12&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG12">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T12="Under offer",LEFT(T12,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X12="",X12="Unknown",Y12="",Y12="Unknown",AND(AND(ISNUMBER(Y12),Y12&lt;Settings!$B$31),OR(Z12="",Z12="Unknown"))),"Needs data: floorplan",IF(FIND(X12,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X12,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y12),Y12&lt;Settings!$B$31),Z12="Major"),"Not suitable: mobility",IF(FIND(X12,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y12),Y12&lt;Settings!$B$31),Z12="Minor works"),"Watchlist: minor mobility works",IF(T12="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA12),AA12&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA12),ABS(AA12-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD12&lt;&gt;"",AD12&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE12&lt;&gt;"",AE12&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB12),AB12&gt;10),AND(ISNUMBER(AC12),AC12&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="15">
       <c r="A13" s="22" t="n">
@@ -22015,6 +23438,14 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-152376824</t>
         </is>
       </c>
+      <c r="AA13">
+        <f>IF(OR(NOT(ISNUMBER(K13)),Settings!$B$35=""),"",IF(K13&lt;=Settings!$B$35,1,IF(K13&lt;=Settings!$B$36,2,IF(K13&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG13">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T13="Under offer",LEFT(T13,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X13="",X13="Unknown",Y13="",Y13="Unknown",AND(AND(ISNUMBER(Y13),Y13&lt;Settings!$B$31),OR(Z13="",Z13="Unknown"))),"Needs data: floorplan",IF(FIND(X13,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X13,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y13),Y13&lt;Settings!$B$31),Z13="Major"),"Not suitable: mobility",IF(FIND(X13,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y13),Y13&lt;Settings!$B$31),Z13="Minor works"),"Watchlist: minor mobility works",IF(T13="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA13),AA13&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA13),ABS(AA13-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD13&lt;&gt;"",AD13&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE13&lt;&gt;"",AE13&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB13),AB13&gt;10),AND(ISNUMBER(AC13),AC13&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="15">
       <c r="A14" s="22" t="n">
@@ -22102,6 +23533,14 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-151903892</t>
         </is>
       </c>
+      <c r="AA14">
+        <f>IF(OR(NOT(ISNUMBER(K14)),Settings!$B$35=""),"",IF(K14&lt;=Settings!$B$35,1,IF(K14&lt;=Settings!$B$36,2,IF(K14&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG14">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T14="Under offer",LEFT(T14,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X14="",X14="Unknown",Y14="",Y14="Unknown",AND(AND(ISNUMBER(Y14),Y14&lt;Settings!$B$31),OR(Z14="",Z14="Unknown"))),"Needs data: floorplan",IF(FIND(X14,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X14,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y14),Y14&lt;Settings!$B$31),Z14="Major"),"Not suitable: mobility",IF(FIND(X14,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y14),Y14&lt;Settings!$B$31),Z14="Minor works"),"Watchlist: minor mobility works",IF(T14="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA14),AA14&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA14),ABS(AA14-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD14&lt;&gt;"",AD14&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE14&lt;&gt;"",AE14&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB14),AB14&gt;10),AND(ISNUMBER(AC14),AC14&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="15">
       <c r="A15" s="22" t="n">
@@ -22190,6 +23629,14 @@
           <t>https://www.realestate.com.au/property-house-vic-arthurs+seat-146680920</t>
         </is>
       </c>
+      <c r="AA15">
+        <f>IF(OR(NOT(ISNUMBER(K15)),Settings!$B$35=""),"",IF(K15&lt;=Settings!$B$35,1,IF(K15&lt;=Settings!$B$36,2,IF(K15&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG15">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T15="Under offer",LEFT(T15,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X15="",X15="Unknown",Y15="",Y15="Unknown",AND(AND(ISNUMBER(Y15),Y15&lt;Settings!$B$31),OR(Z15="",Z15="Unknown"))),"Needs data: floorplan",IF(FIND(X15,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X15,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y15),Y15&lt;Settings!$B$31),Z15="Major"),"Not suitable: mobility",IF(FIND(X15,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y15),Y15&lt;Settings!$B$31),Z15="Minor works"),"Watchlist: minor mobility works",IF(T15="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA15),AA15&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA15),ABS(AA15-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD15&lt;&gt;"",AD15&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE15&lt;&gt;"",AE15&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB15),AB15&gt;10),AND(ISNUMBER(AC15),AC15&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="15">
       <c r="A16" s="22" t="n">
@@ -22278,6 +23725,14 @@
           <t>https://www.realestate.com.au/property-house-vic-dromana-152005848</t>
         </is>
       </c>
+      <c r="AA16">
+        <f>IF(OR(NOT(ISNUMBER(K16)),Settings!$B$35=""),"",IF(K16&lt;=Settings!$B$35,1,IF(K16&lt;=Settings!$B$36,2,IF(K16&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG16">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T16="Under offer",LEFT(T16,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X16="",X16="Unknown",Y16="",Y16="Unknown",AND(AND(ISNUMBER(Y16),Y16&lt;Settings!$B$31),OR(Z16="",Z16="Unknown"))),"Needs data: floorplan",IF(FIND(X16,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X16,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y16),Y16&lt;Settings!$B$31),Z16="Major"),"Not suitable: mobility",IF(FIND(X16,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y16),Y16&lt;Settings!$B$31),Z16="Minor works"),"Watchlist: minor mobility works",IF(T16="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA16),AA16&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA16),ABS(AA16-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD16&lt;&gt;"",AD16&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE16&lt;&gt;"",AE16&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB16),AB16&gt;10),AND(ISNUMBER(AC16),AC16&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="15">
       <c r="A17" s="22" t="n">
@@ -22366,6 +23821,14 @@
           <t>https://www.realestate.com.au/property-house-vic-curlewis-152352192</t>
         </is>
       </c>
+      <c r="AA17">
+        <f>IF(OR(NOT(ISNUMBER(K17)),Settings!$B$35=""),"",IF(K17&lt;=Settings!$B$35,1,IF(K17&lt;=Settings!$B$36,2,IF(K17&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG17">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T17="Under offer",LEFT(T17,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X17="",X17="Unknown",Y17="",Y17="Unknown",AND(AND(ISNUMBER(Y17),Y17&lt;Settings!$B$31),OR(Z17="",Z17="Unknown"))),"Needs data: floorplan",IF(FIND(X17,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X17,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y17),Y17&lt;Settings!$B$31),Z17="Major"),"Not suitable: mobility",IF(FIND(X17,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y17),Y17&lt;Settings!$B$31),Z17="Minor works"),"Watchlist: minor mobility works",IF(T17="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA17),AA17&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA17),ABS(AA17-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD17&lt;&gt;"",AD17&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE17&lt;&gt;"",AE17&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB17),AB17&gt;10),AND(ISNUMBER(AC17),AC17&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="15">
       <c r="A18" s="22" t="n">
@@ -22454,6 +23917,14 @@
           <t>https://www.realestate.com.au/property-house-vic-mccrae-151835348</t>
         </is>
       </c>
+      <c r="AA18">
+        <f>IF(OR(NOT(ISNUMBER(K18)),Settings!$B$35=""),"",IF(K18&lt;=Settings!$B$35,1,IF(K18&lt;=Settings!$B$36,2,IF(K18&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG18">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T18="Under offer",LEFT(T18,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X18="",X18="Unknown",Y18="",Y18="Unknown",AND(AND(ISNUMBER(Y18),Y18&lt;Settings!$B$31),OR(Z18="",Z18="Unknown"))),"Needs data: floorplan",IF(FIND(X18,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X18,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y18),Y18&lt;Settings!$B$31),Z18="Major"),"Not suitable: mobility",IF(FIND(X18,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y18),Y18&lt;Settings!$B$31),Z18="Minor works"),"Watchlist: minor mobility works",IF(T18="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA18),AA18&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA18),ABS(AA18-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD18&lt;&gt;"",AD18&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE18&lt;&gt;"",AE18&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB18),AB18&gt;10),AND(ISNUMBER(AC18),AC18&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="15">
       <c r="A19" s="22" t="n">
@@ -22542,6 +24013,14 @@
           <t>https://www.realestate.com.au/property-house-vic-chelsea-152626264</t>
         </is>
       </c>
+      <c r="AA19">
+        <f>IF(OR(NOT(ISNUMBER(K19)),Settings!$B$35=""),"",IF(K19&lt;=Settings!$B$35,1,IF(K19&lt;=Settings!$B$36,2,IF(K19&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG19">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T19="Under offer",LEFT(T19,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X19="",X19="Unknown",Y19="",Y19="Unknown",AND(AND(ISNUMBER(Y19),Y19&lt;Settings!$B$31),OR(Z19="",Z19="Unknown"))),"Needs data: floorplan",IF(FIND(X19,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X19,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y19),Y19&lt;Settings!$B$31),Z19="Major"),"Not suitable: mobility",IF(FIND(X19,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y19),Y19&lt;Settings!$B$31),Z19="Minor works"),"Watchlist: minor mobility works",IF(T19="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA19),AA19&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA19),ABS(AA19-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD19&lt;&gt;"",AD19&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE19&lt;&gt;"",AE19&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB19),AB19&gt;10),AND(ISNUMBER(AC19),AC19&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="15">
       <c r="A20" s="22" t="n">
@@ -22629,6 +24108,14 @@
           <t>https://www.realestate.com.au/property-house-vic-torquay-152670688</t>
         </is>
       </c>
+      <c r="AA20">
+        <f>IF(OR(NOT(ISNUMBER(K20)),Settings!$B$35=""),"",IF(K20&lt;=Settings!$B$35,1,IF(K20&lt;=Settings!$B$36,2,IF(K20&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG20">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T20="Under offer",LEFT(T20,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X20="",X20="Unknown",Y20="",Y20="Unknown",AND(AND(ISNUMBER(Y20),Y20&lt;Settings!$B$31),OR(Z20="",Z20="Unknown"))),"Needs data: floorplan",IF(FIND(X20,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X20,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y20),Y20&lt;Settings!$B$31),Z20="Major"),"Not suitable: mobility",IF(FIND(X20,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y20),Y20&lt;Settings!$B$31),Z20="Minor works"),"Watchlist: minor mobility works",IF(T20="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA20),AA20&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA20),ABS(AA20-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD20&lt;&gt;"",AD20&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE20&lt;&gt;"",AE20&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB20),AB20&gt;10),AND(ISNUMBER(AC20),AC20&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="15">
       <c r="A21" s="22" t="n">
@@ -22717,6 +24204,14 @@
           <t>https://www.realestate.com.au/property-house-vic-newport-152302080</t>
         </is>
       </c>
+      <c r="AA21">
+        <f>IF(OR(NOT(ISNUMBER(K21)),Settings!$B$35=""),"",IF(K21&lt;=Settings!$B$35,1,IF(K21&lt;=Settings!$B$36,2,IF(K21&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG21">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T21="Under offer",LEFT(T21,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X21="",X21="Unknown",Y21="",Y21="Unknown",AND(AND(ISNUMBER(Y21),Y21&lt;Settings!$B$31),OR(Z21="",Z21="Unknown"))),"Needs data: floorplan",IF(FIND(X21,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X21,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y21),Y21&lt;Settings!$B$31),Z21="Major"),"Not suitable: mobility",IF(FIND(X21,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y21),Y21&lt;Settings!$B$31),Z21="Minor works"),"Watchlist: minor mobility works",IF(T21="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA21),AA21&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA21),ABS(AA21-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD21&lt;&gt;"",AD21&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE21&lt;&gt;"",AE21&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB21),AB21&gt;10),AND(ISNUMBER(AC21),AC21&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="15">
       <c r="A22" s="22" t="n">
@@ -22809,6 +24304,14 @@
           <t>https://www.realestate.com.au/property-house-vic-frankston+south-152212372</t>
         </is>
       </c>
+      <c r="AA22">
+        <f>IF(OR(NOT(ISNUMBER(K22)),Settings!$B$35=""),"",IF(K22&lt;=Settings!$B$35,1,IF(K22&lt;=Settings!$B$36,2,IF(K22&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG22">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T22="Under offer",LEFT(T22,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X22="",X22="Unknown",Y22="",Y22="Unknown",AND(AND(ISNUMBER(Y22),Y22&lt;Settings!$B$31),OR(Z22="",Z22="Unknown"))),"Needs data: floorplan",IF(FIND(X22,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X22,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y22),Y22&lt;Settings!$B$31),Z22="Major"),"Not suitable: mobility",IF(FIND(X22,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y22),Y22&lt;Settings!$B$31),Z22="Minor works"),"Watchlist: minor mobility works",IF(T22="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA22),AA22&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA22),ABS(AA22-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD22&lt;&gt;"",AD22&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE22&lt;&gt;"",AE22&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB22),AB22&gt;10),AND(ISNUMBER(AC22),AC22&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="15">
       <c r="A23" s="22" t="n">
@@ -22896,6 +24399,14 @@
           <t>https://www.realestate.com.au/property-house-vic-tecoma-152652276</t>
         </is>
       </c>
+      <c r="AA23">
+        <f>IF(OR(NOT(ISNUMBER(K23)),Settings!$B$35=""),"",IF(K23&lt;=Settings!$B$35,1,IF(K23&lt;=Settings!$B$36,2,IF(K23&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG23">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T23="Under offer",LEFT(T23,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X23="",X23="Unknown",Y23="",Y23="Unknown",AND(AND(ISNUMBER(Y23),Y23&lt;Settings!$B$31),OR(Z23="",Z23="Unknown"))),"Needs data: floorplan",IF(FIND(X23,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X23,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y23),Y23&lt;Settings!$B$31),Z23="Major"),"Not suitable: mobility",IF(FIND(X23,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y23),Y23&lt;Settings!$B$31),Z23="Minor works"),"Watchlist: minor mobility works",IF(T23="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA23),AA23&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA23),ABS(AA23-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD23&lt;&gt;"",AD23&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE23&lt;&gt;"",AE23&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB23),AB23&gt;10),AND(ISNUMBER(AC23),AC23&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="15">
       <c r="A24" s="22" t="n">
@@ -22988,6 +24499,14 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152722196</t>
         </is>
       </c>
+      <c r="AA24">
+        <f>IF(OR(NOT(ISNUMBER(K24)),Settings!$B$35=""),"",IF(K24&lt;=Settings!$B$35,1,IF(K24&lt;=Settings!$B$36,2,IF(K24&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG24">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T24="Under offer",LEFT(T24,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X24="",X24="Unknown",Y24="",Y24="Unknown",AND(AND(ISNUMBER(Y24),Y24&lt;Settings!$B$31),OR(Z24="",Z24="Unknown"))),"Needs data: floorplan",IF(FIND(X24,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X24,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y24),Y24&lt;Settings!$B$31),Z24="Major"),"Not suitable: mobility",IF(FIND(X24,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y24),Y24&lt;Settings!$B$31),Z24="Minor works"),"Watchlist: minor mobility works",IF(T24="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA24),AA24&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA24),ABS(AA24-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD24&lt;&gt;"",AD24&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE24&lt;&gt;"",AE24&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB24),AB24&gt;10),AND(ISNUMBER(AC24),AC24&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="15">
       <c r="A25" s="22" t="n">
@@ -23077,6 +24596,14 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152535704</t>
         </is>
       </c>
+      <c r="AA25">
+        <f>IF(OR(NOT(ISNUMBER(K25)),Settings!$B$35=""),"",IF(K25&lt;=Settings!$B$35,1,IF(K25&lt;=Settings!$B$36,2,IF(K25&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG25">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T25="Under offer",LEFT(T25,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X25="",X25="Unknown",Y25="",Y25="Unknown",AND(AND(ISNUMBER(Y25),Y25&lt;Settings!$B$31),OR(Z25="",Z25="Unknown"))),"Needs data: floorplan",IF(FIND(X25,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X25,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y25),Y25&lt;Settings!$B$31),Z25="Major"),"Not suitable: mobility",IF(FIND(X25,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y25),Y25&lt;Settings!$B$31),Z25="Minor works"),"Watchlist: minor mobility works",IF(T25="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA25),AA25&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA25),ABS(AA25-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD25&lt;&gt;"",AD25&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE25&lt;&gt;"",AE25&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB25),AB25&gt;10),AND(ISNUMBER(AC25),AC25&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="15">
       <c r="A26" s="22" t="n">
@@ -23164,6 +24691,14 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152654296</t>
         </is>
       </c>
+      <c r="AA26">
+        <f>IF(OR(NOT(ISNUMBER(K26)),Settings!$B$35=""),"",IF(K26&lt;=Settings!$B$35,1,IF(K26&lt;=Settings!$B$36,2,IF(K26&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG26">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T26="Under offer",LEFT(T26,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X26="",X26="Unknown",Y26="",Y26="Unknown",AND(AND(ISNUMBER(Y26),Y26&lt;Settings!$B$31),OR(Z26="",Z26="Unknown"))),"Needs data: floorplan",IF(FIND(X26,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X26,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y26),Y26&lt;Settings!$B$31),Z26="Major"),"Not suitable: mobility",IF(FIND(X26,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y26),Y26&lt;Settings!$B$31),Z26="Minor works"),"Watchlist: minor mobility works",IF(T26="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA26),AA26&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA26),ABS(AA26-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD26&lt;&gt;"",AD26&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE26&lt;&gt;"",AE26&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB26),AB26&gt;10),AND(ISNUMBER(AC26),AC26&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="15">
       <c r="A27" s="22" t="n">
@@ -23251,6 +24786,14 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152729140</t>
         </is>
       </c>
+      <c r="AA27">
+        <f>IF(OR(NOT(ISNUMBER(K27)),Settings!$B$35=""),"",IF(K27&lt;=Settings!$B$35,1,IF(K27&lt;=Settings!$B$36,2,IF(K27&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG27">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T27="Under offer",LEFT(T27,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X27="",X27="Unknown",Y27="",Y27="Unknown",AND(AND(ISNUMBER(Y27),Y27&lt;Settings!$B$31),OR(Z27="",Z27="Unknown"))),"Needs data: floorplan",IF(FIND(X27,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X27,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y27),Y27&lt;Settings!$B$31),Z27="Major"),"Not suitable: mobility",IF(FIND(X27,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y27),Y27&lt;Settings!$B$31),Z27="Minor works"),"Watchlist: minor mobility works",IF(T27="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA27),AA27&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA27),ABS(AA27-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD27&lt;&gt;"",AD27&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE27&lt;&gt;"",AE27&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB27),AB27&gt;10),AND(ISNUMBER(AC27),AC27&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="15">
       <c r="A28" s="22" t="n">
@@ -23339,6 +24882,14 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+martha-152575492</t>
         </is>
       </c>
+      <c r="AA28">
+        <f>IF(OR(NOT(ISNUMBER(K28)),Settings!$B$35=""),"",IF(K28&lt;=Settings!$B$35,1,IF(K28&lt;=Settings!$B$36,2,IF(K28&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG28">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T28="Under offer",LEFT(T28,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X28="",X28="Unknown",Y28="",Y28="Unknown",AND(AND(ISNUMBER(Y28),Y28&lt;Settings!$B$31),OR(Z28="",Z28="Unknown"))),"Needs data: floorplan",IF(FIND(X28,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X28,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y28),Y28&lt;Settings!$B$31),Z28="Major"),"Not suitable: mobility",IF(FIND(X28,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y28),Y28&lt;Settings!$B$31),Z28="Minor works"),"Watchlist: minor mobility works",IF(T28="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA28),AA28&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA28),ABS(AA28-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD28&lt;&gt;"",AD28&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE28&lt;&gt;"",AE28&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB28),AB28&gt;10),AND(ISNUMBER(AC28),AC28&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="15">
       <c r="A29" s="22" t="n">
@@ -23426,6 +24977,14 @@
           <t>https://www.realestate.com.au/property-house-vic-tecoma-152712080</t>
         </is>
       </c>
+      <c r="AA29">
+        <f>IF(OR(NOT(ISNUMBER(K29)),Settings!$B$35=""),"",IF(K29&lt;=Settings!$B$35,1,IF(K29&lt;=Settings!$B$36,2,IF(K29&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG29">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T29="Under offer",LEFT(T29,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X29="",X29="Unknown",Y29="",Y29="Unknown",AND(AND(ISNUMBER(Y29),Y29&lt;Settings!$B$31),OR(Z29="",Z29="Unknown"))),"Needs data: floorplan",IF(FIND(X29,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X29,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y29),Y29&lt;Settings!$B$31),Z29="Major"),"Not suitable: mobility",IF(FIND(X29,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y29),Y29&lt;Settings!$B$31),Z29="Minor works"),"Watchlist: minor mobility works",IF(T29="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA29),AA29&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA29),ABS(AA29-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD29&lt;&gt;"",AD29&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE29&lt;&gt;"",AE29&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB29),AB29&gt;10),AND(ISNUMBER(AC29),AC29&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="15">
       <c r="A30" s="22" t="n">
@@ -23513,6 +25072,14 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152583472</t>
         </is>
       </c>
+      <c r="AA30">
+        <f>IF(OR(NOT(ISNUMBER(K30)),Settings!$B$35=""),"",IF(K30&lt;=Settings!$B$35,1,IF(K30&lt;=Settings!$B$36,2,IF(K30&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG30">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T30="Under offer",LEFT(T30,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X30="",X30="Unknown",Y30="",Y30="Unknown",AND(AND(ISNUMBER(Y30),Y30&lt;Settings!$B$31),OR(Z30="",Z30="Unknown"))),"Needs data: floorplan",IF(FIND(X30,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X30,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y30),Y30&lt;Settings!$B$31),Z30="Major"),"Not suitable: mobility",IF(FIND(X30,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y30),Y30&lt;Settings!$B$31),Z30="Minor works"),"Watchlist: minor mobility works",IF(T30="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA30),AA30&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA30),ABS(AA30-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD30&lt;&gt;"",AD30&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE30&lt;&gt;"",AE30&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB30),AB30&gt;10),AND(ISNUMBER(AC30),AC30&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="15">
       <c r="A31" s="22" t="n">
@@ -23605,6 +25172,14 @@
           <t>https://www.realestate.com.au/property-house-vic-frankston-151132640</t>
         </is>
       </c>
+      <c r="AA31">
+        <f>IF(OR(NOT(ISNUMBER(K31)),Settings!$B$35=""),"",IF(K31&lt;=Settings!$B$35,1,IF(K31&lt;=Settings!$B$36,2,IF(K31&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG31">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T31="Under offer",LEFT(T31,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X31="",X31="Unknown",Y31="",Y31="Unknown",AND(AND(ISNUMBER(Y31),Y31&lt;Settings!$B$31),OR(Z31="",Z31="Unknown"))),"Needs data: floorplan",IF(FIND(X31,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X31,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y31),Y31&lt;Settings!$B$31),Z31="Major"),"Not suitable: mobility",IF(FIND(X31,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y31),Y31&lt;Settings!$B$31),Z31="Minor works"),"Watchlist: minor mobility works",IF(T31="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA31),AA31&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA31),ABS(AA31-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD31&lt;&gt;"",AD31&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE31&lt;&gt;"",AE31&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB31),AB31&gt;10),AND(ISNUMBER(AC31),AC31&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="15">
       <c r="A32" s="22" t="n">
@@ -23692,6 +25267,14 @@
           <t>https://www.realestate.com.au/property-house-vic-frankston+south-152593596</t>
         </is>
       </c>
+      <c r="AA32">
+        <f>IF(OR(NOT(ISNUMBER(K32)),Settings!$B$35=""),"",IF(K32&lt;=Settings!$B$35,1,IF(K32&lt;=Settings!$B$36,2,IF(K32&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG32">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T32="Under offer",LEFT(T32,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X32="",X32="Unknown",Y32="",Y32="Unknown",AND(AND(ISNUMBER(Y32),Y32&lt;Settings!$B$31),OR(Z32="",Z32="Unknown"))),"Needs data: floorplan",IF(FIND(X32,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X32,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y32),Y32&lt;Settings!$B$31),Z32="Major"),"Not suitable: mobility",IF(FIND(X32,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y32),Y32&lt;Settings!$B$31),Z32="Minor works"),"Watchlist: minor mobility works",IF(T32="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA32),AA32&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA32),ABS(AA32-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD32&lt;&gt;"",AD32&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE32&lt;&gt;"",AE32&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB32),AB32&gt;10),AND(ISNUMBER(AC32),AC32&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="15">
       <c r="A33" s="22" t="n">
@@ -23778,6 +25361,14 @@
         <is>
           <t>https://www.realestate.com.au/property-house-vic-frankston+south-152448552</t>
         </is>
+      </c>
+      <c r="AA33">
+        <f>IF(OR(NOT(ISNUMBER(K33)),Settings!$B$35=""),"",IF(K33&lt;=Settings!$B$35,1,IF(K33&lt;=Settings!$B$36,2,IF(K33&lt;=Settings!$B$37,3,4))))</f>
+        <v/>
+      </c>
+      <c r="AG33">
+        <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T33="Under offer",LEFT(T33,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X33="",X33="Unknown",Y33="",Y33="Unknown",AND(AND(ISNUMBER(Y33),Y33&lt;Settings!$B$31),OR(Z33="",Z33="Unknown"))),"Needs data: floorplan",IF(FIND(X33,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X33,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y33),Y33&lt;Settings!$B$31),Z33="Major"),"Not suitable: mobility",IF(FIND(X33,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y33),Y33&lt;Settings!$B$31),Z33="Minor works"),"Watchlist: minor mobility works",IF(T33="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA33),AA33&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA33),ABS(AA33-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD33&lt;&gt;"",AD33&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE33&lt;&gt;"",AE33&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB33),AB33&gt;10),AND(ISNUMBER(AC33),AC33&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add questionnaire v14 import tool, test coverage, and documentation
</commit_message>
<xml_diff>
--- a/Our Next Home — Family Relocation Scoring Model.xlsx
+++ b/Our Next Home — Family Relocation Scoring Model.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="StartHere" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="RawResponses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="CleanedAnswers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Filters" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="PriorityWeights" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ForcedChoiceCorrections" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="SuburbScorecard" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Listings" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DiscussionSummary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StartHere" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RawResponses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CleanedAnswers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filters" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PriorityWeights" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForcedChoiceCorrections" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SuburbScorecard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listings" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DiscussionSummary" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Listings'!$A$1:$U$33</definedName>
@@ -1358,165 +1358,165 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="22" t="inlineStr">
         <is>
           <t>Rounds 5–6 answers (display-only; added 30 Oct 2026; no pass count until N4)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="22" t="inlineStr">
         <is>
           <t>GW firm limit (min)</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="22" t="inlineStr">
         <is>
           <t>GW preferred (min)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>ED firm limit (min)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="22" t="inlineStr">
         <is>
           <t>R5.7 church denomination</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="22" t="inlineStr">
         <is>
           <t>Answer check</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>Mum</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" s="22">
         <f>CleanedAnswers!B59</f>
         <v/>
       </c>
-      <c r="C42">
+      <c r="C42" s="22">
         <f>CleanedAnswers!B60</f>
         <v/>
       </c>
-      <c r="D42">
+      <c r="D42" s="22">
         <f>IF(CleanedAnswers!E44="E","No limit",CleanedAnswers!B61)</f>
         <v/>
       </c>
-      <c r="E42">
+      <c r="E42" s="22">
         <f>CleanedAnswers!B47</f>
         <v/>
       </c>
-      <c r="F42">
+      <c r="F42" s="22">
         <f>CleanedAnswers!B71</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" s="22">
         <f>CleanedAnswers!C59</f>
         <v/>
       </c>
-      <c r="C43">
+      <c r="C43" s="22">
         <f>CleanedAnswers!C60</f>
         <v/>
       </c>
-      <c r="D43">
+      <c r="D43" s="22">
         <f>IF(CleanedAnswers!F44="E","No limit",CleanedAnswers!C61)</f>
         <v/>
       </c>
-      <c r="E43">
+      <c r="E43" s="22">
         <f>CleanedAnswers!C47</f>
         <v/>
       </c>
-      <c r="F43">
+      <c r="F43" s="22">
         <f>CleanedAnswers!C71</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>Me</t>
         </is>
       </c>
-      <c r="B44">
+      <c r="B44" s="22">
         <f>CleanedAnswers!D59</f>
         <v/>
       </c>
-      <c r="C44">
+      <c r="C44" s="22">
         <f>CleanedAnswers!D60</f>
         <v/>
       </c>
-      <c r="D44">
+      <c r="D44" s="22">
         <f>IF(CleanedAnswers!G44="E","No limit",CleanedAnswers!D61)</f>
         <v/>
       </c>
-      <c r="E44">
+      <c r="E44" s="22">
         <f>CleanedAnswers!D47</f>
         <v/>
       </c>
-      <c r="F44">
+      <c r="F44" s="22">
         <f>CleanedAnswers!D71</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>Household (strictest)</t>
         </is>
       </c>
-      <c r="B45">
+      <c r="B45" s="22">
         <f>CleanedAnswers!E59</f>
         <v/>
       </c>
-      <c r="C45">
+      <c r="C45" s="22">
         <f>CleanedAnswers!E60</f>
         <v/>
       </c>
-      <c r="D45">
+      <c r="D45" s="22">
         <f>CleanedAnswers!E61</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>Separation (household floor / ceiling / check)</t>
         </is>
       </c>
-      <c r="B47">
+      <c r="B47" s="22">
         <f>CleanedAnswers!E64</f>
         <v/>
       </c>
-      <c r="C47">
+      <c r="C47" s="22">
         <f>CleanedAnswers!E65</f>
         <v/>
       </c>
-      <c r="D47">
+      <c r="D47" s="22">
         <f>CleanedAnswers!F65</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>Household cells stay blank until all three have answered. GW preferred (R5.3) is a preference only: never a filter or score. Filters change only at G2, with approval.</t>
         </is>
@@ -1836,209 +1836,209 @@
       <c r="C25" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>Property fit parameters (rounds 5–6)</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="22" t="inlineStr">
         <is>
           <t>Value (approved)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="22" t="inlineStr">
         <is>
           <t>Survey reference</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="22" t="inlineStr">
         <is>
           <t>B blank until approved (G5; B38/B39 at G3). Intake changes no fit result</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="22" t="inlineStr">
         <is>
           <t>Separation floor (1–4)</t>
         </is>
       </c>
-      <c r="C28">
+      <c r="C28" s="22">
         <f>CleanedAnswers!E64</f>
         <v/>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>R6.1, household MAX</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>Separation ceiling (1–4)</t>
         </is>
       </c>
-      <c r="C29">
+      <c r="C29" s="22">
         <f>CleanedAnswers!E65</f>
         <v/>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>R6.2, household MIN</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>Separation importance (3 Essential / 2 Important / 1 Nice to have)</t>
         </is>
       </c>
-      <c r="C30">
+      <c r="C30" s="22">
         <f>CleanedAnswers!E66</f>
         <v/>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>R6.3, household MAX</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>Mobility must-have (0–3)</t>
         </is>
       </c>
-      <c r="C31">
+      <c r="C31" s="22">
         <f>CleanedAnswers!E67</f>
         <v/>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>R6.4, household MAX</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>Garden preferred band (1–4)</t>
         </is>
       </c>
-      <c r="C32">
+      <c r="C32" s="22">
         <f>CleanedAnswers!E68</f>
         <v/>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>R6.5a, household MEDIAN</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="22" t="inlineStr">
         <is>
           <t>Garden capacity band (1–4)</t>
         </is>
       </c>
-      <c r="C33">
+      <c r="C33" s="22">
         <f>CleanedAnswers!E69</f>
         <v/>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>R6.5b, household MEDIAN</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>Front-door access (1–4)</t>
         </is>
       </c>
-      <c r="C34">
+      <c r="C34" s="22">
         <f>CleanedAnswers!E70</f>
         <v/>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="22" t="inlineStr">
         <is>
           <t>R6.6, household MIN</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>Land-size band: courtyard (m², up to)</t>
         </is>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" s="22" t="n">
         <v>400</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="22" t="inlineStr">
         <is>
           <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>Land-size band: small garden (m², up to)</t>
         </is>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" s="22" t="n">
         <v>650</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="22" t="inlineStr">
         <is>
           <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>Land-size band: medium garden (m², up to)</t>
         </is>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" s="22" t="n">
         <v>1000</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="22" t="inlineStr">
         <is>
           <t>Estimate; above = large</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>M scale (min)</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" s="22" t="n">
         <v>90</v>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="22" t="inlineStr">
         <is>
           <t>Proposed; B set at G3 (M/O decoupling)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>O scale (min)</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C39" s="22" t="n">
         <v>90</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>Proposed; B set at G3 (M/O decoupling)</t>
         </is>
@@ -2268,87 +2268,87 @@
           <t>[Q13d] Green village vs multicultural neighbourhood (reference-only)</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="22" t="inlineStr">
         <is>
           <t>[R5.1] Time in Glen Waverley in person</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="22" t="inlineStr">
         <is>
           <t>[R5.2] GW drive: firm limit</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="22" t="inlineStr">
         <is>
           <t>[R5.3] GW drive: preferred</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="22" t="inlineStr">
         <is>
           <t>[R5.4] ED drive: firm limit</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="22" t="inlineStr">
         <is>
           <t>[R5.5] Community place used most</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="22" t="inlineStr">
         <is>
           <t>[R5.6] Community place: longest regular drive</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="22" t="inlineStr">
         <is>
           <t>[R5.7] Church: particular denomination</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AV1" s="22" t="inlineStr">
         <is>
           <t>[R5 Notes]</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AW1" s="22" t="inlineStr">
         <is>
           <t>[R6.1] Separation: least that would work</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AX1" s="22" t="inlineStr">
         <is>
           <t>[R6.2] Separation: most that still feels like one household</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AY1" s="22" t="inlineStr">
         <is>
           <t>[R6.3] Separation: importance of having it already</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="AZ1" s="22" t="inlineStr">
         <is>
           <t>[R6.4] Mobility: must-have in 10-15 years</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BA1" s="22" t="inlineStr">
         <is>
           <t>[R6.5a] Outdoor space wanted</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BB1" s="22" t="inlineStr">
         <is>
           <t>[R6.5b] Garden upkeep capacity</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BC1" s="22" t="inlineStr">
         <is>
           <t>[R6.6] Supermarket and GP from the front door</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BD1" s="22" t="inlineStr">
         <is>
           <t>[R6.7] Privacy: one thing that matters most</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BE1" s="22" t="inlineStr">
         <is>
           <t>[R6 Notes]</t>
         </is>
@@ -5376,803 +5376,803 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>[R5.1] Time in Glen Waverley in person</t>
         </is>
       </c>
-      <c r="B41">
+      <c r="B41" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C41">
+      <c r="C41" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D41">
+      <c r="D41" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A41&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E41">
+      <c r="E41" s="22">
         <f>LEFT(B41,1)</f>
         <v/>
       </c>
-      <c r="F41">
+      <c r="F41" s="22">
         <f>LEFT(C41,1)</f>
         <v/>
       </c>
-      <c r="G41">
+      <c r="G41" s="22">
         <f>LEFT(D41,1)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>[R5.2] GW drive: firm limit</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C42">
+      <c r="C42" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D42">
+      <c r="D42" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A42&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E42">
+      <c r="E42" s="22">
         <f>LEFT(B42,1)</f>
         <v/>
       </c>
-      <c r="F42">
+      <c r="F42" s="22">
         <f>LEFT(C42,1)</f>
         <v/>
       </c>
-      <c r="G42">
+      <c r="G42" s="22">
         <f>LEFT(D42,1)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>[R5.3] GW drive: preferred</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C43">
+      <c r="C43" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D43">
+      <c r="D43" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A43&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E43">
+      <c r="E43" s="22">
         <f>LEFT(B43,1)</f>
         <v/>
       </c>
-      <c r="F43">
+      <c r="F43" s="22">
         <f>LEFT(C43,1)</f>
         <v/>
       </c>
-      <c r="G43">
+      <c r="G43" s="22">
         <f>LEFT(D43,1)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>[R5.4] ED drive: firm limit</t>
         </is>
       </c>
-      <c r="B44">
+      <c r="B44" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C44">
+      <c r="C44" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D44">
+      <c r="D44" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A44&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E44">
+      <c r="E44" s="22">
         <f>LEFT(B44,1)</f>
         <v/>
       </c>
-      <c r="F44">
+      <c r="F44" s="22">
         <f>LEFT(C44,1)</f>
         <v/>
       </c>
-      <c r="G44">
+      <c r="G44" s="22">
         <f>LEFT(D44,1)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>[R5.5] Community place used most</t>
         </is>
       </c>
-      <c r="B45">
+      <c r="B45" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C45">
+      <c r="C45" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D45">
+      <c r="D45" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A45&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E45">
+      <c r="E45" s="22">
         <f>LEFT(B45,1)</f>
         <v/>
       </c>
-      <c r="F45">
+      <c r="F45" s="22">
         <f>LEFT(C45,1)</f>
         <v/>
       </c>
-      <c r="G45">
+      <c r="G45" s="22">
         <f>LEFT(D45,1)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>[R5.6] Community place: longest regular drive</t>
         </is>
       </c>
-      <c r="B46">
+      <c r="B46" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C46">
+      <c r="C46" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D46">
+      <c r="D46" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A46&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E46">
+      <c r="E46" s="22">
         <f>LEFT(B46,1)</f>
         <v/>
       </c>
-      <c r="F46">
+      <c r="F46" s="22">
         <f>LEFT(C46,1)</f>
         <v/>
       </c>
-      <c r="G46">
+      <c r="G46" s="22">
         <f>LEFT(D46,1)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>[R5.7] Church: particular denomination</t>
         </is>
       </c>
-      <c r="B47">
+      <c r="B47" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C47">
+      <c r="C47" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D47">
+      <c r="D47" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A47&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E47">
+      <c r="E47" s="22">
         <f>LEFT(B47,1)</f>
         <v/>
       </c>
-      <c r="F47">
+      <c r="F47" s="22">
         <f>LEFT(C47,1)</f>
         <v/>
       </c>
-      <c r="G47">
+      <c r="G47" s="22">
         <f>LEFT(D47,1)</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>[R5 Notes]</t>
         </is>
       </c>
-      <c r="B48">
+      <c r="B48" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C48">
+      <c r="C48" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D48">
+      <c r="D48" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A48&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="22" t="inlineStr">
         <is>
           <t>[R6.1] Separation: least that would work</t>
         </is>
       </c>
-      <c r="B49">
+      <c r="B49" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C49">
+      <c r="C49" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D49">
+      <c r="D49" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A49&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E49">
+      <c r="E49" s="22">
         <f>LEFT(B49,1)</f>
         <v/>
       </c>
-      <c r="F49">
+      <c r="F49" s="22">
         <f>LEFT(C49,1)</f>
         <v/>
       </c>
-      <c r="G49">
+      <c r="G49" s="22">
         <f>LEFT(D49,1)</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>[R6.2] Separation: most that still feels like one household</t>
         </is>
       </c>
-      <c r="B50">
+      <c r="B50" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C50">
+      <c r="C50" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D50">
+      <c r="D50" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A50&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E50">
+      <c r="E50" s="22">
         <f>LEFT(B50,1)</f>
         <v/>
       </c>
-      <c r="F50">
+      <c r="F50" s="22">
         <f>LEFT(C50,1)</f>
         <v/>
       </c>
-      <c r="G50">
+      <c r="G50" s="22">
         <f>LEFT(D50,1)</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>[R6.3] Separation: importance of having it already</t>
         </is>
       </c>
-      <c r="B51">
+      <c r="B51" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C51">
+      <c r="C51" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D51">
+      <c r="D51" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A51&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E51">
+      <c r="E51" s="22">
         <f>LEFT(B51,1)</f>
         <v/>
       </c>
-      <c r="F51">
+      <c r="F51" s="22">
         <f>LEFT(C51,1)</f>
         <v/>
       </c>
-      <c r="G51">
+      <c r="G51" s="22">
         <f>LEFT(D51,1)</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>[R6.4] Mobility: must-have in 10-15 years</t>
         </is>
       </c>
-      <c r="B52">
+      <c r="B52" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C52">
+      <c r="C52" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D52">
+      <c r="D52" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A52&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E52">
+      <c r="E52" s="22">
         <f>LEFT(B52,1)</f>
         <v/>
       </c>
-      <c r="F52">
+      <c r="F52" s="22">
         <f>LEFT(C52,1)</f>
         <v/>
       </c>
-      <c r="G52">
+      <c r="G52" s="22">
         <f>LEFT(D52,1)</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>[R6.5a] Outdoor space wanted</t>
         </is>
       </c>
-      <c r="B53">
+      <c r="B53" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C53">
+      <c r="C53" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D53">
+      <c r="D53" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A53&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E53">
+      <c r="E53" s="22">
         <f>LEFT(B53,1)</f>
         <v/>
       </c>
-      <c r="F53">
+      <c r="F53" s="22">
         <f>LEFT(C53,1)</f>
         <v/>
       </c>
-      <c r="G53">
+      <c r="G53" s="22">
         <f>LEFT(D53,1)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>[R6.5b] Garden upkeep capacity</t>
         </is>
       </c>
-      <c r="B54">
+      <c r="B54" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C54">
+      <c r="C54" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D54">
+      <c r="D54" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A54&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E54">
+      <c r="E54" s="22">
         <f>LEFT(B54,1)</f>
         <v/>
       </c>
-      <c r="F54">
+      <c r="F54" s="22">
         <f>LEFT(C54,1)</f>
         <v/>
       </c>
-      <c r="G54">
+      <c r="G54" s="22">
         <f>LEFT(D54,1)</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>[R6.6] Supermarket and GP from the front door</t>
         </is>
       </c>
-      <c r="B55">
+      <c r="B55" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C55">
+      <c r="C55" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D55">
+      <c r="D55" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A55&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E55">
+      <c r="E55" s="22">
         <f>LEFT(B55,1)</f>
         <v/>
       </c>
-      <c r="F55">
+      <c r="F55" s="22">
         <f>LEFT(C55,1)</f>
         <v/>
       </c>
-      <c r="G55">
+      <c r="G55" s="22">
         <f>LEFT(D55,1)</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>[R6.7] Privacy: one thing that matters most</t>
         </is>
       </c>
-      <c r="B56">
+      <c r="B56" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C56">
+      <c r="C56" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D56">
+      <c r="D56" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A56&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="E56">
+      <c r="E56" s="22">
         <f>LEFT(B56,1)</f>
         <v/>
       </c>
-      <c r="F56">
+      <c r="F56" s="22">
         <f>LEFT(C56,1)</f>
         <v/>
       </c>
-      <c r="G56">
+      <c r="G56" s="22">
         <f>LEFT(D56,1)</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>[R6 Notes]</t>
         </is>
       </c>
-      <c r="B57">
+      <c r="B57" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$2,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$2,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="C57">
+      <c r="C57" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$3,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$3,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
-      <c r="D57">
+      <c r="D57" s="22">
         <f>IFERROR(IF(INDEX(RawResponses!$A:$BE,$B$4,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))="","",INDEX(RawResponses!$A:$BE,$B$4,MATCH($A57&amp;"*",RawResponses!$A$1:$BE$1,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>Derived (B–D per person; E household)</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>GW firm limit (min)</t>
         </is>
       </c>
-      <c r="B59">
+      <c r="B59" s="22">
         <f>IFERROR(IF(E42="","",CHOOSE(FIND(E42,"ABCDE"),25,35,45,60,90)),"")</f>
         <v/>
       </c>
-      <c r="C59">
+      <c r="C59" s="22">
         <f>IFERROR(IF(F42="","",CHOOSE(FIND(F42,"ABCDE"),25,35,45,60,90)),"")</f>
         <v/>
       </c>
-      <c r="D59">
+      <c r="D59" s="22">
         <f>IFERROR(IF(G42="","",CHOOSE(FIND(G42,"ABCDE"),25,35,45,60,90)),"")</f>
         <v/>
       </c>
-      <c r="E59">
+      <c r="E59" s="22">
         <f>IF(COUNTIF(E42:G42,"?")&lt;3,"",MIN(B59:D59))</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>GW preferred (min)</t>
         </is>
       </c>
-      <c r="B60">
+      <c r="B60" s="22">
         <f>IFERROR(IF(E43="","",CHOOSE(FIND(E43,"ABCDE"),25,35,45,60,90)),"")</f>
         <v/>
       </c>
-      <c r="C60">
+      <c r="C60" s="22">
         <f>IFERROR(IF(F43="","",CHOOSE(FIND(F43,"ABCDE"),25,35,45,60,90)),"")</f>
         <v/>
       </c>
-      <c r="D60">
+      <c r="D60" s="22">
         <f>IFERROR(IF(G43="","",CHOOSE(FIND(G43,"ABCDE"),25,35,45,60,90)),"")</f>
         <v/>
       </c>
-      <c r="E60">
+      <c r="E60" s="22">
         <f>IF(COUNTIF(E43:G43,"?")&lt;3,"",MIN(B60:D60))</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="22" t="inlineStr">
         <is>
           <t>ED firm limit (min; blank = no limit)</t>
         </is>
       </c>
-      <c r="B61">
+      <c r="B61" s="22">
         <f>IFERROR(IF(E44="","",CHOOSE(FIND(E44,"ABCDE"),15,20,30,45,"")),"")</f>
         <v/>
       </c>
-      <c r="C61">
+      <c r="C61" s="22">
         <f>IFERROR(IF(F44="","",CHOOSE(FIND(F44,"ABCDE"),15,20,30,45,"")),"")</f>
         <v/>
       </c>
-      <c r="D61">
+      <c r="D61" s="22">
         <f>IFERROR(IF(G44="","",CHOOSE(FIND(G44,"ABCDE"),15,20,30,45,"")),"")</f>
         <v/>
       </c>
-      <c r="E61">
+      <c r="E61" s="22">
         <f>IF(COUNTIF(E44:G44,"?")&lt;3,"",IF(COUNT(B61:D61)=0,"No cap",MIN(B61:D61)))</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="22" t="inlineStr">
         <is>
           <t>Community place index (grocery 1, temple 2, church 3, none 0)</t>
         </is>
       </c>
-      <c r="B62">
+      <c r="B62" s="22">
         <f>IFERROR(IF(E45="","",CHOOSE(FIND(E45,"ABCDE"),1,2,3,0)),"")</f>
         <v/>
       </c>
-      <c r="C62">
+      <c r="C62" s="22">
         <f>IFERROR(IF(F45="","",CHOOSE(FIND(F45,"ABCDE"),1,2,3,0)),"")</f>
         <v/>
       </c>
-      <c r="D62">
+      <c r="D62" s="22">
         <f>IFERROR(IF(G45="","",CHOOSE(FIND(G45,"ABCDE"),1,2,3,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="22" t="inlineStr">
         <is>
           <t>Community drive limit (min)</t>
         </is>
       </c>
-      <c r="B63">
+      <c r="B63" s="22">
         <f>IFERROR(IF(E46="","",CHOOSE(FIND(E46,"ABCDE"),10,20,30,45,"")),"")</f>
         <v/>
       </c>
-      <c r="C63">
+      <c r="C63" s="22">
         <f>IFERROR(IF(F46="","",CHOOSE(FIND(F46,"ABCDE"),10,20,30,45,"")),"")</f>
         <v/>
       </c>
-      <c r="D63">
+      <c r="D63" s="22">
         <f>IFERROR(IF(G46="","",CHOOSE(FIND(G46,"ABCDE"),10,20,30,45,"")),"")</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="22" t="inlineStr">
         <is>
           <t>Separation floor (1–4)</t>
         </is>
       </c>
-      <c r="B64">
+      <c r="B64" s="22">
         <f>IFERROR(IF(E49="","",CHOOSE(FIND(E49,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="C64">
+      <c r="C64" s="22">
         <f>IFERROR(IF(F49="","",CHOOSE(FIND(F49,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="D64">
+      <c r="D64" s="22">
         <f>IFERROR(IF(G49="","",CHOOSE(FIND(G49,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="E64">
-        <f>IF(COUNTIF(E49:G49,"?")&lt;3,"",MAX(B64:D64))</f>
+      <c r="E64" s="22">
+        <f>IF(OR((3-COUNTIF(E13:G13,"B"))=0,COUNTIF(E49:G49,"?")&lt;(3-COUNTIF(E13:G13,"B"))),"",MAX(B64:D64))</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="22" t="inlineStr">
         <is>
           <t>Separation ceiling (1–4)</t>
         </is>
       </c>
-      <c r="B65">
+      <c r="B65" s="22">
         <f>IFERROR(IF(E50="","",CHOOSE(FIND(E50,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="C65">
+      <c r="C65" s="22">
         <f>IFERROR(IF(F50="","",CHOOSE(FIND(F50,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="D65">
+      <c r="D65" s="22">
         <f>IFERROR(IF(G50="","",CHOOSE(FIND(G50,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="E65">
-        <f>IF(COUNTIF(E50:G50,"?")&lt;3,"",MIN(B65:D65))</f>
-        <v/>
-      </c>
-      <c r="F65">
+      <c r="E65" s="22">
+        <f>IF(OR((3-COUNTIF(E13:G13,"B"))=0,COUNTIF(E50:G50,"?")&lt;(3-COUNTIF(E13:G13,"B"))),"",MIN(B65:D65))</f>
+        <v/>
+      </c>
+      <c r="F65" s="22">
         <f>IF(OR(E64="",E65=""),"",IF(E64&gt;E65,"CONFLICT: no layout suits everyone","OK"))</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="22" t="inlineStr">
         <is>
           <t>Separation importance (3 Essential, 2 Important, 1 Nice to have)</t>
         </is>
       </c>
-      <c r="B66">
+      <c r="B66" s="22">
         <f>IFERROR(IF(E51="","",CHOOSE(FIND(E51,"ABCDE"),3,2,1)),"")</f>
         <v/>
       </c>
-      <c r="C66">
+      <c r="C66" s="22">
         <f>IFERROR(IF(F51="","",CHOOSE(FIND(F51,"ABCDE"),3,2,1)),"")</f>
         <v/>
       </c>
-      <c r="D66">
+      <c r="D66" s="22">
         <f>IFERROR(IF(G51="","",CHOOSE(FIND(G51,"ABCDE"),3,2,1)),"")</f>
         <v/>
       </c>
-      <c r="E66">
-        <f>IF(COUNTIF(E51:G51,"?")&lt;3,"",MAX(B66:D66))</f>
+      <c r="E66" s="22">
+        <f>IF(OR((3-COUNTIF(E13:G13,"B"))=0,COUNTIF(E51:G51,"?")&lt;(3-COUNTIF(E13:G13,"B"))),"",MAX(B66:D66))</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="22" t="inlineStr">
         <is>
           <t>Mobility must-have (0–3)</t>
         </is>
       </c>
-      <c r="B67">
+      <c r="B67" s="22">
         <f>IFERROR(IF(E52="","",CHOOSE(FIND(E52,"ABCDE"),0,1,2,3)),"")</f>
         <v/>
       </c>
-      <c r="C67">
+      <c r="C67" s="22">
         <f>IFERROR(IF(F52="","",CHOOSE(FIND(F52,"ABCDE"),0,1,2,3)),"")</f>
         <v/>
       </c>
-      <c r="D67">
+      <c r="D67" s="22">
         <f>IFERROR(IF(G52="","",CHOOSE(FIND(G52,"ABCDE"),0,1,2,3)),"")</f>
         <v/>
       </c>
-      <c r="E67">
+      <c r="E67" s="22">
         <f>IF(COUNTIF(E52:G52,"?")&lt;3,"",MAX(B67:D67))</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="22" t="inlineStr">
         <is>
           <t>Garden preferred band (1–4)</t>
         </is>
       </c>
-      <c r="B68">
+      <c r="B68" s="22">
         <f>IFERROR(IF(E53="","",CHOOSE(FIND(E53,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="C68">
+      <c r="C68" s="22">
         <f>IFERROR(IF(F53="","",CHOOSE(FIND(F53,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="D68">
+      <c r="D68" s="22">
         <f>IFERROR(IF(G53="","",CHOOSE(FIND(G53,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="E68">
+      <c r="E68" s="22">
         <f>IF(COUNTIF(E53:G53,"?")&lt;3,"",MEDIAN(B68:D68))</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="22" t="inlineStr">
         <is>
           <t>Garden capacity band (1–4)</t>
         </is>
       </c>
-      <c r="B69">
+      <c r="B69" s="22">
         <f>IFERROR(IF(E54="","",CHOOSE(FIND(E54,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="C69">
+      <c r="C69" s="22">
         <f>IFERROR(IF(F54="","",CHOOSE(FIND(F54,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="D69">
+      <c r="D69" s="22">
         <f>IFERROR(IF(G54="","",CHOOSE(FIND(G54,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="E69">
+      <c r="E69" s="22">
         <f>IF(COUNTIF(E54:G54,"?")&lt;3,"",MEDIAN(B69:D69))</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="22" t="inlineStr">
         <is>
           <t>Front-door access (1 must walk … 4 drive up to 20 min)</t>
         </is>
       </c>
-      <c r="B70">
+      <c r="B70" s="22">
         <f>IFERROR(IF(E55="","",CHOOSE(FIND(E55,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="C70">
+      <c r="C70" s="22">
         <f>IFERROR(IF(F55="","",CHOOSE(FIND(F55,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="D70">
+      <c r="D70" s="22">
         <f>IFERROR(IF(G55="","",CHOOSE(FIND(G55,"ABCDE"),1,2,3,4)),"")</f>
         <v/>
       </c>
-      <c r="E70">
+      <c r="E70" s="22">
         <f>IF(COUNTIF(E55:G55,"?")&lt;3,"",MIN(B70:D70))</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Validation (R6.2 ≥ R6.1; R5.5/R5.6 and R5.5/R5.7 consistent)</t>
-        </is>
-      </c>
-      <c r="B71">
-        <f>IFERROR(IF(E45&amp;E46&amp;E47&amp;E49&amp;E50="","",IF(AND(LEN(E45&amp;E46&amp;E47&amp;E49&amp;E50)=5,E50&gt;=E49,IF(E45="D",E46="E",E46&lt;&gt;"E"),IF(E45="C",E47&lt;&gt;"C",E47="C")),"OK","Check")),"Check")</f>
-        <v/>
-      </c>
-      <c r="C71">
-        <f>IFERROR(IF(F45&amp;F46&amp;F47&amp;F49&amp;F50="","",IF(AND(LEN(F45&amp;F46&amp;F47&amp;F49&amp;F50)=5,F50&gt;=F49,IF(F45="D",F46="E",F46&lt;&gt;"E"),IF(F45="C",F47&lt;&gt;"C",F47="C")),"OK","Check")),"Check")</f>
-        <v/>
-      </c>
-      <c r="D71">
-        <f>IFERROR(IF(G45&amp;G46&amp;G47&amp;G49&amp;G50="","",IF(AND(LEN(G45&amp;G46&amp;G47&amp;G49&amp;G50)=5,G50&gt;=G49,IF(G45="D",G46="E",G46&lt;&gt;"E"),IF(G45="C",G47&lt;&gt;"C",G47="C")),"OK","Check")),"Check")</f>
+      <c r="A71" s="22" t="inlineStr">
+        <is>
+          <t>Validation (R6.2 ≥ R6.1, skipped if parents only; R5.5/R5.6 and R5.5/R5.7 consistent)</t>
+        </is>
+      </c>
+      <c r="B71" s="22">
+        <f>IFERROR(IF(E45&amp;E46&amp;E47&amp;E49&amp;E50="","",IF(AND(LEN(E45&amp;E46&amp;E47)=3,IF(E13="B",E49&amp;E50="",AND(LEN(E49&amp;E50)=2,E50&gt;=E49)),IF(E45="D",E46="E",E46&lt;&gt;"E"),IF(E45="C",E47&lt;&gt;"C",E47="C")),"OK","Check")),"Check")</f>
+        <v/>
+      </c>
+      <c r="C71" s="22">
+        <f>IFERROR(IF(F45&amp;F46&amp;F47&amp;F49&amp;F50="","",IF(AND(LEN(F45&amp;F46&amp;F47)=3,IF(F13="B",F49&amp;F50="",AND(LEN(F49&amp;F50)=2,F50&gt;=F49)),IF(F45="D",F46="E",F46&lt;&gt;"E"),IF(F45="C",F47&lt;&gt;"C",F47="C")),"OK","Check")),"Check")</f>
+        <v/>
+      </c>
+      <c r="D71" s="22">
+        <f>IFERROR(IF(G45&amp;G46&amp;G47&amp;G49&amp;G50="","",IF(AND(LEN(G45&amp;G46&amp;G47)=3,IF(G13="B",G49&amp;G50="",AND(LEN(G49&amp;G50)=2,G50&gt;=G49)),IF(G45="D",G46="E",G46&lt;&gt;"E"),IF(G45="C",G47&lt;&gt;"C",G47="C")),"OK","Check")),"Check")</f>
         <v/>
       </c>
     </row>
@@ -7836,27 +7836,27 @@
           <t>Community comparison band (display-only)</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AY1" s="22" t="inlineStr">
         <is>
           <t>Drive to nearest Indian grocery (min; 10:00 weekday, top of range)</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="AZ1" s="22" t="inlineStr">
         <is>
           <t>Drive to nearest Hindu temple (min; 10:00 weekday, top of range)</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BA1" s="22" t="inlineStr">
         <is>
           <t>Drive to nearest church (min; 10:00 weekday, top of range)</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BB1" s="22" t="inlineStr">
         <is>
           <t>Community drive basis and evidence (Checked / Estimate / Needs verification)</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BF1" s="22" t="inlineStr">
         <is>
           <t>Slope/stairs risk (display-only, Estimate; feeds nothing)</t>
         </is>
@@ -22252,52 +22252,52 @@
           <t>Source: realestate.com.au collection 'Parents.', read from browser 27 Oct 2026 (copied from the Google Sheet version of this tab). A–F, H–O, U are pasted values; G and P–T are formulas. Prices are agent guides (purchase price, before costs), compared with Filters!B2 purchase cap. Drive times and train are suburb-level from SuburbScorecard, not per address. Inspection times go stale after 31 Oct. Refresh = re-read the collection and overwrite pasted columns only.</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="22" t="inlineStr">
         <is>
           <t>Separation tier now (A–D / Unknown; R6.1 ladder, from floorplan)</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="22" t="inlineStr">
         <is>
           <t>Mobility level met now (0–3 / Unknown; R6.4 ladder)</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="22" t="inlineStr">
         <is>
           <t>Mobility gap (None / Minor works / Major / Unknown)</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="22" t="inlineStr">
         <is>
           <t>Garden band 1–4 (formula: K vs Settings B35:B37; photos override, note in AF)</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="22" t="inlineStr">
         <is>
           <t>Walk to supermarket (min; basis named)</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="22" t="inlineStr">
         <is>
           <t>Walk to GP (min; basis named)</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="22" t="inlineStr">
         <is>
           <t>Noise flag (Highway / Rail / Flight path / None)</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="22" t="inlineStr">
         <is>
           <t>Overlay (Bushfire / Flood / Heritage / None; task B3)</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="22" t="inlineStr">
         <is>
           <t>Evidence basis + date (Floorplan seen / Photos only / Not checked)</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="22" t="inlineStr">
         <is>
           <t>Home fit (formula: first matching rule, design doc section 5)</t>
         </is>
@@ -22389,11 +22389,11 @@
           <t>https://www.realestate.com.au/property-house-vic-torquay-152666740</t>
         </is>
       </c>
-      <c r="AA2">
+      <c r="AA2" s="22">
         <f>IF(OR(NOT(ISNUMBER(K2)),Settings!$B$35=""),"",IF(K2&lt;=Settings!$B$35,1,IF(K2&lt;=Settings!$B$36,2,IF(K2&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG2">
+      <c r="AG2" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T2="Under offer",LEFT(T2,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X2="",X2="Unknown",Y2="",Y2="Unknown",AND(AND(ISNUMBER(Y2),Y2&lt;Settings!$B$31),OR(Z2="",Z2="Unknown"))),"Needs data: floorplan",IF(FIND(X2,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X2,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y2),Y2&lt;Settings!$B$31),Z2="Major"),"Not suitable: mobility",IF(FIND(X2,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y2),Y2&lt;Settings!$B$31),Z2="Minor works"),"Watchlist: minor mobility works",IF(T2="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA2),AA2&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA2),ABS(AA2-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD2&lt;&gt;"",AD2&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE2&lt;&gt;"",AE2&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB2),AB2&gt;10),AND(ISNUMBER(AC2),AC2&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -22482,11 +22482,11 @@
           <t>https://www.realestate.com.au/property-house-vic-west+footscray-152623144</t>
         </is>
       </c>
-      <c r="AA3">
+      <c r="AA3" s="22">
         <f>IF(OR(NOT(ISNUMBER(K3)),Settings!$B$35=""),"",IF(K3&lt;=Settings!$B$35,1,IF(K3&lt;=Settings!$B$36,2,IF(K3&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG3">
+      <c r="AG3" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T3="Under offer",LEFT(T3,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X3="",X3="Unknown",Y3="",Y3="Unknown",AND(AND(ISNUMBER(Y3),Y3&lt;Settings!$B$31),OR(Z3="",Z3="Unknown"))),"Needs data: floorplan",IF(FIND(X3,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X3,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y3),Y3&lt;Settings!$B$31),Z3="Major"),"Not suitable: mobility",IF(FIND(X3,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y3),Y3&lt;Settings!$B$31),Z3="Minor works"),"Watchlist: minor mobility works",IF(T3="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA3),AA3&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA3),ABS(AA3-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD3&lt;&gt;"",AD3&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE3&lt;&gt;"",AE3&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB3),AB3&gt;10),AND(ISNUMBER(AC3),AC3&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -22582,11 +22582,11 @@
           <t>https://www.realestate.com.au/property-house-vic-warburton-150763740</t>
         </is>
       </c>
-      <c r="AA4">
+      <c r="AA4" s="22">
         <f>IF(OR(NOT(ISNUMBER(K4)),Settings!$B$35=""),"",IF(K4&lt;=Settings!$B$35,1,IF(K4&lt;=Settings!$B$36,2,IF(K4&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG4">
+      <c r="AG4" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T4="Under offer",LEFT(T4,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X4="",X4="Unknown",Y4="",Y4="Unknown",AND(AND(ISNUMBER(Y4),Y4&lt;Settings!$B$31),OR(Z4="",Z4="Unknown"))),"Needs data: floorplan",IF(FIND(X4,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X4,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y4),Y4&lt;Settings!$B$31),Z4="Major"),"Not suitable: mobility",IF(FIND(X4,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y4),Y4&lt;Settings!$B$31),Z4="Minor works"),"Watchlist: minor mobility works",IF(T4="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA4),AA4&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA4),ABS(AA4-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD4&lt;&gt;"",AD4&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE4&lt;&gt;"",AE4&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB4),AB4&gt;10),AND(ISNUMBER(AC4),AC4&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -22674,11 +22674,11 @@
           <t>https://www.realestate.com.au/property-house-vic-williamstown-152686328</t>
         </is>
       </c>
-      <c r="AA5">
+      <c r="AA5" s="22">
         <f>IF(OR(NOT(ISNUMBER(K5)),Settings!$B$35=""),"",IF(K5&lt;=Settings!$B$35,1,IF(K5&lt;=Settings!$B$36,2,IF(K5&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG5">
+      <c r="AG5" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T5="Under offer",LEFT(T5,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X5="",X5="Unknown",Y5="",Y5="Unknown",AND(AND(ISNUMBER(Y5),Y5&lt;Settings!$B$31),OR(Z5="",Z5="Unknown"))),"Needs data: floorplan",IF(FIND(X5,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X5,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y5),Y5&lt;Settings!$B$31),Z5="Major"),"Not suitable: mobility",IF(FIND(X5,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y5),Y5&lt;Settings!$B$31),Z5="Minor works"),"Watchlist: minor mobility works",IF(T5="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA5),AA5&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA5),ABS(AA5-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD5&lt;&gt;"",AD5&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE5&lt;&gt;"",AE5&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB5),AB5&gt;10),AND(ISNUMBER(AC5),AC5&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -22770,11 +22770,11 @@
           <t>https://www.realestate.com.au/property-house-vic-rosanna-152574468</t>
         </is>
       </c>
-      <c r="AA6">
+      <c r="AA6" s="22">
         <f>IF(OR(NOT(ISNUMBER(K6)),Settings!$B$35=""),"",IF(K6&lt;=Settings!$B$35,1,IF(K6&lt;=Settings!$B$36,2,IF(K6&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG6">
+      <c r="AG6" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T6="Under offer",LEFT(T6,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X6="",X6="Unknown",Y6="",Y6="Unknown",AND(AND(ISNUMBER(Y6),Y6&lt;Settings!$B$31),OR(Z6="",Z6="Unknown"))),"Needs data: floorplan",IF(FIND(X6,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X6,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y6),Y6&lt;Settings!$B$31),Z6="Major"),"Not suitable: mobility",IF(FIND(X6,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y6),Y6&lt;Settings!$B$31),Z6="Minor works"),"Watchlist: minor mobility works",IF(T6="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA6),AA6&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA6),ABS(AA6-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD6&lt;&gt;"",AD6&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE6&lt;&gt;"",AE6&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB6),AB6&gt;10),AND(ISNUMBER(AC6),AC6&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -22865,11 +22865,11 @@
           <t>https://www.realestate.com.au/property-house-vic-diamond+creek-152290624</t>
         </is>
       </c>
-      <c r="AA7">
+      <c r="AA7" s="22">
         <f>IF(OR(NOT(ISNUMBER(K7)),Settings!$B$35=""),"",IF(K7&lt;=Settings!$B$35,1,IF(K7&lt;=Settings!$B$36,2,IF(K7&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG7">
+      <c r="AG7" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T7="Under offer",LEFT(T7,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X7="",X7="Unknown",Y7="",Y7="Unknown",AND(AND(ISNUMBER(Y7),Y7&lt;Settings!$B$31),OR(Z7="",Z7="Unknown"))),"Needs data: floorplan",IF(FIND(X7,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X7,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y7),Y7&lt;Settings!$B$31),Z7="Major"),"Not suitable: mobility",IF(FIND(X7,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y7),Y7&lt;Settings!$B$31),Z7="Minor works"),"Watchlist: minor mobility works",IF(T7="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA7),AA7&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA7),ABS(AA7-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD7&lt;&gt;"",AD7&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE7&lt;&gt;"",AE7&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB7),AB7&gt;10),AND(ISNUMBER(AC7),AC7&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -22961,11 +22961,11 @@
           <t>https://www.realestate.com.au/property-house-vic-mordialloc-152622844</t>
         </is>
       </c>
-      <c r="AA8">
+      <c r="AA8" s="22">
         <f>IF(OR(NOT(ISNUMBER(K8)),Settings!$B$35=""),"",IF(K8&lt;=Settings!$B$35,1,IF(K8&lt;=Settings!$B$36,2,IF(K8&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG8">
+      <c r="AG8" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T8="Under offer",LEFT(T8,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X8="",X8="Unknown",Y8="",Y8="Unknown",AND(AND(ISNUMBER(Y8),Y8&lt;Settings!$B$31),OR(Z8="",Z8="Unknown"))),"Needs data: floorplan",IF(FIND(X8,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X8,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y8),Y8&lt;Settings!$B$31),Z8="Major"),"Not suitable: mobility",IF(FIND(X8,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y8),Y8&lt;Settings!$B$31),Z8="Minor works"),"Watchlist: minor mobility works",IF(T8="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA8),AA8&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA8),ABS(AA8-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD8&lt;&gt;"",AD8&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE8&lt;&gt;"",AE8&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB8),AB8&gt;10),AND(ISNUMBER(AC8),AC8&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23057,11 +23057,11 @@
           <t>https://www.realestate.com.au/property-house-vic-seaford-152011424</t>
         </is>
       </c>
-      <c r="AA9">
+      <c r="AA9" s="22">
         <f>IF(OR(NOT(ISNUMBER(K9)),Settings!$B$35=""),"",IF(K9&lt;=Settings!$B$35,1,IF(K9&lt;=Settings!$B$36,2,IF(K9&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG9">
+      <c r="AG9" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T9="Under offer",LEFT(T9,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X9="",X9="Unknown",Y9="",Y9="Unknown",AND(AND(ISNUMBER(Y9),Y9&lt;Settings!$B$31),OR(Z9="",Z9="Unknown"))),"Needs data: floorplan",IF(FIND(X9,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X9,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y9),Y9&lt;Settings!$B$31),Z9="Major"),"Not suitable: mobility",IF(FIND(X9,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y9),Y9&lt;Settings!$B$31),Z9="Minor works"),"Watchlist: minor mobility works",IF(T9="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA9),AA9&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA9),ABS(AA9-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD9&lt;&gt;"",AD9&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE9&lt;&gt;"",AE9&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB9),AB9&gt;10),AND(ISNUMBER(AC9),AC9&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23153,11 +23153,11 @@
           <t>https://www.realestate.com.au/property-house-vic-seaford-151815440</t>
         </is>
       </c>
-      <c r="AA10">
+      <c r="AA10" s="22">
         <f>IF(OR(NOT(ISNUMBER(K10)),Settings!$B$35=""),"",IF(K10&lt;=Settings!$B$35,1,IF(K10&lt;=Settings!$B$36,2,IF(K10&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG10">
+      <c r="AG10" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T10="Under offer",LEFT(T10,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X10="",X10="Unknown",Y10="",Y10="Unknown",AND(AND(ISNUMBER(Y10),Y10&lt;Settings!$B$31),OR(Z10="",Z10="Unknown"))),"Needs data: floorplan",IF(FIND(X10,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X10,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y10),Y10&lt;Settings!$B$31),Z10="Major"),"Not suitable: mobility",IF(FIND(X10,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y10),Y10&lt;Settings!$B$31),Z10="Minor works"),"Watchlist: minor mobility works",IF(T10="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA10),AA10&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA10),ABS(AA10-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD10&lt;&gt;"",AD10&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE10&lt;&gt;"",AE10&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB10),AB10&gt;10),AND(ISNUMBER(AC10),AC10&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23248,11 +23248,11 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-151176748</t>
         </is>
       </c>
-      <c r="AA11">
+      <c r="AA11" s="22">
         <f>IF(OR(NOT(ISNUMBER(K11)),Settings!$B$35=""),"",IF(K11&lt;=Settings!$B$35,1,IF(K11&lt;=Settings!$B$36,2,IF(K11&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG11">
+      <c r="AG11" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T11="Under offer",LEFT(T11,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X11="",X11="Unknown",Y11="",Y11="Unknown",AND(AND(ISNUMBER(Y11),Y11&lt;Settings!$B$31),OR(Z11="",Z11="Unknown"))),"Needs data: floorplan",IF(FIND(X11,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X11,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y11),Y11&lt;Settings!$B$31),Z11="Major"),"Not suitable: mobility",IF(FIND(X11,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y11),Y11&lt;Settings!$B$31),Z11="Minor works"),"Watchlist: minor mobility works",IF(T11="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA11),AA11&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA11),ABS(AA11-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD11&lt;&gt;"",AD11&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE11&lt;&gt;"",AE11&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB11),AB11&gt;10),AND(ISNUMBER(AC11),AC11&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23343,11 +23343,11 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-152450032</t>
         </is>
       </c>
-      <c r="AA12">
+      <c r="AA12" s="22">
         <f>IF(OR(NOT(ISNUMBER(K12)),Settings!$B$35=""),"",IF(K12&lt;=Settings!$B$35,1,IF(K12&lt;=Settings!$B$36,2,IF(K12&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG12">
+      <c r="AG12" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T12="Under offer",LEFT(T12,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X12="",X12="Unknown",Y12="",Y12="Unknown",AND(AND(ISNUMBER(Y12),Y12&lt;Settings!$B$31),OR(Z12="",Z12="Unknown"))),"Needs data: floorplan",IF(FIND(X12,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X12,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y12),Y12&lt;Settings!$B$31),Z12="Major"),"Not suitable: mobility",IF(FIND(X12,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y12),Y12&lt;Settings!$B$31),Z12="Minor works"),"Watchlist: minor mobility works",IF(T12="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA12),AA12&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA12),ABS(AA12-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD12&lt;&gt;"",AD12&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE12&lt;&gt;"",AE12&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB12),AB12&gt;10),AND(ISNUMBER(AC12),AC12&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23438,11 +23438,11 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-152376824</t>
         </is>
       </c>
-      <c r="AA13">
+      <c r="AA13" s="22">
         <f>IF(OR(NOT(ISNUMBER(K13)),Settings!$B$35=""),"",IF(K13&lt;=Settings!$B$35,1,IF(K13&lt;=Settings!$B$36,2,IF(K13&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG13">
+      <c r="AG13" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T13="Under offer",LEFT(T13,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X13="",X13="Unknown",Y13="",Y13="Unknown",AND(AND(ISNUMBER(Y13),Y13&lt;Settings!$B$31),OR(Z13="",Z13="Unknown"))),"Needs data: floorplan",IF(FIND(X13,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X13,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y13),Y13&lt;Settings!$B$31),Z13="Major"),"Not suitable: mobility",IF(FIND(X13,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y13),Y13&lt;Settings!$B$31),Z13="Minor works"),"Watchlist: minor mobility works",IF(T13="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA13),AA13&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA13),ABS(AA13-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD13&lt;&gt;"",AD13&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE13&lt;&gt;"",AE13&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB13),AB13&gt;10),AND(ISNUMBER(AC13),AC13&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23533,11 +23533,11 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+eliza-151903892</t>
         </is>
       </c>
-      <c r="AA14">
+      <c r="AA14" s="22">
         <f>IF(OR(NOT(ISNUMBER(K14)),Settings!$B$35=""),"",IF(K14&lt;=Settings!$B$35,1,IF(K14&lt;=Settings!$B$36,2,IF(K14&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG14">
+      <c r="AG14" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T14="Under offer",LEFT(T14,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X14="",X14="Unknown",Y14="",Y14="Unknown",AND(AND(ISNUMBER(Y14),Y14&lt;Settings!$B$31),OR(Z14="",Z14="Unknown"))),"Needs data: floorplan",IF(FIND(X14,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X14,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y14),Y14&lt;Settings!$B$31),Z14="Major"),"Not suitable: mobility",IF(FIND(X14,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y14),Y14&lt;Settings!$B$31),Z14="Minor works"),"Watchlist: minor mobility works",IF(T14="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA14),AA14&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA14),ABS(AA14-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD14&lt;&gt;"",AD14&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE14&lt;&gt;"",AE14&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB14),AB14&gt;10),AND(ISNUMBER(AC14),AC14&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23629,11 +23629,11 @@
           <t>https://www.realestate.com.au/property-house-vic-arthurs+seat-146680920</t>
         </is>
       </c>
-      <c r="AA15">
+      <c r="AA15" s="22">
         <f>IF(OR(NOT(ISNUMBER(K15)),Settings!$B$35=""),"",IF(K15&lt;=Settings!$B$35,1,IF(K15&lt;=Settings!$B$36,2,IF(K15&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG15">
+      <c r="AG15" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T15="Under offer",LEFT(T15,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X15="",X15="Unknown",Y15="",Y15="Unknown",AND(AND(ISNUMBER(Y15),Y15&lt;Settings!$B$31),OR(Z15="",Z15="Unknown"))),"Needs data: floorplan",IF(FIND(X15,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X15,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y15),Y15&lt;Settings!$B$31),Z15="Major"),"Not suitable: mobility",IF(FIND(X15,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y15),Y15&lt;Settings!$B$31),Z15="Minor works"),"Watchlist: minor mobility works",IF(T15="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA15),AA15&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA15),ABS(AA15-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD15&lt;&gt;"",AD15&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE15&lt;&gt;"",AE15&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB15),AB15&gt;10),AND(ISNUMBER(AC15),AC15&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23725,11 +23725,11 @@
           <t>https://www.realestate.com.au/property-house-vic-dromana-152005848</t>
         </is>
       </c>
-      <c r="AA16">
+      <c r="AA16" s="22">
         <f>IF(OR(NOT(ISNUMBER(K16)),Settings!$B$35=""),"",IF(K16&lt;=Settings!$B$35,1,IF(K16&lt;=Settings!$B$36,2,IF(K16&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG16">
+      <c r="AG16" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T16="Under offer",LEFT(T16,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X16="",X16="Unknown",Y16="",Y16="Unknown",AND(AND(ISNUMBER(Y16),Y16&lt;Settings!$B$31),OR(Z16="",Z16="Unknown"))),"Needs data: floorplan",IF(FIND(X16,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X16,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y16),Y16&lt;Settings!$B$31),Z16="Major"),"Not suitable: mobility",IF(FIND(X16,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y16),Y16&lt;Settings!$B$31),Z16="Minor works"),"Watchlist: minor mobility works",IF(T16="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA16),AA16&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA16),ABS(AA16-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD16&lt;&gt;"",AD16&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE16&lt;&gt;"",AE16&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB16),AB16&gt;10),AND(ISNUMBER(AC16),AC16&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23821,11 +23821,11 @@
           <t>https://www.realestate.com.au/property-house-vic-curlewis-152352192</t>
         </is>
       </c>
-      <c r="AA17">
+      <c r="AA17" s="22">
         <f>IF(OR(NOT(ISNUMBER(K17)),Settings!$B$35=""),"",IF(K17&lt;=Settings!$B$35,1,IF(K17&lt;=Settings!$B$36,2,IF(K17&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG17">
+      <c r="AG17" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T17="Under offer",LEFT(T17,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X17="",X17="Unknown",Y17="",Y17="Unknown",AND(AND(ISNUMBER(Y17),Y17&lt;Settings!$B$31),OR(Z17="",Z17="Unknown"))),"Needs data: floorplan",IF(FIND(X17,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X17,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y17),Y17&lt;Settings!$B$31),Z17="Major"),"Not suitable: mobility",IF(FIND(X17,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y17),Y17&lt;Settings!$B$31),Z17="Minor works"),"Watchlist: minor mobility works",IF(T17="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA17),AA17&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA17),ABS(AA17-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD17&lt;&gt;"",AD17&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE17&lt;&gt;"",AE17&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB17),AB17&gt;10),AND(ISNUMBER(AC17),AC17&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -23917,11 +23917,11 @@
           <t>https://www.realestate.com.au/property-house-vic-mccrae-151835348</t>
         </is>
       </c>
-      <c r="AA18">
+      <c r="AA18" s="22">
         <f>IF(OR(NOT(ISNUMBER(K18)),Settings!$B$35=""),"",IF(K18&lt;=Settings!$B$35,1,IF(K18&lt;=Settings!$B$36,2,IF(K18&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG18">
+      <c r="AG18" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T18="Under offer",LEFT(T18,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X18="",X18="Unknown",Y18="",Y18="Unknown",AND(AND(ISNUMBER(Y18),Y18&lt;Settings!$B$31),OR(Z18="",Z18="Unknown"))),"Needs data: floorplan",IF(FIND(X18,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X18,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y18),Y18&lt;Settings!$B$31),Z18="Major"),"Not suitable: mobility",IF(FIND(X18,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y18),Y18&lt;Settings!$B$31),Z18="Minor works"),"Watchlist: minor mobility works",IF(T18="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA18),AA18&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA18),ABS(AA18-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD18&lt;&gt;"",AD18&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE18&lt;&gt;"",AE18&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB18),AB18&gt;10),AND(ISNUMBER(AC18),AC18&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24013,11 +24013,11 @@
           <t>https://www.realestate.com.au/property-house-vic-chelsea-152626264</t>
         </is>
       </c>
-      <c r="AA19">
+      <c r="AA19" s="22">
         <f>IF(OR(NOT(ISNUMBER(K19)),Settings!$B$35=""),"",IF(K19&lt;=Settings!$B$35,1,IF(K19&lt;=Settings!$B$36,2,IF(K19&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG19">
+      <c r="AG19" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T19="Under offer",LEFT(T19,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X19="",X19="Unknown",Y19="",Y19="Unknown",AND(AND(ISNUMBER(Y19),Y19&lt;Settings!$B$31),OR(Z19="",Z19="Unknown"))),"Needs data: floorplan",IF(FIND(X19,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X19,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y19),Y19&lt;Settings!$B$31),Z19="Major"),"Not suitable: mobility",IF(FIND(X19,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y19),Y19&lt;Settings!$B$31),Z19="Minor works"),"Watchlist: minor mobility works",IF(T19="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA19),AA19&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA19),ABS(AA19-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD19&lt;&gt;"",AD19&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE19&lt;&gt;"",AE19&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB19),AB19&gt;10),AND(ISNUMBER(AC19),AC19&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24108,11 +24108,11 @@
           <t>https://www.realestate.com.au/property-house-vic-torquay-152670688</t>
         </is>
       </c>
-      <c r="AA20">
+      <c r="AA20" s="22">
         <f>IF(OR(NOT(ISNUMBER(K20)),Settings!$B$35=""),"",IF(K20&lt;=Settings!$B$35,1,IF(K20&lt;=Settings!$B$36,2,IF(K20&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG20">
+      <c r="AG20" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T20="Under offer",LEFT(T20,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X20="",X20="Unknown",Y20="",Y20="Unknown",AND(AND(ISNUMBER(Y20),Y20&lt;Settings!$B$31),OR(Z20="",Z20="Unknown"))),"Needs data: floorplan",IF(FIND(X20,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X20,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y20),Y20&lt;Settings!$B$31),Z20="Major"),"Not suitable: mobility",IF(FIND(X20,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y20),Y20&lt;Settings!$B$31),Z20="Minor works"),"Watchlist: minor mobility works",IF(T20="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA20),AA20&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA20),ABS(AA20-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD20&lt;&gt;"",AD20&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE20&lt;&gt;"",AE20&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB20),AB20&gt;10),AND(ISNUMBER(AC20),AC20&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24204,11 +24204,11 @@
           <t>https://www.realestate.com.au/property-house-vic-newport-152302080</t>
         </is>
       </c>
-      <c r="AA21">
+      <c r="AA21" s="22">
         <f>IF(OR(NOT(ISNUMBER(K21)),Settings!$B$35=""),"",IF(K21&lt;=Settings!$B$35,1,IF(K21&lt;=Settings!$B$36,2,IF(K21&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG21">
+      <c r="AG21" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T21="Under offer",LEFT(T21,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X21="",X21="Unknown",Y21="",Y21="Unknown",AND(AND(ISNUMBER(Y21),Y21&lt;Settings!$B$31),OR(Z21="",Z21="Unknown"))),"Needs data: floorplan",IF(FIND(X21,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X21,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y21),Y21&lt;Settings!$B$31),Z21="Major"),"Not suitable: mobility",IF(FIND(X21,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y21),Y21&lt;Settings!$B$31),Z21="Minor works"),"Watchlist: minor mobility works",IF(T21="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA21),AA21&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA21),ABS(AA21-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD21&lt;&gt;"",AD21&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE21&lt;&gt;"",AE21&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB21),AB21&gt;10),AND(ISNUMBER(AC21),AC21&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24304,11 +24304,11 @@
           <t>https://www.realestate.com.au/property-house-vic-frankston+south-152212372</t>
         </is>
       </c>
-      <c r="AA22">
+      <c r="AA22" s="22">
         <f>IF(OR(NOT(ISNUMBER(K22)),Settings!$B$35=""),"",IF(K22&lt;=Settings!$B$35,1,IF(K22&lt;=Settings!$B$36,2,IF(K22&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG22">
+      <c r="AG22" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T22="Under offer",LEFT(T22,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X22="",X22="Unknown",Y22="",Y22="Unknown",AND(AND(ISNUMBER(Y22),Y22&lt;Settings!$B$31),OR(Z22="",Z22="Unknown"))),"Needs data: floorplan",IF(FIND(X22,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X22,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y22),Y22&lt;Settings!$B$31),Z22="Major"),"Not suitable: mobility",IF(FIND(X22,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y22),Y22&lt;Settings!$B$31),Z22="Minor works"),"Watchlist: minor mobility works",IF(T22="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA22),AA22&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA22),ABS(AA22-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD22&lt;&gt;"",AD22&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE22&lt;&gt;"",AE22&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB22),AB22&gt;10),AND(ISNUMBER(AC22),AC22&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24399,11 +24399,11 @@
           <t>https://www.realestate.com.au/property-house-vic-tecoma-152652276</t>
         </is>
       </c>
-      <c r="AA23">
+      <c r="AA23" s="22">
         <f>IF(OR(NOT(ISNUMBER(K23)),Settings!$B$35=""),"",IF(K23&lt;=Settings!$B$35,1,IF(K23&lt;=Settings!$B$36,2,IF(K23&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG23">
+      <c r="AG23" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T23="Under offer",LEFT(T23,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X23="",X23="Unknown",Y23="",Y23="Unknown",AND(AND(ISNUMBER(Y23),Y23&lt;Settings!$B$31),OR(Z23="",Z23="Unknown"))),"Needs data: floorplan",IF(FIND(X23,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X23,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y23),Y23&lt;Settings!$B$31),Z23="Major"),"Not suitable: mobility",IF(FIND(X23,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y23),Y23&lt;Settings!$B$31),Z23="Minor works"),"Watchlist: minor mobility works",IF(T23="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA23),AA23&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA23),ABS(AA23-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD23&lt;&gt;"",AD23&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE23&lt;&gt;"",AE23&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB23),AB23&gt;10),AND(ISNUMBER(AC23),AC23&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24499,11 +24499,11 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152722196</t>
         </is>
       </c>
-      <c r="AA24">
+      <c r="AA24" s="22">
         <f>IF(OR(NOT(ISNUMBER(K24)),Settings!$B$35=""),"",IF(K24&lt;=Settings!$B$35,1,IF(K24&lt;=Settings!$B$36,2,IF(K24&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG24">
+      <c r="AG24" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T24="Under offer",LEFT(T24,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X24="",X24="Unknown",Y24="",Y24="Unknown",AND(AND(ISNUMBER(Y24),Y24&lt;Settings!$B$31),OR(Z24="",Z24="Unknown"))),"Needs data: floorplan",IF(FIND(X24,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X24,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y24),Y24&lt;Settings!$B$31),Z24="Major"),"Not suitable: mobility",IF(FIND(X24,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y24),Y24&lt;Settings!$B$31),Z24="Minor works"),"Watchlist: minor mobility works",IF(T24="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA24),AA24&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA24),ABS(AA24-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD24&lt;&gt;"",AD24&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE24&lt;&gt;"",AE24&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB24),AB24&gt;10),AND(ISNUMBER(AC24),AC24&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24596,11 +24596,11 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152535704</t>
         </is>
       </c>
-      <c r="AA25">
+      <c r="AA25" s="22">
         <f>IF(OR(NOT(ISNUMBER(K25)),Settings!$B$35=""),"",IF(K25&lt;=Settings!$B$35,1,IF(K25&lt;=Settings!$B$36,2,IF(K25&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG25">
+      <c r="AG25" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T25="Under offer",LEFT(T25,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X25="",X25="Unknown",Y25="",Y25="Unknown",AND(AND(ISNUMBER(Y25),Y25&lt;Settings!$B$31),OR(Z25="",Z25="Unknown"))),"Needs data: floorplan",IF(FIND(X25,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X25,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y25),Y25&lt;Settings!$B$31),Z25="Major"),"Not suitable: mobility",IF(FIND(X25,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y25),Y25&lt;Settings!$B$31),Z25="Minor works"),"Watchlist: minor mobility works",IF(T25="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA25),AA25&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA25),ABS(AA25-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD25&lt;&gt;"",AD25&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE25&lt;&gt;"",AE25&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB25),AB25&gt;10),AND(ISNUMBER(AC25),AC25&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24691,11 +24691,11 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152654296</t>
         </is>
       </c>
-      <c r="AA26">
+      <c r="AA26" s="22">
         <f>IF(OR(NOT(ISNUMBER(K26)),Settings!$B$35=""),"",IF(K26&lt;=Settings!$B$35,1,IF(K26&lt;=Settings!$B$36,2,IF(K26&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG26">
+      <c r="AG26" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T26="Under offer",LEFT(T26,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X26="",X26="Unknown",Y26="",Y26="Unknown",AND(AND(ISNUMBER(Y26),Y26&lt;Settings!$B$31),OR(Z26="",Z26="Unknown"))),"Needs data: floorplan",IF(FIND(X26,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X26,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y26),Y26&lt;Settings!$B$31),Z26="Major"),"Not suitable: mobility",IF(FIND(X26,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y26),Y26&lt;Settings!$B$31),Z26="Minor works"),"Watchlist: minor mobility works",IF(T26="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA26),AA26&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA26),ABS(AA26-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD26&lt;&gt;"",AD26&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE26&lt;&gt;"",AE26&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB26),AB26&gt;10),AND(ISNUMBER(AC26),AC26&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24786,11 +24786,11 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152729140</t>
         </is>
       </c>
-      <c r="AA27">
+      <c r="AA27" s="22">
         <f>IF(OR(NOT(ISNUMBER(K27)),Settings!$B$35=""),"",IF(K27&lt;=Settings!$B$35,1,IF(K27&lt;=Settings!$B$36,2,IF(K27&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG27">
+      <c r="AG27" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T27="Under offer",LEFT(T27,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X27="",X27="Unknown",Y27="",Y27="Unknown",AND(AND(ISNUMBER(Y27),Y27&lt;Settings!$B$31),OR(Z27="",Z27="Unknown"))),"Needs data: floorplan",IF(FIND(X27,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X27,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y27),Y27&lt;Settings!$B$31),Z27="Major"),"Not suitable: mobility",IF(FIND(X27,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y27),Y27&lt;Settings!$B$31),Z27="Minor works"),"Watchlist: minor mobility works",IF(T27="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA27),AA27&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA27),ABS(AA27-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD27&lt;&gt;"",AD27&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE27&lt;&gt;"",AE27&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB27),AB27&gt;10),AND(ISNUMBER(AC27),AC27&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24882,11 +24882,11 @@
           <t>https://www.realestate.com.au/property-house-vic-mount+martha-152575492</t>
         </is>
       </c>
-      <c r="AA28">
+      <c r="AA28" s="22">
         <f>IF(OR(NOT(ISNUMBER(K28)),Settings!$B$35=""),"",IF(K28&lt;=Settings!$B$35,1,IF(K28&lt;=Settings!$B$36,2,IF(K28&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG28">
+      <c r="AG28" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T28="Under offer",LEFT(T28,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X28="",X28="Unknown",Y28="",Y28="Unknown",AND(AND(ISNUMBER(Y28),Y28&lt;Settings!$B$31),OR(Z28="",Z28="Unknown"))),"Needs data: floorplan",IF(FIND(X28,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X28,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y28),Y28&lt;Settings!$B$31),Z28="Major"),"Not suitable: mobility",IF(FIND(X28,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y28),Y28&lt;Settings!$B$31),Z28="Minor works"),"Watchlist: minor mobility works",IF(T28="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA28),AA28&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA28),ABS(AA28-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD28&lt;&gt;"",AD28&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE28&lt;&gt;"",AE28&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB28),AB28&gt;10),AND(ISNUMBER(AC28),AC28&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -24977,11 +24977,11 @@
           <t>https://www.realestate.com.au/property-house-vic-tecoma-152712080</t>
         </is>
       </c>
-      <c r="AA29">
+      <c r="AA29" s="22">
         <f>IF(OR(NOT(ISNUMBER(K29)),Settings!$B$35=""),"",IF(K29&lt;=Settings!$B$35,1,IF(K29&lt;=Settings!$B$36,2,IF(K29&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG29">
+      <c r="AG29" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T29="Under offer",LEFT(T29,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X29="",X29="Unknown",Y29="",Y29="Unknown",AND(AND(ISNUMBER(Y29),Y29&lt;Settings!$B$31),OR(Z29="",Z29="Unknown"))),"Needs data: floorplan",IF(FIND(X29,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X29,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y29),Y29&lt;Settings!$B$31),Z29="Major"),"Not suitable: mobility",IF(FIND(X29,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y29),Y29&lt;Settings!$B$31),Z29="Minor works"),"Watchlist: minor mobility works",IF(T29="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA29),AA29&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA29),ABS(AA29-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD29&lt;&gt;"",AD29&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE29&lt;&gt;"",AE29&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB29),AB29&gt;10),AND(ISNUMBER(AC29),AC29&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -25072,11 +25072,11 @@
           <t>https://www.realestate.com.au/property-house-vic-belgrave-152583472</t>
         </is>
       </c>
-      <c r="AA30">
+      <c r="AA30" s="22">
         <f>IF(OR(NOT(ISNUMBER(K30)),Settings!$B$35=""),"",IF(K30&lt;=Settings!$B$35,1,IF(K30&lt;=Settings!$B$36,2,IF(K30&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG30">
+      <c r="AG30" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T30="Under offer",LEFT(T30,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X30="",X30="Unknown",Y30="",Y30="Unknown",AND(AND(ISNUMBER(Y30),Y30&lt;Settings!$B$31),OR(Z30="",Z30="Unknown"))),"Needs data: floorplan",IF(FIND(X30,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X30,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y30),Y30&lt;Settings!$B$31),Z30="Major"),"Not suitable: mobility",IF(FIND(X30,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y30),Y30&lt;Settings!$B$31),Z30="Minor works"),"Watchlist: minor mobility works",IF(T30="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA30),AA30&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA30),ABS(AA30-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD30&lt;&gt;"",AD30&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE30&lt;&gt;"",AE30&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB30),AB30&gt;10),AND(ISNUMBER(AC30),AC30&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -25172,11 +25172,11 @@
           <t>https://www.realestate.com.au/property-house-vic-frankston-151132640</t>
         </is>
       </c>
-      <c r="AA31">
+      <c r="AA31" s="22">
         <f>IF(OR(NOT(ISNUMBER(K31)),Settings!$B$35=""),"",IF(K31&lt;=Settings!$B$35,1,IF(K31&lt;=Settings!$B$36,2,IF(K31&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG31">
+      <c r="AG31" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T31="Under offer",LEFT(T31,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X31="",X31="Unknown",Y31="",Y31="Unknown",AND(AND(ISNUMBER(Y31),Y31&lt;Settings!$B$31),OR(Z31="",Z31="Unknown"))),"Needs data: floorplan",IF(FIND(X31,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X31,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y31),Y31&lt;Settings!$B$31),Z31="Major"),"Not suitable: mobility",IF(FIND(X31,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y31),Y31&lt;Settings!$B$31),Z31="Minor works"),"Watchlist: minor mobility works",IF(T31="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA31),AA31&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA31),ABS(AA31-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD31&lt;&gt;"",AD31&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE31&lt;&gt;"",AE31&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB31),AB31&gt;10),AND(ISNUMBER(AC31),AC31&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -25267,11 +25267,11 @@
           <t>https://www.realestate.com.au/property-house-vic-frankston+south-152593596</t>
         </is>
       </c>
-      <c r="AA32">
+      <c r="AA32" s="22">
         <f>IF(OR(NOT(ISNUMBER(K32)),Settings!$B$35=""),"",IF(K32&lt;=Settings!$B$35,1,IF(K32&lt;=Settings!$B$36,2,IF(K32&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG32">
+      <c r="AG32" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T32="Under offer",LEFT(T32,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X32="",X32="Unknown",Y32="",Y32="Unknown",AND(AND(ISNUMBER(Y32),Y32&lt;Settings!$B$31),OR(Z32="",Z32="Unknown"))),"Needs data: floorplan",IF(FIND(X32,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X32,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y32),Y32&lt;Settings!$B$31),Z32="Major"),"Not suitable: mobility",IF(FIND(X32,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y32),Y32&lt;Settings!$B$31),Z32="Minor works"),"Watchlist: minor mobility works",IF(T32="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA32),AA32&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA32),ABS(AA32-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD32&lt;&gt;"",AD32&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE32&lt;&gt;"",AE32&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB32),AB32&gt;10),AND(ISNUMBER(AC32),AC32&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>
@@ -25362,11 +25362,11 @@
           <t>https://www.realestate.com.au/property-house-vic-frankston+south-152448552</t>
         </is>
       </c>
-      <c r="AA33">
+      <c r="AA33" s="22">
         <f>IF(OR(NOT(ISNUMBER(K33)),Settings!$B$35=""),"",IF(K33&lt;=Settings!$B$35,1,IF(K33&lt;=Settings!$B$36,2,IF(K33&lt;=Settings!$B$37,3,4))))</f>
         <v/>
       </c>
-      <c r="AG33">
+      <c r="AG33" s="22">
         <f>IF(Settings!$B$28="","Pending rules",IFERROR(IF(OR(T33="Under offer",LEFT(T33,5)="Fails"),"Not suitable: suburb/budget check",IF(OR(X33="",X33="Unknown",Y33="",Y33="Unknown",AND(AND(ISNUMBER(Y33),Y33&lt;Settings!$B$31),OR(Z33="",Z33="Unknown"))),"Needs data: floorplan",IF(FIND(X33,"ABCD")&gt;Settings!$B$29,"Not suitable: more separation than wanted",IF(AND(FIND(X33,"ABCD")&lt;Settings!$B$28,Settings!$B$30=3),"Not suitable: not enough separation",IF(AND(AND(ISNUMBER(Y33),Y33&lt;Settings!$B$31),Z33="Major"),"Not suitable: mobility",IF(FIND(X33,"ABCD")&lt;Settings!$B$28,"Watchlist: less separation than wanted",IF(AND(AND(ISNUMBER(Y33),Y33&lt;Settings!$B$31),Z33="Minor works"),"Watchlist: minor mobility works",IF(T33="Pass if bought near low end","Watchlist: pass if bought near low end",IF(AND(ISNUMBER(AA33),AA33&gt;Settings!$B$33),"Watchlist: garden upkeep",IF(AND(ISNUMBER(AA33),ABS(AA33-Settings!$B$32)&gt;=2),"Watchlist: outdoor space",IF(AND(AD33&lt;&gt;"",AD33&lt;&gt;"None"),"Watchlist: noise",IF(AND(AE33&lt;&gt;"",AE33&lt;&gt;"None"),"Watchlist: overlay",IF(AND(Settings!$B$34=1,OR(AND(ISNUMBER(AB33),AB33&gt;10),AND(ISNUMBER(AC33),AC33&gt;10))),"Watchlist: walk to shops/GP","Strong fit"))))))))))))),"Needs data: check X–AE values"))</f>
         <v/>
       </c>

</xml_diff>